<commit_message>
Sprint 17 & 18 Update code 10/03/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{267F8896-1D29-455D-AD65-2DDA36EB07BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84742FD-445A-4D32-AE6D-F8063DF0CC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Happy_Path_Patient_Web_and_MR" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2496" uniqueCount="1286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2513" uniqueCount="1299">
   <si>
     <t>KEY</t>
   </si>
@@ -3914,12 +3914,51 @@
   <si>
     <t>Automation1_HC1;Invite for Video Consultation;Video Consultations Msg Testing_RANDOM</t>
   </si>
+  <si>
+    <t>13 Feb 2025;13 Feb 2025;Lab Test;;Automation1_Loc1</t>
+  </si>
+  <si>
+    <t>Automation1_Loc1;GP1 A1 L1</t>
+  </si>
+  <si>
+    <t>Lab Results Test</t>
+  </si>
+  <si>
+    <t>SMS_LOCATION</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Secure Message - SMS</t>
+  </si>
+  <si>
+    <t>VM07 HC Evo Prod;Secure Message - SMS</t>
+  </si>
+  <si>
+    <t>REASON_DATA</t>
+  </si>
+  <si>
+    <t>Automation</t>
+  </si>
+  <si>
+    <t>UPADTE_REASON_DATA</t>
+  </si>
+  <si>
+    <t>AutomationUpdate</t>
+  </si>
+  <si>
+    <t>Automation1_Loc1;Automation Pre Screening Questionnaire</t>
+  </si>
+  <si>
+    <t>VM07 Loc1 Evo Prod;Automation Pre Screening Questionnaire</t>
+  </si>
+  <si>
+    <t>PRE_SCREENING_QUESTIONNAIRE_DATA</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4073,6 +4112,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9.8000000000000007"/>
+      <color rgb="FF5C92FF"/>
+      <name val="JetBrains Mono"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="13">
@@ -4362,7 +4407,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4603,6 +4648,9 @@
     <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="2" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -8764,7 +8812,7 @@
         <v>201</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>1251</v>
+        <v>1286</v>
       </c>
       <c r="C129" s="78" t="s">
         <v>1190</v>
@@ -8797,7 +8845,7 @@
         <v>203</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>1151</v>
+        <v>1287</v>
       </c>
       <c r="C130" s="87" t="s">
         <v>1100</v>
@@ -8830,7 +8878,7 @@
         <v>205</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>206</v>
+        <v>1288</v>
       </c>
       <c r="C131" s="78" t="s">
         <v>207</v>
@@ -29403,33 +29451,71 @@
       <c r="C166" s="64" t="s">
         <v>1272</v>
       </c>
+      <c r="D166" s="9" t="s">
+        <v>1212</v>
+      </c>
     </row>
     <row r="167" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A167" s="9"/>
-      <c r="B167" s="9"/>
-      <c r="C167" s="9"/>
+      <c r="A167" s="9" t="s">
+        <v>1289</v>
+      </c>
+      <c r="B167" s="9" t="s">
+        <v>1290</v>
+      </c>
+      <c r="C167" s="64" t="s">
+        <v>1291</v>
+      </c>
+      <c r="D167" s="9" t="s">
+        <v>1290</v>
+      </c>
     </row>
     <row r="168" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A168" s="9"/>
-      <c r="B168" s="9"/>
-      <c r="C168" s="9"/>
-    </row>
-    <row r="169" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A169" s="9"/>
-      <c r="B169" s="9"/>
-      <c r="C169" s="9"/>
-    </row>
-    <row r="170" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A170" s="9"/>
-      <c r="B170" s="9"/>
-      <c r="C170" s="9"/>
-    </row>
-    <row r="171" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A171" s="9"/>
+      <c r="A168" s="9" t="s">
+        <v>1292</v>
+      </c>
+      <c r="B168" s="9" t="s">
+        <v>1293</v>
+      </c>
+      <c r="C168" s="9" t="s">
+        <v>1293</v>
+      </c>
+      <c r="D168" s="9" t="s">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="169" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A169" s="94" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B169" s="9" t="s">
+        <v>1295</v>
+      </c>
+      <c r="C169" s="9" t="s">
+        <v>1295</v>
+      </c>
+      <c r="D169" s="9" t="s">
+        <v>1295</v>
+      </c>
+    </row>
+    <row r="170" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A170" s="9" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B170" s="9" t="s">
+        <v>1296</v>
+      </c>
+      <c r="C170" s="9" t="s">
+        <v>1297</v>
+      </c>
+      <c r="D170" s="9" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="171" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="B171" s="9"/>
       <c r="C171" s="9"/>
     </row>
-    <row r="172" spans="1:4" ht="15.75" customHeight="1">
+    <row r="172" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A172" s="9"/>
       <c r="B172" s="9"/>
       <c r="C172" s="9"/>

</xml_diff>

<commit_message>
BAU Sprint v5.6.1 updated code
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Automation_Framework\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{562B582F-ECF7-4B17-A2A1-02158F8B54AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95304062-A25B-449B-A016-C57D1FAD0ABF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="1560" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2561" uniqueCount="1266">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2561" uniqueCount="1265">
   <si>
     <t>KEY</t>
   </si>
@@ -3532,9 +3532,6 @@
   </si>
   <si>
     <t>Automation1_HC1;Invite for Video Consultation;Video Consultations Msg Testing_RANDOM</t>
-  </si>
-  <si>
-    <t>13 Feb 2025;13 Feb 2025;Lab Test;;Automation1_Loc1</t>
   </si>
   <si>
     <t>Automation1_Loc1;GP1 A1 L1</t>
@@ -4824,7 +4821,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="C2" s="74" t="s">
         <v>1048</v>
@@ -8719,7 +8716,7 @@
         <v>188</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>1159</v>
+        <v>1261</v>
       </c>
       <c r="C129" s="76" t="s">
         <v>1065</v>
@@ -8752,7 +8749,7 @@
         <v>189</v>
       </c>
       <c r="B130" s="10" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="C130" s="85" t="s">
         <v>976</v>
@@ -8785,7 +8782,7 @@
         <v>190</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="C131" s="76" t="s">
         <v>192</v>
@@ -8843,7 +8840,7 @@
         <v>193</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="C133" s="76" t="s">
         <v>1066</v>
@@ -16164,7 +16161,7 @@
         <v>218</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="C12" s="76" t="s">
         <v>1132</v>
@@ -16175,10 +16172,10 @@
         <v>557</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -16189,7 +16186,7 @@
         <v>559</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="30">
@@ -16197,10 +16194,10 @@
         <v>375</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -16233,7 +16230,7 @@
         <v>1079</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -16587,7 +16584,7 @@
         <v>571</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>573</v>
@@ -16599,7 +16596,7 @@
         <v>574</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="C69" s="9" t="s">
         <v>576</v>
@@ -16610,7 +16607,7 @@
         <v>577</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="C70" s="9" t="s">
         <v>578</v>
@@ -16621,7 +16618,7 @@
         <v>579</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="C71" s="9" t="s">
         <v>581</v>
@@ -16668,7 +16665,7 @@
         <v>589</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="C78" s="9" t="s">
         <v>591</v>
@@ -16701,7 +16698,7 @@
         <v>382</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="15.75" customHeight="1"/>
@@ -16710,10 +16707,10 @@
         <v>596</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="C86" s="9" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="15.75" customHeight="1">
@@ -16862,10 +16859,10 @@
         <v>626</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="C110" s="9" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="15.75" customHeight="1">
@@ -16873,10 +16870,10 @@
         <v>627</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="15.75" customHeight="1">
@@ -16884,10 +16881,10 @@
         <v>628</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C112" s="9" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="15.75" customHeight="1"/>
@@ -16896,10 +16893,10 @@
         <v>629</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="C114" s="9" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="15.75" customHeight="1">
@@ -16907,10 +16904,10 @@
         <v>630</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="C115" s="9" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="15.75" customHeight="1">
@@ -16918,10 +16915,10 @@
         <v>631</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="C116" s="9" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="15.75" customHeight="1"/>
@@ -16967,7 +16964,7 @@
         <v>641</v>
       </c>
       <c r="C122" s="9" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="15.75" customHeight="1"/>
@@ -16979,7 +16976,7 @@
         <v>643</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="15.75" customHeight="1">
@@ -16990,7 +16987,7 @@
         <v>645</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15.75" customHeight="1">
@@ -17001,7 +16998,7 @@
         <v>645</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17909,7 +17906,7 @@
         <v>188</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="C229" s="76" t="s">
         <v>1065</v>
@@ -17920,7 +17917,7 @@
         <v>189</v>
       </c>
       <c r="B230" s="10" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="C230" s="85" t="s">
         <v>976</v>
@@ -17931,7 +17928,7 @@
         <v>190</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="C231" s="76" t="s">
         <v>192</v>
@@ -17943,7 +17940,7 @@
         <v>193</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="C233" s="76" t="s">
         <v>1066</v>
@@ -21290,7 +21287,7 @@
         <v>39</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="18"/>
@@ -22106,7 +22103,7 @@
         <v>281</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C54" s="18"/>
       <c r="D54" s="18"/>
@@ -22134,7 +22131,7 @@
         <v>282</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C55" s="18"/>
       <c r="D55" s="18"/>
@@ -22162,7 +22159,7 @@
         <v>283</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C56" s="18"/>
       <c r="D56" s="18"/>
@@ -22190,7 +22187,7 @@
         <v>284</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="C57" s="18"/>
       <c r="D57" s="18"/>
@@ -22218,7 +22215,7 @@
         <v>285</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C58" s="18"/>
       <c r="D58" s="18"/>
@@ -22246,7 +22243,7 @@
         <v>286</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="C59" s="18"/>
       <c r="D59" s="18"/>
@@ -22274,7 +22271,7 @@
         <v>287</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="C60" s="18"/>
       <c r="D60" s="18"/>
@@ -22302,7 +22299,7 @@
         <v>288</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="C61" s="18"/>
       <c r="D61" s="18"/>
@@ -22330,7 +22327,7 @@
         <v>289</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="C62" s="18"/>
       <c r="D62" s="18"/>
@@ -22358,7 +22355,7 @@
         <v>290</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="C63" s="18"/>
       <c r="D63" s="18"/>
@@ -22386,7 +22383,7 @@
         <v>291</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C64" s="18"/>
       <c r="D64" s="18"/>
@@ -22414,7 +22411,7 @@
         <v>292</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="C65" s="18"/>
       <c r="D65" s="18"/>
@@ -22442,7 +22439,7 @@
         <v>293</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="C66" s="18"/>
       <c r="D66" s="18"/>
@@ -22470,7 +22467,7 @@
         <v>294</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C67" s="18"/>
       <c r="D67" s="18"/>
@@ -22522,7 +22519,7 @@
         <v>295</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="C69" s="18"/>
       <c r="D69" s="18"/>
@@ -22578,7 +22575,7 @@
         <v>298</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C71" s="18"/>
       <c r="D71" s="18"/>
@@ -22630,7 +22627,7 @@
         <v>299</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C73" s="18"/>
       <c r="D73" s="18"/>
@@ -22658,7 +22655,7 @@
         <v>300</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="C74" s="18"/>
       <c r="D74" s="18"/>
@@ -23142,7 +23139,7 @@
         <v>319</v>
       </c>
       <c r="B92" s="22" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="C92" s="18"/>
       <c r="D92" s="18"/>
@@ -23170,7 +23167,7 @@
         <v>320</v>
       </c>
       <c r="B93" s="22" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="18"/>
@@ -23278,7 +23275,7 @@
         <v>323</v>
       </c>
       <c r="B97" s="9" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="C97" s="18"/>
       <c r="D97" s="18"/>
@@ -23306,7 +23303,7 @@
         <v>324</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="C98" s="18"/>
       <c r="D98" s="18"/>
@@ -23334,7 +23331,7 @@
         <v>325</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="C99" s="18"/>
       <c r="D99" s="18"/>
@@ -23386,7 +23383,7 @@
         <v>326</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="C101" s="18"/>
       <c r="D101" s="18"/>
@@ -23442,7 +23439,7 @@
         <v>327</v>
       </c>
       <c r="B103" s="22" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="C103" s="18"/>
       <c r="D103" s="18"/>
@@ -23522,7 +23519,7 @@
         <v>330</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="C106" s="18"/>
       <c r="D106" s="18"/>
@@ -23550,7 +23547,7 @@
         <v>331</v>
       </c>
       <c r="B107" s="9" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="C107" s="18"/>
       <c r="D107" s="18"/>
@@ -23702,7 +23699,7 @@
         <v>333</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C113" s="18"/>
       <c r="D113" s="18"/>
@@ -23754,7 +23751,7 @@
         <v>334</v>
       </c>
       <c r="B115" s="24" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="C115" s="18"/>
       <c r="D115" s="18"/>
@@ -23806,7 +23803,7 @@
         <v>335</v>
       </c>
       <c r="B117" s="93" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="C117" s="18"/>
       <c r="D117" s="18"/>
@@ -24114,7 +24111,7 @@
         <v>340</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C129" s="18"/>
       <c r="D129" s="18"/>
@@ -24170,7 +24167,7 @@
         <v>341</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C131" s="18"/>
       <c r="D131" s="18"/>
@@ -24922,7 +24919,7 @@
         <v>370</v>
       </c>
       <c r="B159" s="95" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="C159" s="18"/>
       <c r="D159" s="18"/>
@@ -25298,7 +25295,7 @@
         <v>441</v>
       </c>
       <c r="B173" s="9" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C173" s="18"/>
       <c r="D173" s="18"/>
@@ -25347,10 +25344,10 @@
     </row>
     <row r="175" spans="1:22" ht="15.75" customHeight="1">
       <c r="A175" s="92" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="B175" s="95" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="C175" s="18"/>
       <c r="D175" s="18"/>
@@ -25375,10 +25372,10 @@
     </row>
     <row r="176" spans="1:22" ht="15.75" customHeight="1">
       <c r="A176" s="92" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="B176" s="95" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="C176" s="18"/>
       <c r="D176" s="18"/>
@@ -25403,10 +25400,10 @@
     </row>
     <row r="177" spans="1:22" ht="15.75" customHeight="1">
       <c r="A177" s="92" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="B177" s="95" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="C177" s="18"/>
       <c r="D177" s="18"/>
@@ -25431,10 +25428,10 @@
     </row>
     <row r="178" spans="1:22" ht="15.75" customHeight="1">
       <c r="A178" s="92" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="B178" s="95" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="C178" s="18"/>
       <c r="D178" s="18"/>
@@ -25459,10 +25456,10 @@
     </row>
     <row r="179" spans="1:22" ht="15.75" customHeight="1">
       <c r="A179" s="92" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="B179" s="95" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="C179" s="18"/>
       <c r="D179" s="18"/>
@@ -25571,10 +25568,10 @@
     </row>
     <row r="183" spans="1:22" ht="15.75" customHeight="1" thickBot="1">
       <c r="A183" s="92" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="B183" s="95" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="C183" s="18"/>
       <c r="D183" s="18"/>
@@ -25629,10 +25626,10 @@
     </row>
     <row r="185" spans="1:22" ht="15.75" customHeight="1">
       <c r="A185" s="92" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="B185" s="95" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="C185" s="18"/>
       <c r="D185" s="18"/>
@@ -25681,10 +25678,10 @@
     </row>
     <row r="187" spans="1:22" ht="15.75" customHeight="1">
       <c r="A187" s="92" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="B187" s="95" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="C187" s="18"/>
       <c r="D187" s="18"/>
@@ -32075,7 +32072,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="C2" s="51" t="s">
         <v>1048</v>
@@ -32273,10 +32270,10 @@
         <v>441</v>
       </c>
       <c r="B17" s="9" t="s">
+        <v>1218</v>
+      </c>
+      <c r="C17" s="62" t="s">
         <v>1219</v>
-      </c>
-      <c r="C17" s="62" t="s">
-        <v>1220</v>
       </c>
       <c r="D17" s="9" t="s">
         <v>442</v>
@@ -32550,7 +32547,7 @@
         <v>67</v>
       </c>
       <c r="C42" s="60" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>67</v>
@@ -32584,7 +32581,7 @@
         <v>1070</v>
       </c>
       <c r="C45" s="60" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>1070</v>
@@ -32595,13 +32592,13 @@
         <v>89</v>
       </c>
       <c r="B46" s="9" t="s">
+        <v>1223</v>
+      </c>
+      <c r="C46" s="60" t="s">
         <v>1224</v>
       </c>
-      <c r="C46" s="60" t="s">
-        <v>1225</v>
-      </c>
       <c r="D46" s="9" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="47" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -32632,7 +32629,7 @@
         <v>482</v>
       </c>
       <c r="C49" s="60" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>482</v>
@@ -34044,58 +34041,58 @@
     </row>
     <row r="169" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A169" s="9" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B169" s="9" t="s">
         <v>1162</v>
       </c>
-      <c r="B169" s="9" t="s">
+      <c r="C169" s="62" t="s">
         <v>1163</v>
       </c>
-      <c r="C169" s="62" t="s">
-        <v>1164</v>
-      </c>
       <c r="D169" s="9" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A170" s="9" t="s">
+        <v>1164</v>
+      </c>
+      <c r="B170" s="9" t="s">
         <v>1165</v>
       </c>
-      <c r="B170" s="9" t="s">
-        <v>1166</v>
-      </c>
       <c r="C170" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="D170" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="171" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A171" s="92" t="s">
+        <v>1166</v>
+      </c>
+      <c r="B171" s="9" t="s">
         <v>1167</v>
       </c>
-      <c r="B171" s="9" t="s">
-        <v>1168</v>
-      </c>
       <c r="C171" s="9" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="D171" s="9" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A172" s="9" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B172" s="9" t="s">
+        <v>1168</v>
+      </c>
+      <c r="C172" s="9" t="s">
         <v>1169</v>
       </c>
-      <c r="C172" s="9" t="s">
-        <v>1170</v>
-      </c>
       <c r="D172" s="9" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -34105,39 +34102,39 @@
     <row r="174" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A174" s="29"/>
       <c r="B174" s="35" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C174" s="66"/>
     </row>
     <row r="175" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A175" s="9" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="B175" s="9" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="C175" s="62" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="D175" s="9" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A176" s="9" t="s">
+        <v>1230</v>
+      </c>
+      <c r="B176" s="9" t="s">
         <v>1231</v>
-      </c>
-      <c r="B176" s="9" t="s">
-        <v>1232</v>
       </c>
       <c r="C176" s="9"/>
     </row>
     <row r="177" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A177" s="92" t="s">
+        <v>1232</v>
+      </c>
+      <c r="B177" s="9" t="s">
         <v>1233</v>
-      </c>
-      <c r="B177" s="9" t="s">
-        <v>1234</v>
       </c>
       <c r="C177" s="9"/>
     </row>

</xml_diff>

<commit_message>
Patient & Provider Happy Path  Updated code 09/05/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B0C8326-C362-4610-AC69-4FCF85F670DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA572738-7A69-4413-B516-BCC5322A0949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2632" uniqueCount="1299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2632" uniqueCount="1302">
   <si>
     <t>KEY</t>
   </si>
@@ -3951,7 +3951,16 @@
     <t>VISIT_APPOINTMENT_DETAILS_UHC_USING_CARD_PAYMENT</t>
   </si>
   <si>
-    <t>Automation1_HC1;Automation1_Loc1;Myself (AUTO AUTOCHRISC4);A new issue;Visit;9:00 AM;GP2WHITE;AFTER_THREE_DAYS</t>
+    <t>https://v2webprdfeature.mmh-demo.com/home</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Automation1_Loc1;Myself (CHRISC4 AUTOCHRISC4);A new issue;Visit;9:00 AM;GP2WHITE;AFTER_THREE_DAYS</t>
+  </si>
+  <si>
+    <t>https://v2portal.mmhnz.cloud/home</t>
+  </si>
+  <si>
+    <t>31 Jan 2025;03 Apr 2025;Prod Test 31 jan 25;VM07 Loc1 Evo Prod;</t>
   </si>
 </sst>
 </file>
@@ -4032,6 +4041,7 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Quattrocento Sans"/>
+      <family val="2"/>
     </font>
     <font>
       <u/>
@@ -4925,7 +4935,7 @@
         <v>1261</v>
       </c>
       <c r="C2" s="74" t="s">
-        <v>1048</v>
+        <v>1300</v>
       </c>
       <c r="D2" s="57" t="s">
         <v>1124</v>
@@ -9299,7 +9309,7 @@
         <v>1258</v>
       </c>
       <c r="C146" s="76" t="s">
-        <v>1065</v>
+        <v>1301</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>1125</v>
@@ -10953,7 +10963,7 @@
         <v>1296</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>1298</v>
+        <v>1299</v>
       </c>
       <c r="C200" s="76" t="s">
         <v>1127</v>
@@ -16717,7 +16727,7 @@
     <hyperlink ref="C2" r:id="rId3" xr:uid="{51DC6A58-9863-4BA4-8D62-1794D9D55E09}"/>
     <hyperlink ref="D2" r:id="rId4" xr:uid="{1F6963B5-04E2-4635-B2CC-308E91119C44}"/>
     <hyperlink ref="B2" r:id="rId5" xr:uid="{8629E203-331A-40A5-8963-16BA6F44E7E0}"/>
-    <hyperlink ref="B5" r:id="rId6" tooltip="mailto:autochrisc4@mmh-demo.com" display="mailto:Autochrisc4@mmh-demo.com" xr:uid="{D1666DDB-633D-47C3-AC1F-E8A14BD8B3D3}"/>
+    <hyperlink ref="B5" r:id="rId6" xr:uid="{D1666DDB-633D-47C3-AC1F-E8A14BD8B3D3}"/>
     <hyperlink ref="B4" r:id="rId7" tooltip="mailto:autochrisc4@mmh-demo.com" display="mailto:Autochrisc4@mmh-demo.com" xr:uid="{F7DB5A72-67FE-429D-AD24-95A3552918F2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
@@ -16777,7 +16787,7 @@
       <c r="B2" s="51" t="s">
         <v>1261</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="51" t="s">
         <v>1048</v>
       </c>
     </row>
@@ -21297,6 +21307,7 @@
     <hyperlink ref="C16" r:id="rId19" xr:uid="{6BAF1573-2EFB-4846-8986-088AD7BBB8AE}"/>
     <hyperlink ref="C3" r:id="rId20" xr:uid="{0014955C-7397-4069-B2DC-1F6C4B21F53F}"/>
     <hyperlink ref="B2" r:id="rId21" xr:uid="{FDCB0381-0C4A-4281-8093-8D3F723B9334}"/>
+    <hyperlink ref="C2" r:id="rId22" xr:uid="{A07F2944-7E15-41CA-AD10-4E6BD1E11282}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait"/>
@@ -32737,7 +32748,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>1261</v>
+        <v>1298</v>
       </c>
       <c r="C2" s="51" t="s">
         <v>1048</v>
@@ -36392,8 +36403,8 @@
     <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{3EFD36B0-2228-45CC-AC19-2290C035AA1A}"/>
     <hyperlink ref="C145" r:id="rId3" xr:uid="{D585080A-FC84-4C4E-BBDD-A485B5C6854A}"/>
-    <hyperlink ref="B2" r:id="rId4" xr:uid="{AE460962-5ECE-43B9-8307-F9744D2F7A7C}"/>
-    <hyperlink ref="C2" r:id="rId5" xr:uid="{A4DEE308-051E-4F9C-9C85-8307AF9E1ACB}"/>
+    <hyperlink ref="C2" r:id="rId4" xr:uid="{A4DEE308-051E-4F9C-9C85-8307AF9E1ACB}"/>
+    <hyperlink ref="B2" r:id="rId5" xr:uid="{6B02F5FD-321A-4EC6-B083-48F8A4F10673}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId6"/>

</xml_diff>

<commit_message>
Patient Happy Path  Updated code 20/05/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA572738-7A69-4413-B516-BCC5322A0949}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57015136-9C9D-4DB4-9347-531F3B407720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3957,10 +3957,10 @@
     <t>Automation1_HC1;Automation1_Loc1;Myself (CHRISC4 AUTOCHRISC4);A new issue;Visit;9:00 AM;GP2WHITE;AFTER_THREE_DAYS</t>
   </si>
   <si>
-    <t>https://v2portal.mmhnz.cloud/home</t>
-  </si>
-  <si>
-    <t>31 Jan 2025;03 Apr 2025;Prod Test 31 jan 25;VM07 Loc1 Evo Prod;</t>
+    <t>https://app.managemyhealth.co.nz/home</t>
+  </si>
+  <si>
+    <t>31 Jan 2025;16 May 2025;Prod Test 31 jan 25;VM07 Loc1 Evo Prod;</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Patient Happy Path  Updated code 29/05/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57015136-9C9D-4DB4-9347-531F3B407720}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB49A04-3DCF-441B-BC98-4A0B83DE31C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2632" uniqueCount="1302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2670" uniqueCount="1316">
   <si>
     <t>KEY</t>
   </si>
@@ -3324,9 +3324,6 @@
     <t>Automation1_HC1;Automation1_Loc1;AFTER_FIVE_DAYS;15;AUTO AUTOCHRISC1;GP2WHITE;A new issue;Pay at Health Centre;TODAY</t>
   </si>
   <si>
-    <t>Automation1_HC1;Automation1_Loc2;Myself (AUTO AUTOCHRISC1);A new issue;Video;9:00 AM;Book Video Appointment;GP3 White;AFTER_THREE_DAYS</t>
-  </si>
-  <si>
     <t>Automation1_HC1;Automation1_Loc2;Myself (AUTO AUTOCHRISC1);A new issue;Visit;9:00 AM;GP3 White;AFTER_THREE_DAYS;Automation1_Loc1;Automation1_Loc2</t>
   </si>
   <si>
@@ -3522,9 +3519,6 @@
     <t>VM07 HC Evo Prod;2;Hour(s);Day(s);12:00 AM - 01:00 AM;1</t>
   </si>
   <si>
-    <t>Dr B Beta;Dr Percival Chapman;GP1 Vm07 Loc1</t>
-  </si>
-  <si>
     <t>UAT</t>
   </si>
   <si>
@@ -3711,9 +3705,6 @@
     <t>BOOK_VISIT_APPOINTMENT_RULE_C</t>
   </si>
   <si>
-    <t>Automation1_HC1;Repeat Prescription;Gp2White;Gp1 A1 L1</t>
-  </si>
-  <si>
     <t>VM07 HC Evo Prod;Repeat Prescription;Dr B Beta</t>
   </si>
   <si>
@@ -3951,16 +3942,67 @@
     <t>VISIT_APPOINTMENT_DETAILS_UHC_USING_CARD_PAYMENT</t>
   </si>
   <si>
-    <t>https://v2webprdfeature.mmh-demo.com/home</t>
-  </si>
-  <si>
     <t>Automation1_HC1;Automation1_Loc1;Myself (CHRISC4 AUTOCHRISC4);A new issue;Visit;9:00 AM;GP2WHITE;AFTER_THREE_DAYS</t>
   </si>
   <si>
-    <t>https://app.managemyhealth.co.nz/home</t>
-  </si>
-  <si>
     <t>31 Jan 2025;16 May 2025;Prod Test 31 jan 25;VM07 Loc1 Evo Prod;</t>
+  </si>
+  <si>
+    <t>PATIENT_REPEAT_SCRIPT_SETTINGS_DATA</t>
+  </si>
+  <si>
+    <t>VM07 Loc1 Evo Prod;Repeat Prescription;Dr B Beta;Gp2 Vm07 Loc2</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Repeat Prescription;Gp1 A1 L1;Gp3 White</t>
+  </si>
+  <si>
+    <t>Automation1_Loc1;Gp1 A1 L1;Deliver Meds by Pharmacy</t>
+  </si>
+  <si>
+    <t>Automation1_Loc1;Pacifen 10mg Tab;pending;48 Hours;GP2WHITE</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Automation1_Loc1;Lab Result enquiry;Clinical Staff;Gp2White;Compose Msg Testing_RANDOM;Compose Message Testing_RANDOM;MMHtest.jpg</t>
+  </si>
+  <si>
+    <t>SETUP_SERVICE_RECEIVED_MESSAGE_DETAILS</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Automation1_Loc1;TestAutomation;Patient;Auto;Received Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg;Compose Message_RANDOM;Body : Reply Message Testing_RANDOM;Compose Message Testing_RANDOM;TestAutomation</t>
+  </si>
+  <si>
+    <t>VM07 HC Evo Prod;VM07 Loc1 Evo Prod;TestAutomation;Patient;peter;Received Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg</t>
+  </si>
+  <si>
+    <t>Dr Percival Chapman;Dr B Beta;GP1 Vm07 Loc1</t>
+  </si>
+  <si>
+    <t>AUTO_PRA_LOC1_PHONE_APPOINTMENT_DETAILS</t>
+  </si>
+  <si>
+    <t>Phone;VM07 Loc2 Evo Prod;GP2 VM07 Loc2</t>
+  </si>
+  <si>
+    <t>AUTO_PRA_LOC1_PHONE_APPOINTMENT_SUMMARY</t>
+  </si>
+  <si>
+    <t>AUTO_PRA_LOC1_APPOINTMENT_DETAILS_FOR_CANCEL</t>
+  </si>
+  <si>
+    <t>AUTO_PRA_LOC1_APPOINTMENT_DETAILS_AFTER_CANCELLED</t>
+  </si>
+  <si>
+    <t>Bruce Wayne;GP1 A1 L1;GP2WHITE;GP3 White;Gp4 White;Gp5white;Gp6 White</t>
+  </si>
+  <si>
+    <t>Bruce Wayne;GP1 A1 L1;GP2WHITE;Gp5white</t>
+  </si>
+  <si>
+    <t>VM07 Loc1 Evo Prod;2 g, Twice Daily, 1 week;Dr B Beta</t>
+  </si>
+  <si>
+    <t>2 time per day</t>
   </si>
 </sst>
 </file>
@@ -4417,7 +4459,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4666,6 +4708,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" xfId="3"/>
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="3" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4899,7 +4945,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="C1" s="73" t="s">
         <v>1</v>
@@ -4932,13 +4978,13 @@
         <v>2</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="C2" s="74" t="s">
-        <v>1300</v>
+        <v>1048</v>
       </c>
       <c r="D2" s="57" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
@@ -4995,10 +5041,10 @@
     </row>
     <row r="4" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A4" s="1" t="s">
-        <v>1262</v>
+        <v>1259</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>1264</v>
+        <v>1261</v>
       </c>
       <c r="C4" s="75"/>
       <c r="D4" s="4"/>
@@ -5024,10 +5070,10 @@
     </row>
     <row r="5" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A5" s="1" t="s">
-        <v>1265</v>
+        <v>1262</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>1263</v>
+        <v>1260</v>
       </c>
       <c r="C5" s="75"/>
       <c r="D5" s="4"/>
@@ -5177,7 +5223,7 @@
         <v>1072</v>
       </c>
       <c r="C10" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>1072</v>
@@ -5334,7 +5380,7 @@
         <v>1073</v>
       </c>
       <c r="C15" s="76" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>1073</v>
@@ -5483,7 +5529,7 @@
         <v>1074</v>
       </c>
       <c r="C20" s="76" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>1074</v>
@@ -5632,7 +5678,7 @@
         <v>1075</v>
       </c>
       <c r="C25" s="76" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>1075</v>
@@ -5781,7 +5827,7 @@
         <v>1072</v>
       </c>
       <c r="C30" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>1072</v>
@@ -6169,7 +6215,7 @@
     </row>
     <row r="43" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="B43" s="8" t="s">
-        <v>1266</v>
+        <v>1263</v>
       </c>
       <c r="C43"/>
       <c r="E43" s="2"/>
@@ -6194,13 +6240,13 @@
     </row>
     <row r="44" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A44" s="1" t="s">
-        <v>1270</v>
+        <v>1267</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1267</v>
+        <v>1264</v>
       </c>
       <c r="C44" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D44" s="1" t="s">
         <v>1072</v>
@@ -6227,10 +6273,10 @@
     </row>
     <row r="45" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A45" s="1" t="s">
-        <v>1271</v>
+        <v>1268</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>1268</v>
+        <v>1265</v>
       </c>
       <c r="C45" s="76" t="s">
         <v>13</v>
@@ -6260,10 +6306,10 @@
     </row>
     <row r="46" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A46" s="1" t="s">
-        <v>1272</v>
+        <v>1269</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>1269</v>
+        <v>1266</v>
       </c>
       <c r="C46" s="76" t="s">
         <v>16</v>
@@ -6326,10 +6372,10 @@
     </row>
     <row r="48" spans="1:23" ht="13.5" customHeight="1">
       <c r="A48" t="s">
-        <v>1273</v>
+        <v>1270</v>
       </c>
       <c r="B48" t="s">
-        <v>1274</v>
+        <v>1271</v>
       </c>
       <c r="C48"/>
       <c r="E48" s="2"/>
@@ -6398,13 +6444,13 @@
     </row>
     <row r="51" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A51" s="1" t="s">
-        <v>1275</v>
+        <v>1272</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>1279</v>
+        <v>1276</v>
       </c>
       <c r="C51" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="E51" s="2"/>
       <c r="F51" s="2"/>
@@ -6428,10 +6474,10 @@
     </row>
     <row r="52" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A52" s="1" t="s">
-        <v>1276</v>
+        <v>1273</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>1280</v>
+        <v>1277</v>
       </c>
       <c r="C52" s="76" t="s">
         <v>13</v>
@@ -6458,10 +6504,10 @@
     </row>
     <row r="53" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A53" s="1" t="s">
-        <v>1277</v>
+        <v>1274</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>1281</v>
+        <v>1278</v>
       </c>
       <c r="C53" s="76" t="s">
         <v>16</v>
@@ -6518,10 +6564,10 @@
     </row>
     <row r="55" spans="1:23" ht="13.5" customHeight="1">
       <c r="A55" t="s">
-        <v>1278</v>
+        <v>1275</v>
       </c>
       <c r="B55" t="s">
-        <v>1282</v>
+        <v>1279</v>
       </c>
       <c r="C55"/>
       <c r="E55" s="2"/>
@@ -7707,7 +7753,7 @@
         <v>106</v>
       </c>
       <c r="C94" s="76" t="s">
-        <v>1050</v>
+        <v>1314</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>106</v>
@@ -8040,10 +8086,18 @@
       <c r="W104" s="2"/>
     </row>
     <row r="105" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
-      <c r="A105" s="9"/>
-      <c r="B105" s="9"/>
-      <c r="C105" s="77"/>
-      <c r="D105" s="9"/>
+      <c r="A105" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C105" s="76" t="s">
+        <v>1315</v>
+      </c>
+      <c r="D105" s="1" t="s">
+        <v>112</v>
+      </c>
       <c r="E105" s="2"/>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
@@ -8060,6 +8114,9 @@
       <c r="R105" s="2"/>
       <c r="S105" s="2"/>
       <c r="T105" s="2"/>
+      <c r="U105" s="2"/>
+      <c r="V105" s="2"/>
+      <c r="W105" s="2"/>
     </row>
     <row r="106" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A106" s="1" t="s">
@@ -9306,13 +9363,13 @@
         <v>188</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>1258</v>
+        <v>1255</v>
       </c>
       <c r="C146" s="76" t="s">
-        <v>1301</v>
+        <v>1296</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="E146" s="2"/>
       <c r="F146" s="2"/>
@@ -9339,7 +9396,7 @@
         <v>189</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="C147" s="85" t="s">
         <v>976</v>
@@ -9372,7 +9429,7 @@
         <v>190</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="C148" s="76" t="s">
         <v>192</v>
@@ -9430,7 +9487,7 @@
         <v>193</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
       <c r="C150" s="76" t="s">
         <v>1066</v>
@@ -9499,7 +9556,7 @@
         <v>1033</v>
       </c>
       <c r="C152" s="76" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D152" s="1" t="s">
         <v>1033</v>
@@ -9999,7 +10056,7 @@
         <v>1076</v>
       </c>
       <c r="C168" s="76" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="D168" s="1" t="s">
         <v>1076</v>
@@ -10032,7 +10089,7 @@
         <v>1076</v>
       </c>
       <c r="C169" s="76" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="D169" s="1" t="s">
         <v>1076</v>
@@ -10230,7 +10287,7 @@
         <v>1077</v>
       </c>
       <c r="C175" s="87" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="D175" s="15" t="s">
         <v>1077</v>
@@ -10263,7 +10320,7 @@
         <v>1078</v>
       </c>
       <c r="C176" s="76" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>1078</v>
@@ -10296,7 +10353,7 @@
         <v>1079</v>
       </c>
       <c r="C177" s="76" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="D177" s="1" t="s">
         <v>1079</v>
@@ -10362,7 +10419,7 @@
         <v>1080</v>
       </c>
       <c r="C179" s="76" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="D179" s="1" t="s">
         <v>1080</v>
@@ -10648,10 +10705,10 @@
     </row>
     <row r="189" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A189" s="1" t="s">
-        <v>1287</v>
+        <v>1284</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>1289</v>
+        <v>1286</v>
       </c>
       <c r="C189" s="55"/>
       <c r="D189" s="2"/>
@@ -10677,10 +10734,10 @@
     </row>
     <row r="190" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A190" s="1" t="s">
-        <v>1288</v>
+        <v>1285</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>1290</v>
+        <v>1287</v>
       </c>
       <c r="C190" s="55"/>
       <c r="D190" s="2"/>
@@ -10730,10 +10787,10 @@
     </row>
     <row r="192" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A192" s="1" t="s">
-        <v>1291</v>
+        <v>1288</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>1289</v>
+        <v>1286</v>
       </c>
       <c r="C192"/>
       <c r="D192" s="2"/>
@@ -10759,10 +10816,10 @@
     </row>
     <row r="193" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A193" s="1" t="s">
-        <v>1292</v>
+        <v>1289</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>1290</v>
+        <v>1287</v>
       </c>
       <c r="C193" s="55"/>
       <c r="D193" s="2"/>
@@ -10812,13 +10869,13 @@
     </row>
     <row r="195" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A195" s="1" t="s">
-        <v>1294</v>
+        <v>1291</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>1293</v>
+        <v>1290</v>
       </c>
       <c r="C195" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D195" s="2"/>
       <c r="E195" s="2"/>
@@ -10843,7 +10900,7 @@
     </row>
     <row r="196" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A196" s="1" t="s">
-        <v>1295</v>
+        <v>1292</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>12</v>
@@ -10960,13 +11017,13 @@
     </row>
     <row r="200" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A200" s="1" t="s">
-        <v>1296</v>
+        <v>1293</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>1299</v>
+        <v>1295</v>
       </c>
       <c r="C200" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="D200" s="2"/>
       <c r="E200" s="2"/>
@@ -10991,7 +11048,7 @@
     </row>
     <row r="201" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A201" s="1" t="s">
-        <v>1297</v>
+        <v>1294</v>
       </c>
       <c r="B201" s="1" t="s">
         <v>12</v>
@@ -16754,7 +16811,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>1</v>
@@ -16785,7 +16842,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>1261</v>
+        <v>1258</v>
       </c>
       <c r="C2" s="51" t="s">
         <v>1048</v>
@@ -16827,7 +16884,7 @@
         <v>1076</v>
       </c>
       <c r="C11" s="76" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
     </row>
     <row r="12" spans="1:23" ht="30" thickBot="1">
@@ -16835,10 +16892,10 @@
         <v>218</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="C12" s="76" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
     </row>
     <row r="13" spans="1:23" ht="30.75" thickBot="1">
@@ -16846,10 +16903,10 @@
         <v>557</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>1231</v>
+        <v>1228</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>1233</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -16860,7 +16917,7 @@
         <v>559</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>1234</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="30">
@@ -16868,10 +16925,10 @@
         <v>375</v>
       </c>
       <c r="B15" s="9" t="s">
+        <v>1229</v>
+      </c>
+      <c r="C15" s="9" t="s">
         <v>1232</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>1235</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -16904,7 +16961,7 @@
         <v>1079</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>1236</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -16978,7 +17035,7 @@
         <v>1072</v>
       </c>
       <c r="C28" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
@@ -17023,7 +17080,7 @@
         <v>1073</v>
       </c>
       <c r="C33" s="76" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="13.5" customHeight="1" thickBot="1">
@@ -17058,7 +17115,7 @@
         <v>1074</v>
       </c>
       <c r="C38" s="76" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
     </row>
     <row r="39" spans="1:3" ht="13.5" customHeight="1" thickBot="1">
@@ -17093,7 +17150,7 @@
         <v>1075</v>
       </c>
       <c r="C43" s="76" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
     </row>
     <row r="44" spans="1:3" ht="13.5" customHeight="1" thickBot="1">
@@ -17128,7 +17185,7 @@
         <v>1072</v>
       </c>
       <c r="C48" s="76" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
     </row>
     <row r="49" spans="1:3" ht="13.5" customHeight="1" thickBot="1">
@@ -17258,7 +17315,7 @@
         <v>571</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>1254</v>
+        <v>1251</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>573</v>
@@ -17270,7 +17327,7 @@
         <v>574</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>1256</v>
+        <v>1253</v>
       </c>
       <c r="C69" s="9" t="s">
         <v>576</v>
@@ -17281,7 +17338,7 @@
         <v>577</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>1255</v>
+        <v>1252</v>
       </c>
       <c r="C70" s="9" t="s">
         <v>578</v>
@@ -17292,7 +17349,7 @@
         <v>579</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>1253</v>
+        <v>1250</v>
       </c>
       <c r="C71" s="9" t="s">
         <v>581</v>
@@ -17339,7 +17396,7 @@
         <v>589</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>1257</v>
+        <v>1254</v>
       </c>
       <c r="C78" s="9" t="s">
         <v>591</v>
@@ -17372,7 +17429,7 @@
         <v>382</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>1245</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17381,10 +17438,10 @@
         <v>596</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>1260</v>
+        <v>1257</v>
       </c>
       <c r="C86" s="9" t="s">
-        <v>1246</v>
+        <v>1243</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="15.75" customHeight="1">
@@ -17533,10 +17590,10 @@
         <v>626</v>
       </c>
       <c r="B110" s="9" t="s">
+        <v>1236</v>
+      </c>
+      <c r="C110" s="9" t="s">
         <v>1239</v>
-      </c>
-      <c r="C110" s="9" t="s">
-        <v>1242</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="15.75" customHeight="1">
@@ -17544,10 +17601,10 @@
         <v>627</v>
       </c>
       <c r="B111" s="9" t="s">
+        <v>1237</v>
+      </c>
+      <c r="C111" s="9" t="s">
         <v>1240</v>
-      </c>
-      <c r="C111" s="9" t="s">
-        <v>1243</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="15.75" customHeight="1">
@@ -17555,10 +17612,10 @@
         <v>628</v>
       </c>
       <c r="B112" s="9" t="s">
+        <v>1238</v>
+      </c>
+      <c r="C112" s="9" t="s">
         <v>1241</v>
-      </c>
-      <c r="C112" s="9" t="s">
-        <v>1244</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17567,10 +17624,10 @@
         <v>629</v>
       </c>
       <c r="B114" s="9" t="s">
+        <v>1244</v>
+      </c>
+      <c r="C114" s="9" t="s">
         <v>1247</v>
-      </c>
-      <c r="C114" s="9" t="s">
-        <v>1250</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="15.75" customHeight="1">
@@ -17578,10 +17635,10 @@
         <v>630</v>
       </c>
       <c r="B115" s="9" t="s">
+        <v>1245</v>
+      </c>
+      <c r="C115" s="9" t="s">
         <v>1248</v>
-      </c>
-      <c r="C115" s="9" t="s">
-        <v>1251</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="15.75" customHeight="1">
@@ -17589,10 +17646,10 @@
         <v>631</v>
       </c>
       <c r="B116" s="9" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C116" s="9" t="s">
         <v>1249</v>
-      </c>
-      <c r="C116" s="9" t="s">
-        <v>1252</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17638,7 +17695,7 @@
         <v>641</v>
       </c>
       <c r="C122" s="9" t="s">
-        <v>1237</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17650,7 +17707,7 @@
         <v>643</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="15.75" customHeight="1">
@@ -17661,7 +17718,7 @@
         <v>645</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15.75" customHeight="1">
@@ -17672,7 +17729,7 @@
         <v>645</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>1238</v>
+        <v>1235</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="15.75" customHeight="1"/>
@@ -18580,7 +18637,7 @@
         <v>188</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>1258</v>
+        <v>1255</v>
       </c>
       <c r="C229" s="76" t="s">
         <v>1065</v>
@@ -18591,7 +18648,7 @@
         <v>189</v>
       </c>
       <c r="B230" s="10" t="s">
-        <v>1159</v>
+        <v>1157</v>
       </c>
       <c r="C230" s="85" t="s">
         <v>976</v>
@@ -18602,7 +18659,7 @@
         <v>190</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>1160</v>
+        <v>1158</v>
       </c>
       <c r="C231" s="76" t="s">
         <v>192</v>
@@ -18614,7 +18671,7 @@
         <v>193</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>1259</v>
+        <v>1256</v>
       </c>
       <c r="C233" s="76" t="s">
         <v>1066</v>
@@ -18639,7 +18696,7 @@
         <v>1033</v>
       </c>
       <c r="C235" s="76" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
     </row>
     <row r="236" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
@@ -21329,7 +21386,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>1</v>
@@ -21359,7 +21416,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="C2" s="18"/>
       <c r="D2" s="18"/>
@@ -21963,7 +22020,7 @@
         <v>39</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1171</v>
+        <v>1169</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="18"/>
@@ -22779,7 +22836,7 @@
         <v>281</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>1172</v>
+        <v>1170</v>
       </c>
       <c r="C54" s="18"/>
       <c r="D54" s="18"/>
@@ -22807,7 +22864,7 @@
         <v>282</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>1173</v>
+        <v>1171</v>
       </c>
       <c r="C55" s="18"/>
       <c r="D55" s="18"/>
@@ -22835,7 +22892,7 @@
         <v>283</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>1174</v>
+        <v>1172</v>
       </c>
       <c r="C56" s="18"/>
       <c r="D56" s="18"/>
@@ -22863,7 +22920,7 @@
         <v>284</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>1175</v>
+        <v>1173</v>
       </c>
       <c r="C57" s="18"/>
       <c r="D57" s="18"/>
@@ -22891,7 +22948,7 @@
         <v>285</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>1176</v>
+        <v>1174</v>
       </c>
       <c r="C58" s="18"/>
       <c r="D58" s="18"/>
@@ -22919,7 +22976,7 @@
         <v>286</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>1177</v>
+        <v>1175</v>
       </c>
       <c r="C59" s="18"/>
       <c r="D59" s="18"/>
@@ -22947,7 +23004,7 @@
         <v>287</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>1178</v>
+        <v>1176</v>
       </c>
       <c r="C60" s="18"/>
       <c r="D60" s="18"/>
@@ -22975,7 +23032,7 @@
         <v>288</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>1179</v>
+        <v>1177</v>
       </c>
       <c r="C61" s="18"/>
       <c r="D61" s="18"/>
@@ -23003,7 +23060,7 @@
         <v>289</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>1180</v>
+        <v>1178</v>
       </c>
       <c r="C62" s="18"/>
       <c r="D62" s="18"/>
@@ -23031,7 +23088,7 @@
         <v>290</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>1181</v>
+        <v>1179</v>
       </c>
       <c r="C63" s="18"/>
       <c r="D63" s="18"/>
@@ -23059,7 +23116,7 @@
         <v>291</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>1182</v>
+        <v>1180</v>
       </c>
       <c r="C64" s="18"/>
       <c r="D64" s="18"/>
@@ -23087,7 +23144,7 @@
         <v>292</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>1183</v>
+        <v>1181</v>
       </c>
       <c r="C65" s="18"/>
       <c r="D65" s="18"/>
@@ -23115,7 +23172,7 @@
         <v>293</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>1184</v>
+        <v>1182</v>
       </c>
       <c r="C66" s="18"/>
       <c r="D66" s="18"/>
@@ -23143,7 +23200,7 @@
         <v>294</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>1185</v>
+        <v>1183</v>
       </c>
       <c r="C67" s="18"/>
       <c r="D67" s="18"/>
@@ -23195,7 +23252,7 @@
         <v>295</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>1204</v>
+        <v>1202</v>
       </c>
       <c r="C69" s="18"/>
       <c r="D69" s="18"/>
@@ -23251,7 +23308,7 @@
         <v>298</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>1186</v>
+        <v>1184</v>
       </c>
       <c r="C71" s="18"/>
       <c r="D71" s="18"/>
@@ -23303,7 +23360,7 @@
         <v>299</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>1201</v>
+        <v>1199</v>
       </c>
       <c r="C73" s="18"/>
       <c r="D73" s="18"/>
@@ -23331,7 +23388,7 @@
         <v>300</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>1202</v>
+        <v>1200</v>
       </c>
       <c r="C74" s="18"/>
       <c r="D74" s="18"/>
@@ -23815,7 +23872,7 @@
         <v>319</v>
       </c>
       <c r="B92" s="22" t="s">
-        <v>1187</v>
+        <v>1185</v>
       </c>
       <c r="C92" s="18"/>
       <c r="D92" s="18"/>
@@ -23843,7 +23900,7 @@
         <v>320</v>
       </c>
       <c r="B93" s="22" t="s">
-        <v>1188</v>
+        <v>1186</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="18"/>
@@ -23951,7 +24008,7 @@
         <v>323</v>
       </c>
       <c r="B97" s="9" t="s">
-        <v>1189</v>
+        <v>1187</v>
       </c>
       <c r="C97" s="18"/>
       <c r="D97" s="18"/>
@@ -23979,7 +24036,7 @@
         <v>324</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>1190</v>
+        <v>1188</v>
       </c>
       <c r="C98" s="18"/>
       <c r="D98" s="18"/>
@@ -24007,7 +24064,7 @@
         <v>325</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>1191</v>
+        <v>1189</v>
       </c>
       <c r="C99" s="18"/>
       <c r="D99" s="18"/>
@@ -24059,7 +24116,7 @@
         <v>326</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>1199</v>
+        <v>1197</v>
       </c>
       <c r="C101" s="18"/>
       <c r="D101" s="18"/>
@@ -24115,7 +24172,7 @@
         <v>327</v>
       </c>
       <c r="B103" s="22" t="s">
-        <v>1192</v>
+        <v>1190</v>
       </c>
       <c r="C103" s="18"/>
       <c r="D103" s="18"/>
@@ -24195,7 +24252,7 @@
         <v>330</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>1200</v>
+        <v>1198</v>
       </c>
       <c r="C106" s="18"/>
       <c r="D106" s="18"/>
@@ -24223,7 +24280,7 @@
         <v>331</v>
       </c>
       <c r="B107" s="9" t="s">
-        <v>1193</v>
+        <v>1191</v>
       </c>
       <c r="C107" s="18"/>
       <c r="D107" s="18"/>
@@ -24375,7 +24432,7 @@
         <v>333</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>1196</v>
+        <v>1194</v>
       </c>
       <c r="C113" s="18"/>
       <c r="D113" s="18"/>
@@ -24427,7 +24484,7 @@
         <v>334</v>
       </c>
       <c r="B115" s="24" t="s">
-        <v>1197</v>
+        <v>1195</v>
       </c>
       <c r="C115" s="18"/>
       <c r="D115" s="18"/>
@@ -24479,7 +24536,7 @@
         <v>335</v>
       </c>
       <c r="B117" s="92" t="s">
-        <v>1198</v>
+        <v>1196</v>
       </c>
       <c r="C117" s="18"/>
       <c r="D117" s="18"/>
@@ -24787,7 +24844,7 @@
         <v>340</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>1194</v>
+        <v>1192</v>
       </c>
       <c r="C129" s="18"/>
       <c r="D129" s="18"/>
@@ -24843,7 +24900,7 @@
         <v>341</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>1195</v>
+        <v>1193</v>
       </c>
       <c r="C131" s="18"/>
       <c r="D131" s="18"/>
@@ -25595,7 +25652,7 @@
         <v>370</v>
       </c>
       <c r="B159" s="94" t="s">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="C159" s="18"/>
       <c r="D159" s="18"/>
@@ -25971,7 +26028,7 @@
         <v>441</v>
       </c>
       <c r="B173" s="9" t="s">
-        <v>1205</v>
+        <v>1203</v>
       </c>
       <c r="C173" s="18"/>
       <c r="D173" s="18"/>
@@ -26020,10 +26077,10 @@
     </row>
     <row r="175" spans="1:22" ht="15.75" customHeight="1">
       <c r="A175" s="91" t="s">
+        <v>1204</v>
+      </c>
+      <c r="B175" s="94" t="s">
         <v>1206</v>
-      </c>
-      <c r="B175" s="94" t="s">
-        <v>1208</v>
       </c>
       <c r="C175" s="18"/>
       <c r="D175" s="18"/>
@@ -26048,10 +26105,10 @@
     </row>
     <row r="176" spans="1:22" ht="15.75" customHeight="1">
       <c r="A176" s="91" t="s">
+        <v>1205</v>
+      </c>
+      <c r="B176" s="94" t="s">
         <v>1207</v>
-      </c>
-      <c r="B176" s="94" t="s">
-        <v>1209</v>
       </c>
       <c r="C176" s="18"/>
       <c r="D176" s="18"/>
@@ -26076,10 +26133,10 @@
     </row>
     <row r="177" spans="1:22" ht="15.75" customHeight="1">
       <c r="A177" s="91" t="s">
-        <v>1210</v>
+        <v>1208</v>
       </c>
       <c r="B177" s="94" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="C177" s="18"/>
       <c r="D177" s="18"/>
@@ -26104,10 +26161,10 @@
     </row>
     <row r="178" spans="1:22" ht="15.75" customHeight="1">
       <c r="A178" s="91" t="s">
+        <v>1209</v>
+      </c>
+      <c r="B178" s="94" t="s">
         <v>1211</v>
-      </c>
-      <c r="B178" s="94" t="s">
-        <v>1213</v>
       </c>
       <c r="C178" s="18"/>
       <c r="D178" s="18"/>
@@ -26132,10 +26189,10 @@
     </row>
     <row r="179" spans="1:22" ht="15.75" customHeight="1">
       <c r="A179" s="91" t="s">
-        <v>1214</v>
+        <v>1212</v>
       </c>
       <c r="B179" s="94" t="s">
-        <v>1209</v>
+        <v>1207</v>
       </c>
       <c r="C179" s="18"/>
       <c r="D179" s="18"/>
@@ -26190,7 +26247,7 @@
         <v>1087</v>
       </c>
       <c r="C181" s="62" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D181" s="18"/>
       <c r="E181" s="18"/>
@@ -26244,10 +26301,10 @@
     </row>
     <row r="183" spans="1:22" ht="15.75" customHeight="1" thickBot="1">
       <c r="A183" s="91" t="s">
-        <v>1215</v>
+        <v>1213</v>
       </c>
       <c r="B183" s="94" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="C183" s="18"/>
       <c r="D183" s="18"/>
@@ -26278,7 +26335,7 @@
         <v>505</v>
       </c>
       <c r="C184" s="62" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="D184" s="18"/>
       <c r="E184" s="18"/>
@@ -26302,10 +26359,10 @@
     </row>
     <row r="185" spans="1:22" ht="15.75" customHeight="1">
       <c r="A185" s="91" t="s">
-        <v>1216</v>
+        <v>1214</v>
       </c>
       <c r="B185" s="94" t="s">
-        <v>1212</v>
+        <v>1210</v>
       </c>
       <c r="C185" s="18"/>
       <c r="D185" s="18"/>
@@ -26354,10 +26411,10 @@
     </row>
     <row r="187" spans="1:22" ht="15.75" customHeight="1">
       <c r="A187" s="91" t="s">
-        <v>1217</v>
+        <v>1215</v>
       </c>
       <c r="B187" s="94" t="s">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="C187" s="18"/>
       <c r="D187" s="18"/>
@@ -30872,7 +30929,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="C1" s="26" t="s">
         <v>1</v>
@@ -32734,7 +32791,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>1156</v>
+        <v>1154</v>
       </c>
       <c r="C1" s="65" t="s">
         <v>1</v>
@@ -32747,10 +32804,10 @@
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="57" t="s">
-        <v>1298</v>
-      </c>
-      <c r="C2" s="51" t="s">
+      <c r="B2" s="96" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C2" s="72" t="s">
         <v>1048</v>
       </c>
       <c r="D2" t="s">
@@ -32823,7 +32880,7 @@
         <v>1082</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>417</v>
@@ -32837,7 +32894,7 @@
         <v>1083</v>
       </c>
       <c r="C9" s="62" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>420</v>
@@ -32848,10 +32905,10 @@
         <v>422</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="C10" s="62" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>423</v>
@@ -32862,10 +32919,10 @@
         <v>425</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="C11" s="62" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>426</v>
@@ -32876,10 +32933,10 @@
         <v>428</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="C12" s="62" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>429</v>
@@ -32890,10 +32947,10 @@
         <v>431</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C13" s="62" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>432</v>
@@ -32904,10 +32961,10 @@
         <v>434</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>435</v>
@@ -32942,94 +32999,100 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A17" s="9" t="s">
-        <v>441</v>
+      <c r="A17" s="91" t="s">
+        <v>1297</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>1218</v>
+        <v>442</v>
       </c>
       <c r="C17" s="62" t="s">
-        <v>1219</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>442</v>
-      </c>
+        <v>1298</v>
+      </c>
+      <c r="D17" s="9"/>
     </row>
     <row r="18" spans="1:4" ht="15.75" thickBot="1">
       <c r="A18" s="9" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>98</v>
+        <v>1299</v>
       </c>
       <c r="C18" s="62" t="s">
-        <v>976</v>
+        <v>1216</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>98</v>
+        <v>442</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" thickBot="1">
       <c r="A19" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>1300</v>
+      </c>
+      <c r="C19" s="62" t="s">
+        <v>976</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.75" thickBot="1">
+      <c r="A20" s="9" t="s">
         <v>446</v>
       </c>
-      <c r="B19" s="31" t="s">
+      <c r="B20" s="31" t="s">
         <v>447</v>
       </c>
-      <c r="C19" s="62" t="s">
+      <c r="C20" s="62" t="s">
         <v>448</v>
       </c>
-      <c r="D19" s="31" t="s">
+      <c r="D20" s="31" t="s">
         <v>447</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="30.75" thickBot="1">
-      <c r="A20" s="9" t="s">
-        <v>449</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>450</v>
-      </c>
-      <c r="C20" s="62" t="s">
-        <v>451</v>
-      </c>
-      <c r="D20" s="9" t="s">
-        <v>450</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A21" s="9" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="C21" s="62" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A22" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>453</v>
+      </c>
+      <c r="C22" s="62" t="s">
+        <v>454</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A23" s="9" t="s">
         <v>455</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B23" s="9" t="s">
         <v>456</v>
       </c>
-      <c r="C22" s="62" t="s">
+      <c r="C23" s="62" t="s">
         <v>457</v>
       </c>
-      <c r="D22" s="9" t="s">
+      <c r="D23" s="9" t="s">
         <v>456</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A23" s="9"/>
-      <c r="B23" s="9"/>
-      <c r="C23" s="62"/>
-      <c r="D23" s="9"/>
     </row>
     <row r="24" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A24" s="9"/>
@@ -33068,261 +33131,253 @@
       <c r="D29" s="9"/>
     </row>
     <row r="30" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A30" s="29"/>
-      <c r="B30" s="29" t="s">
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="62"/>
+      <c r="D30" s="9"/>
+    </row>
+    <row r="31" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A31" s="29"/>
+      <c r="B31" s="29" t="s">
         <v>458</v>
       </c>
-      <c r="C30" s="66"/>
-      <c r="D30" s="29" t="s">
+      <c r="C31" s="66"/>
+      <c r="D31" s="29" t="s">
         <v>458</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A31" s="9" t="s">
-        <v>459</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>460</v>
-      </c>
-      <c r="C31" s="61" t="s">
-        <v>1103</v>
-      </c>
-      <c r="D31" s="9" t="s">
-        <v>460</v>
       </c>
     </row>
     <row r="32" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A32" s="9" t="s">
-        <v>462</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C32" s="67" t="s">
-        <v>968</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>5</v>
+        <v>459</v>
+      </c>
+      <c r="B32" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="C32" s="61" t="s">
+        <v>1102</v>
+      </c>
+      <c r="D32" s="9" t="s">
+        <v>460</v>
       </c>
     </row>
     <row r="33" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A33" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>56</v>
-      </c>
-      <c r="C33" s="60" t="s">
-        <v>57</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>56</v>
+        <v>462</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C33" s="67" t="s">
+        <v>968</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A34" s="9" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C34" s="60" t="s">
-        <v>966</v>
+        <v>57</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A35" s="9" t="s">
-        <v>468</v>
-      </c>
-      <c r="B35" s="9" t="s">
-        <v>469</v>
-      </c>
-      <c r="C35" s="62" t="s">
-        <v>469</v>
-      </c>
-      <c r="D35" s="9" t="s">
-        <v>469</v>
+        <v>58</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C35" s="60" t="s">
+        <v>966</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A36" s="9" t="s">
+        <v>468</v>
+      </c>
+      <c r="B36" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="C36" s="62" t="s">
+        <v>469</v>
+      </c>
+      <c r="D36" s="9" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A37" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B37" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="C36" s="59" t="s">
+      <c r="C37" s="59" t="s">
         <v>92</v>
       </c>
-      <c r="D36" s="1" t="s">
+      <c r="D37" s="1" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="37" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A37" s="9"/>
-      <c r="B37" s="9"/>
-      <c r="C37" s="62"/>
-      <c r="D37" s="9"/>
-    </row>
     <row r="38" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A38" s="1" t="s">
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="62"/>
+      <c r="D38" s="9"/>
+    </row>
+    <row r="39" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A39" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B39" s="1" t="s">
         <v>1068</v>
       </c>
-      <c r="C38" s="60" t="s">
+      <c r="C39" s="60" t="s">
         <v>989</v>
       </c>
-      <c r="D38" s="1" t="s">
+      <c r="D39" s="1" t="s">
         <v>1068</v>
       </c>
     </row>
-    <row r="39" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A39" s="33" t="s">
+    <row r="40" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A40" s="33" t="s">
         <v>79</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B40" s="1" t="s">
         <v>1069</v>
       </c>
-      <c r="C39" s="60" t="s">
+      <c r="C40" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="D39" s="1" t="s">
+      <c r="D40" s="1" t="s">
         <v>1069</v>
       </c>
     </row>
-    <row r="40" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A40" s="9"/>
-      <c r="B40" s="9"/>
-      <c r="C40" s="62"/>
-      <c r="D40" s="9"/>
-    </row>
     <row r="41" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A41" s="13" t="s">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9"/>
+      <c r="C41" s="62"/>
+      <c r="D41" s="9"/>
+    </row>
+    <row r="42" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A42" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B42" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C41" s="60" t="s">
+      <c r="C42" s="60" t="s">
         <v>65</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>64</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A42" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="C42" s="60" t="s">
-        <v>1220</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A43" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C43" s="60" t="s">
+        <v>1217</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A44" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B44" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="C43" s="76" t="s">
+      <c r="C44" s="76" t="s">
         <v>71</v>
       </c>
-      <c r="D43" s="1" t="s">
+      <c r="D44" s="1" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="44" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A44" s="1"/>
-      <c r="B44" s="1"/>
-      <c r="C44" s="76"/>
-      <c r="D44" s="1"/>
-    </row>
     <row r="45" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A45" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>1070</v>
-      </c>
-      <c r="C45" s="60" t="s">
-        <v>1222</v>
-      </c>
-      <c r="D45" s="1" t="s">
-        <v>1070</v>
-      </c>
+      <c r="A45" s="1"/>
+      <c r="B45" s="1"/>
+      <c r="C45" s="76"/>
+      <c r="D45" s="1"/>
     </row>
     <row r="46" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A46" s="9" t="s">
+        <v>87</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>1070</v>
+      </c>
+      <c r="C46" s="60" t="s">
+        <v>1219</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>1070</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A47" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B46" s="9" t="s">
-        <v>1223</v>
-      </c>
-      <c r="C46" s="60" t="s">
-        <v>1224</v>
-      </c>
-      <c r="D46" s="9" t="s">
-        <v>1223</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A47" s="9"/>
-      <c r="B47" s="1"/>
-      <c r="C47" s="59"/>
-      <c r="D47" s="1"/>
+      <c r="B47" s="9" t="s">
+        <v>1301</v>
+      </c>
+      <c r="C47" s="60" t="s">
+        <v>1221</v>
+      </c>
+      <c r="D47" s="9" t="s">
+        <v>1220</v>
+      </c>
     </row>
     <row r="48" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A48" s="9" t="s">
+      <c r="A48" s="9"/>
+      <c r="B48" s="1"/>
+      <c r="C48" s="59"/>
+      <c r="D48" s="1"/>
+    </row>
+    <row r="49" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A49" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B49" s="1" t="s">
         <v>480</v>
       </c>
-      <c r="C48" s="60" t="s">
+      <c r="C49" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="D48" s="1" t="s">
+      <c r="D49" s="1" t="s">
         <v>480</v>
-      </c>
-    </row>
-    <row r="49" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A49" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>482</v>
-      </c>
-      <c r="C49" s="60" t="s">
-        <v>1221</v>
-      </c>
-      <c r="D49" s="1" t="s">
-        <v>482</v>
       </c>
     </row>
     <row r="50" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A50" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>1047</v>
-      </c>
-      <c r="C50" s="76" t="s">
-        <v>77</v>
+        <v>482</v>
+      </c>
+      <c r="C50" s="60" t="s">
+        <v>1218</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>1047</v>
+        <v>482</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
@@ -33345,224 +33400,238 @@
       <c r="W50" s="2"/>
     </row>
     <row r="51" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A51" s="34"/>
-      <c r="B51" s="34" t="s">
+      <c r="A51" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>1047</v>
+      </c>
+      <c r="C51" s="76" t="s">
+        <v>77</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>1047</v>
+      </c>
+    </row>
+    <row r="52" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A52" s="34"/>
+      <c r="B52" s="34" t="s">
         <v>484</v>
       </c>
-      <c r="C51" s="68"/>
-      <c r="D51" s="34" t="s">
+      <c r="C52" s="68"/>
+      <c r="D52" s="34" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="52" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A52" s="9"/>
-      <c r="B52" s="9"/>
-      <c r="C52" s="62"/>
-      <c r="D52" s="9"/>
-    </row>
     <row r="53" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A53" s="1" t="s">
-        <v>485</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>1076</v>
-      </c>
-      <c r="C53" s="59" t="s">
-        <v>1131</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>217</v>
-      </c>
+      <c r="A53" s="9"/>
+      <c r="B53" s="9"/>
+      <c r="C53" s="62"/>
+      <c r="D53" s="9"/>
     </row>
     <row r="54" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
       <c r="A54" s="1" t="s">
+        <v>485</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>1302</v>
+      </c>
+      <c r="C54" s="59" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="55" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A55" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="B54" s="15" t="s">
+      <c r="B55" s="15" t="s">
         <v>1084</v>
       </c>
-      <c r="C54" s="64" t="s">
-        <v>1133</v>
-      </c>
-      <c r="D54" s="15" t="s">
+      <c r="C55" s="64" t="s">
+        <v>1132</v>
+      </c>
+      <c r="D55" s="15" t="s">
         <v>1020</v>
       </c>
     </row>
-    <row r="55" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A55" s="1"/>
-      <c r="B55" s="1"/>
-      <c r="C55" s="59"/>
-      <c r="D55" s="1"/>
-    </row>
     <row r="56" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A56" s="1" t="s">
-        <v>231</v>
-      </c>
-      <c r="B56" s="1" t="s">
-        <v>1079</v>
-      </c>
-      <c r="C56" s="60" t="s">
-        <v>1135</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>232</v>
-      </c>
+      <c r="A56" s="91" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B56" s="15" t="s">
+        <v>1304</v>
+      </c>
+      <c r="C56" s="64" t="s">
+        <v>1305</v>
+      </c>
+      <c r="D56" s="1"/>
     </row>
     <row r="57" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
       <c r="A57" s="1" t="s">
-        <v>486</v>
+        <v>231</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="C57" s="59" t="s">
-        <v>222</v>
+        <v>1079</v>
+      </c>
+      <c r="C57" s="60" t="s">
+        <v>1134</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
     </row>
     <row r="58" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
       <c r="A58" s="1" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C58" s="59" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="59" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
       <c r="A59" s="1" t="s">
+        <v>487</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="C59" s="59" t="s">
+        <v>224</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="60" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A60" s="1" t="s">
         <v>488</v>
       </c>
-      <c r="B59" s="1" t="s">
+      <c r="B60" s="1" t="s">
         <v>226</v>
       </c>
-      <c r="C59" s="59" t="s">
+      <c r="C60" s="59" t="s">
         <v>226</v>
       </c>
-      <c r="D59" s="1" t="s">
+      <c r="D60" s="1" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="60" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A60" s="28" t="s">
+    <row r="61" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A61" s="28" t="s">
         <v>227</v>
       </c>
-      <c r="B60" s="1" t="s">
+      <c r="B61" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="C60" s="59" t="s">
+      <c r="C61" s="59" t="s">
         <v>980</v>
       </c>
-      <c r="D60" s="1" t="s">
+      <c r="D61" s="1" t="s">
         <v>228</v>
-      </c>
-    </row>
-    <row r="61" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A61" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="B61" s="1" t="s">
-        <v>1076</v>
-      </c>
-      <c r="C61" s="60" t="s">
-        <v>1131</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="62" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
       <c r="A62" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>1076</v>
+      </c>
+      <c r="C62" s="60" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D62" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="63" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A63" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B62" s="1" t="s">
+      <c r="B63" s="1" t="s">
         <v>490</v>
       </c>
-      <c r="C62" s="60" t="s">
+      <c r="C63" s="60" t="s">
         <v>966</v>
       </c>
-      <c r="D62" s="1" t="s">
+      <c r="D63" s="1" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="63" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A63" s="34"/>
-      <c r="B63" s="34" t="s">
+    <row r="64" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A64" s="34"/>
+      <c r="B64" s="34" t="s">
         <v>491</v>
       </c>
-      <c r="C63" s="68"/>
-      <c r="D63" s="34" t="s">
+      <c r="C64" s="68"/>
+      <c r="D64" s="34" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="64" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A64" s="1" t="s">
+    <row r="65" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A65" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B64" s="1" t="s">
+      <c r="B65" s="1" t="s">
         <v>492</v>
       </c>
-      <c r="C64" s="60" t="s">
+      <c r="C65" s="60" t="s">
         <v>57</v>
       </c>
-      <c r="D64" s="1" t="s">
+      <c r="D65" s="1" t="s">
         <v>492</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A65" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B65" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C65" s="62" t="s">
-        <v>18</v>
-      </c>
-      <c r="D65" s="9" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="66" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A66" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>1044</v>
-      </c>
-      <c r="C66" s="59" t="s">
-        <v>94</v>
-      </c>
-      <c r="D66" s="1" t="s">
-        <v>1044</v>
+        <v>17</v>
+      </c>
+      <c r="B66" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C66" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="D66" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="67" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A67" s="9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>1044</v>
+      </c>
+      <c r="C67" s="59" t="s">
+        <v>94</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>1044</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A68" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="B67" s="1" t="s">
+      <c r="B68" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C67" s="59" t="s">
+      <c r="C68" s="59" t="s">
         <v>96</v>
       </c>
-      <c r="D67" s="1" t="s">
+      <c r="D68" s="1" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="68" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A68" s="9"/>
-      <c r="B68" s="9"/>
-      <c r="C68" s="62"/>
-      <c r="D68" s="9"/>
     </row>
     <row r="69" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A69" s="9"/>
@@ -33589,190 +33658,190 @@
       <c r="D72" s="9"/>
     </row>
     <row r="73" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A73" s="34"/>
-      <c r="B73" s="34" t="s">
+      <c r="A73" s="9"/>
+      <c r="B73" s="9"/>
+      <c r="C73" s="62"/>
+      <c r="D73" s="9"/>
+    </row>
+    <row r="74" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A74" s="34"/>
+      <c r="B74" s="34" t="s">
         <v>493</v>
       </c>
-      <c r="C73" s="68"/>
-      <c r="D73" s="34" t="s">
+      <c r="C74" s="68"/>
+      <c r="D74" s="34" t="s">
         <v>493</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A74" s="9" t="s">
-        <v>494</v>
-      </c>
-      <c r="B74" s="9" t="s">
-        <v>1085</v>
-      </c>
-      <c r="C74" s="62" t="s">
-        <v>1144</v>
-      </c>
-      <c r="D74" s="9" t="s">
-        <v>495</v>
       </c>
     </row>
     <row r="75" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A75" s="9" t="s">
+        <v>494</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C75" s="62" t="s">
+        <v>1143</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A76" s="9" t="s">
         <v>496</v>
       </c>
-      <c r="B75" s="9" t="s">
+      <c r="B76" s="9" t="s">
         <v>497</v>
       </c>
-      <c r="C75" s="62" t="s">
+      <c r="C76" s="62" t="s">
         <v>497</v>
       </c>
-      <c r="D75" s="9" t="s">
+      <c r="D76" s="9" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="76" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A76" s="9"/>
-      <c r="B76" s="9" t="s">
+    <row r="77" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A77" s="9"/>
+      <c r="B77" s="9" t="s">
         <v>498</v>
       </c>
-      <c r="C76" s="62" t="s">
+      <c r="C77" s="62" t="s">
         <v>498</v>
       </c>
-      <c r="D76" s="9" t="s">
+      <c r="D77" s="9" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="77" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A77" s="9" t="s">
+    <row r="78" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A78" s="9" t="s">
         <v>499</v>
       </c>
-      <c r="B77" s="1" t="s">
+      <c r="B78" s="1" t="s">
         <v>1086</v>
       </c>
-      <c r="C77" s="60" t="s">
-        <v>1131</v>
-      </c>
-      <c r="D77" s="1" t="s">
+      <c r="C78" s="60" t="s">
+        <v>1130</v>
+      </c>
+      <c r="D78" s="1" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="78" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A78" s="1"/>
-      <c r="B78" s="1"/>
-      <c r="C78" s="62"/>
-      <c r="D78" s="1"/>
-    </row>
     <row r="79" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A79" s="9" t="s">
+      <c r="A79" s="1"/>
+      <c r="B79" s="1"/>
+      <c r="C79" s="62"/>
+      <c r="D79" s="1"/>
+    </row>
+    <row r="80" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A80" s="9" t="s">
         <v>501</v>
       </c>
-      <c r="B79" s="9" t="s">
+      <c r="B80" s="9" t="s">
         <v>498</v>
       </c>
-      <c r="C79" s="62" t="s">
+      <c r="C80" s="62" t="s">
         <v>498</v>
       </c>
-      <c r="D79" s="9" t="s">
+      <c r="D80" s="9" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="80" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A80" s="34"/>
-      <c r="B80" s="34" t="s">
+    <row r="81" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A81" s="34"/>
+      <c r="B81" s="34" t="s">
         <v>502</v>
       </c>
-      <c r="C80" s="68"/>
-      <c r="D80" s="34" t="s">
+      <c r="C81" s="68"/>
+      <c r="D81" s="34" t="s">
         <v>502</v>
       </c>
     </row>
-    <row r="81" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A81" s="9"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="62"/>
-      <c r="D81" s="9"/>
-    </row>
     <row r="82" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A82" s="9" t="s">
-        <v>381</v>
-      </c>
-      <c r="B82" s="9" t="s">
-        <v>1087</v>
-      </c>
-      <c r="C82" s="62" t="s">
-        <v>1145</v>
-      </c>
-      <c r="D82" s="9" t="s">
-        <v>382</v>
-      </c>
+      <c r="A82" s="9"/>
+      <c r="B82" s="9"/>
+      <c r="C82" s="62"/>
+      <c r="D82" s="9"/>
     </row>
     <row r="83" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A83" s="9" t="s">
-        <v>383</v>
+        <v>381</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>384</v>
+        <v>1087</v>
       </c>
       <c r="C83" s="62" t="s">
-        <v>503</v>
+        <v>1144</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>384</v>
+        <v>382</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A84" s="9" t="s">
-        <v>385</v>
+        <v>383</v>
       </c>
       <c r="B84" s="9" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
       <c r="C84" s="62" t="s">
-        <v>386</v>
+        <v>503</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A85" s="9" t="s">
-        <v>411</v>
+        <v>385</v>
       </c>
       <c r="B85" s="9" t="s">
-        <v>412</v>
+        <v>386</v>
       </c>
       <c r="C85" s="62" t="s">
-        <v>1104</v>
+        <v>386</v>
       </c>
       <c r="D85" s="9" t="s">
-        <v>412</v>
+        <v>386</v>
       </c>
     </row>
     <row r="86" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A86" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B86" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="C86" s="62" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D86" s="9" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A87" s="9" t="s">
         <v>504</v>
       </c>
-      <c r="B86" s="9" t="s">
+      <c r="B87" s="9" t="s">
         <v>505</v>
       </c>
-      <c r="C86" s="62" t="s">
-        <v>1105</v>
-      </c>
-      <c r="D86" s="9" t="s">
+      <c r="C87" s="62" t="s">
+        <v>1104</v>
+      </c>
+      <c r="D87" s="9" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="87" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A87" s="34"/>
-      <c r="B87" s="34" t="s">
+    <row r="88" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A88" s="34"/>
+      <c r="B88" s="34" t="s">
         <v>506</v>
       </c>
-      <c r="C87" s="68"/>
-      <c r="D87" s="34" t="s">
+      <c r="C88" s="68"/>
+      <c r="D88" s="34" t="s">
         <v>506</v>
       </c>
-    </row>
-    <row r="88" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A88" s="9"/>
-      <c r="B88" s="9"/>
-      <c r="C88" s="62"/>
-      <c r="D88" s="9"/>
     </row>
     <row r="89" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A89" s="9"/>
@@ -33787,290 +33856,274 @@
       <c r="D90" s="9"/>
     </row>
     <row r="91" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A91" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B91" s="9" t="s">
-        <v>1072</v>
-      </c>
-      <c r="C91" s="60" t="s">
-        <v>1127</v>
-      </c>
-      <c r="D91" s="9" t="s">
-        <v>10</v>
-      </c>
+      <c r="A91" s="9"/>
+      <c r="B91" s="9"/>
+      <c r="C91" s="62"/>
+      <c r="D91" s="9"/>
     </row>
     <row r="92" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A92" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B92" s="9" t="s">
-        <v>12</v>
+        <v>1072</v>
       </c>
       <c r="C92" s="60" t="s">
-        <v>13</v>
+        <v>1126</v>
       </c>
       <c r="D92" s="9" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="93" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A93" s="9" t="s">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="B93" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C93" s="62" t="s">
-        <v>18</v>
+        <v>12</v>
+      </c>
+      <c r="C93" s="60" t="s">
+        <v>13</v>
       </c>
       <c r="D93" s="9" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
     </row>
     <row r="94" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A94" s="9" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B94" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C94" s="60" t="s">
-        <v>16</v>
+        <v>18</v>
+      </c>
+      <c r="C94" s="62" t="s">
+        <v>18</v>
       </c>
       <c r="D94" s="9" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="95" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A95" s="9" t="s">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="C95" s="60" t="s">
-        <v>46</v>
+        <v>16</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>45</v>
+        <v>15</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A96" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B96" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C96" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="D96" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A97" s="9" t="s">
         <v>507</v>
       </c>
-      <c r="B96" s="9" t="s">
+      <c r="B97" s="9" t="s">
         <v>1088</v>
       </c>
-      <c r="C96" s="62" t="s">
-        <v>1146</v>
-      </c>
-      <c r="D96" s="9" t="s">
+      <c r="C97" s="62" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D97" s="9" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="97" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A97" s="9"/>
-      <c r="B97" s="9"/>
-      <c r="C97" s="62"/>
-      <c r="D97" s="9"/>
-    </row>
     <row r="98" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A98" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B98" s="9" t="s">
-        <v>1089</v>
-      </c>
-      <c r="C98" s="60" t="s">
-        <v>1128</v>
-      </c>
-      <c r="D98" s="9" t="s">
-        <v>20</v>
-      </c>
+      <c r="A98" s="9"/>
+      <c r="B98" s="9"/>
+      <c r="C98" s="62"/>
+      <c r="D98" s="9"/>
     </row>
     <row r="99" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A99" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>22</v>
+        <v>1101</v>
       </c>
       <c r="C99" s="60" t="s">
-        <v>23</v>
+        <v>1127</v>
       </c>
       <c r="D99" s="9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="100" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A100" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B100" s="9" t="s">
+        <v>555</v>
+      </c>
+      <c r="C100" s="60" t="s">
+        <v>23</v>
+      </c>
+      <c r="D100" s="9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A101" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B100" s="9" t="s">
+      <c r="B101" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C101" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="D101" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C100" s="60" t="s">
-        <v>16</v>
-      </c>
-      <c r="D100" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="101" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A101" s="9"/>
-      <c r="B101" s="9"/>
-      <c r="C101" s="62"/>
-      <c r="D101" s="9"/>
     </row>
     <row r="102" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A102" s="29"/>
-      <c r="B102" s="35" t="s">
+      <c r="A102" s="9"/>
+      <c r="B102" s="9"/>
+      <c r="C102" s="62"/>
+      <c r="D102" s="9"/>
+    </row>
+    <row r="103" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A103" s="29"/>
+      <c r="B103" s="35" t="s">
         <v>509</v>
       </c>
-      <c r="C102" s="66"/>
-      <c r="D102" s="35" t="s">
+      <c r="C103" s="66"/>
+      <c r="D103" s="35" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="103" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A103" s="28" t="s">
+    <row r="104" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A104" s="28" t="s">
         <v>391</v>
       </c>
-      <c r="B103" s="9" t="s">
-        <v>1090</v>
-      </c>
-      <c r="C103" s="63" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D103" s="9" t="s">
+      <c r="B104" s="9" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C104" s="63" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D104" s="9" t="s">
         <v>392</v>
-      </c>
-    </row>
-    <row r="104" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A104" s="9" t="s">
-        <v>393</v>
-      </c>
-      <c r="B104" s="9" t="s">
-        <v>394</v>
-      </c>
-      <c r="C104" s="62" t="s">
-        <v>1155</v>
-      </c>
-      <c r="D104" s="9" t="s">
-        <v>394</v>
       </c>
     </row>
     <row r="105" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A105" s="9" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="B105" s="9" t="s">
-        <v>396</v>
+        <v>1313</v>
       </c>
       <c r="C105" s="62" t="s">
-        <v>1106</v>
+        <v>1306</v>
       </c>
       <c r="D105" s="9" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
     </row>
     <row r="106" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A106" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="B106" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="C106" s="62" t="s">
+        <v>1105</v>
+      </c>
+      <c r="D106" s="9" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A107" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="B106" s="9" t="s">
+      <c r="B107" s="9" t="s">
         <v>510</v>
       </c>
-      <c r="C106" s="62" t="s">
+      <c r="C107" s="62" t="s">
         <v>49</v>
       </c>
-      <c r="D106" s="9" t="s">
+      <c r="D107" s="9" t="s">
         <v>510</v>
       </c>
     </row>
-    <row r="107" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A107" s="9"/>
-      <c r="B107" s="9"/>
-      <c r="C107" s="62"/>
-      <c r="D107" s="9"/>
-    </row>
     <row r="108" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A108" s="9" t="s">
-        <v>402</v>
-      </c>
-      <c r="B108" s="9" t="s">
-        <v>511</v>
-      </c>
-      <c r="C108" s="62" t="s">
-        <v>1107</v>
-      </c>
-      <c r="D108" s="9" t="s">
-        <v>511</v>
-      </c>
+      <c r="A108" s="9"/>
+      <c r="B108" s="9"/>
+      <c r="C108" s="62"/>
+      <c r="D108" s="9"/>
     </row>
     <row r="109" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A109" s="9" t="s">
-        <v>403</v>
+        <v>1307</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C109" s="62" t="s">
-        <v>1108</v>
-      </c>
-      <c r="D109" s="9" t="s">
-        <v>25</v>
-      </c>
+        <v>1308</v>
+      </c>
+      <c r="D109" s="9"/>
     </row>
     <row r="110" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A110" s="9" t="s">
-        <v>512</v>
+      <c r="A110" s="91" t="s">
+        <v>1309</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C110" s="62" t="s">
-        <v>1109</v>
-      </c>
-      <c r="D110" s="9" t="s">
-        <v>53</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="C110" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D110" s="9"/>
     </row>
     <row r="111" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A111" s="9"/>
-      <c r="B111" s="9"/>
-      <c r="C111" s="62"/>
+      <c r="A111" s="9" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B111" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C111" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="D111" s="9"/>
     </row>
     <row r="112" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A112" s="9" t="s">
-        <v>513</v>
+        <v>1311</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>1091</v>
-      </c>
-      <c r="C112" s="63" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D112" s="9" t="s">
-        <v>400</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="C112" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D112" s="9"/>
     </row>
     <row r="113" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A113" s="9" t="s">
-        <v>514</v>
-      </c>
-      <c r="B113" s="9" t="s">
-        <v>1091</v>
-      </c>
-      <c r="C113" s="63" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D113" s="9" t="s">
-        <v>400</v>
-      </c>
+      <c r="A113" s="9"/>
+      <c r="B113" s="9"/>
+      <c r="C113" s="62"/>
+      <c r="D113" s="9"/>
     </row>
     <row r="114" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A114" s="9"/>
@@ -34080,44 +34133,44 @@
     </row>
     <row r="115" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A115" s="9" t="s">
-        <v>515</v>
+        <v>402</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>1092</v>
-      </c>
-      <c r="C115" s="63" t="s">
-        <v>1148</v>
+        <v>511</v>
+      </c>
+      <c r="C115" s="62" t="s">
+        <v>1106</v>
       </c>
       <c r="D115" s="9" t="s">
-        <v>516</v>
+        <v>511</v>
       </c>
     </row>
     <row r="116" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A116" s="9" t="s">
-        <v>397</v>
+        <v>403</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>1093</v>
-      </c>
-      <c r="C116" s="63" t="s">
-        <v>1148</v>
+        <v>25</v>
+      </c>
+      <c r="C116" s="62" t="s">
+        <v>1107</v>
       </c>
       <c r="D116" s="9" t="s">
-        <v>398</v>
+        <v>25</v>
       </c>
     </row>
     <row r="117" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A117" s="9" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
       <c r="B117" s="9" t="s">
-        <v>1093</v>
-      </c>
-      <c r="C117" s="63" t="s">
-        <v>1148</v>
+        <v>53</v>
+      </c>
+      <c r="C117" s="62" t="s">
+        <v>1108</v>
       </c>
       <c r="D117" s="9" t="s">
-        <v>398</v>
+        <v>53</v>
       </c>
     </row>
     <row r="118" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -34128,222 +34181,222 @@
     </row>
     <row r="119" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A119" s="9" t="s">
-        <v>518</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C119" s="59" t="s">
-        <v>1149</v>
-      </c>
-      <c r="D119" s="1" t="s">
-        <v>519</v>
+        <v>513</v>
+      </c>
+      <c r="B119" s="9" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C119" s="63" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D119" s="9" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A120" s="9" t="s">
-        <v>520</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C120" s="59" t="s">
-        <v>1149</v>
-      </c>
-      <c r="D120" s="1" t="s">
-        <v>521</v>
+        <v>514</v>
+      </c>
+      <c r="B120" s="9" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C120" s="63" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D120" s="9" t="s">
+        <v>400</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A121" s="9" t="s">
-        <v>522</v>
-      </c>
-      <c r="B121" s="9" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C121" s="63" t="s">
-        <v>1149</v>
-      </c>
-      <c r="D121" s="9" t="s">
-        <v>521</v>
-      </c>
+      <c r="A121" s="9"/>
+      <c r="B121" s="9"/>
+      <c r="C121" s="62"/>
+      <c r="D121" s="9"/>
     </row>
     <row r="122" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A122" s="9"/>
-      <c r="B122" s="9"/>
-      <c r="C122" s="62"/>
-      <c r="D122" s="9"/>
+      <c r="A122" s="9" t="s">
+        <v>515</v>
+      </c>
+      <c r="B122" s="9" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C122" s="63" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D122" s="9" t="s">
+        <v>516</v>
+      </c>
     </row>
     <row r="123" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A123" s="9" t="s">
-        <v>399</v>
+        <v>397</v>
       </c>
       <c r="B123" s="9" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="C123" s="63" t="s">
         <v>1147</v>
       </c>
       <c r="D123" s="9" t="s">
-        <v>400</v>
+        <v>398</v>
       </c>
     </row>
     <row r="124" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A124" s="9" t="s">
-        <v>523</v>
+        <v>517</v>
       </c>
       <c r="B124" s="9" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="C124" s="63" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D124" s="9" t="s">
         <v>398</v>
       </c>
     </row>
     <row r="125" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A125" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>1096</v>
-      </c>
-      <c r="C125" s="59" t="s">
-        <v>1149</v>
-      </c>
-      <c r="D125" s="1" t="s">
-        <v>525</v>
-      </c>
+      <c r="A125" s="9"/>
+      <c r="B125" s="9"/>
+      <c r="C125" s="62"/>
+      <c r="D125" s="9"/>
     </row>
     <row r="126" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A126" s="9"/>
-      <c r="B126" s="9"/>
-      <c r="C126" s="62"/>
-      <c r="D126" s="9"/>
+      <c r="A126" s="9" t="s">
+        <v>518</v>
+      </c>
+      <c r="B126" s="1" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C126" s="59" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D126" s="1" t="s">
+        <v>519</v>
+      </c>
     </row>
     <row r="127" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A127" s="9" t="s">
-        <v>526</v>
-      </c>
-      <c r="B127" s="9" t="s">
-        <v>527</v>
-      </c>
-      <c r="C127" s="62" t="s">
-        <v>1110</v>
-      </c>
-      <c r="D127" s="9" t="s">
-        <v>527</v>
+        <v>520</v>
+      </c>
+      <c r="B127" s="1" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C127" s="59" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D127" s="1" t="s">
+        <v>521</v>
       </c>
     </row>
     <row r="128" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A128" s="9" t="s">
-        <v>528</v>
+        <v>522</v>
       </c>
       <c r="B128" s="9" t="s">
-        <v>1060</v>
-      </c>
-      <c r="C128" s="62" t="s">
-        <v>530</v>
+        <v>1094</v>
+      </c>
+      <c r="C128" s="63" t="s">
+        <v>1148</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
     </row>
     <row r="129" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A129" s="9" t="s">
-        <v>401</v>
-      </c>
-      <c r="B129" s="9" t="s">
-        <v>394</v>
-      </c>
-      <c r="C129" s="62" t="s">
-        <v>530</v>
-      </c>
-      <c r="D129" s="9" t="s">
-        <v>394</v>
-      </c>
+      <c r="A129" s="9"/>
+      <c r="B129" s="9"/>
+      <c r="C129" s="62"/>
+      <c r="D129" s="9"/>
     </row>
     <row r="130" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A130" s="9"/>
-      <c r="B130" s="9"/>
-      <c r="C130" s="62"/>
-      <c r="D130" s="9"/>
+      <c r="A130" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="B130" s="9" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C130" s="63" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D130" s="9" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="131" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A131" s="9" t="s">
-        <v>406</v>
+        <v>523</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>407</v>
-      </c>
-      <c r="C131" s="62" t="s">
-        <v>1111</v>
+        <v>1092</v>
+      </c>
+      <c r="C131" s="63" t="s">
+        <v>1147</v>
       </c>
       <c r="D131" s="9" t="s">
-        <v>407</v>
+        <v>398</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A132" s="9"/>
-      <c r="B132" s="9"/>
-      <c r="C132" s="62"/>
-      <c r="D132" s="9"/>
+      <c r="A132" s="9" t="s">
+        <v>524</v>
+      </c>
+      <c r="B132" s="1" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C132" s="59" t="s">
+        <v>1148</v>
+      </c>
+      <c r="D132" s="1" t="s">
+        <v>525</v>
+      </c>
     </row>
     <row r="133" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A133" s="9" t="s">
-        <v>531</v>
-      </c>
-      <c r="B133" s="9" t="s">
-        <v>1097</v>
-      </c>
-      <c r="C133" s="62" t="s">
-        <v>1150</v>
-      </c>
-      <c r="D133" s="9" t="s">
-        <v>1023</v>
-      </c>
+      <c r="A133" s="9"/>
+      <c r="B133" s="9"/>
+      <c r="C133" s="62"/>
+      <c r="D133" s="9"/>
     </row>
     <row r="134" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A134" s="9" t="s">
-        <v>532</v>
+        <v>526</v>
       </c>
       <c r="B134" s="9" t="s">
-        <v>12</v>
+        <v>527</v>
       </c>
       <c r="C134" s="62" t="s">
-        <v>13</v>
+        <v>1109</v>
       </c>
       <c r="D134" s="9" t="s">
-        <v>12</v>
+        <v>527</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A135" s="9" t="s">
-        <v>533</v>
+        <v>528</v>
       </c>
       <c r="B135" s="9" t="s">
-        <v>380</v>
+        <v>1312</v>
       </c>
       <c r="C135" s="62" t="s">
-        <v>380</v>
+        <v>530</v>
       </c>
       <c r="D135" s="9" t="s">
-        <v>380</v>
+        <v>529</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A136" s="9" t="s">
-        <v>534</v>
+        <v>401</v>
       </c>
       <c r="B136" s="9" t="s">
-        <v>535</v>
+        <v>1312</v>
       </c>
       <c r="C136" s="62" t="s">
-        <v>1112</v>
+        <v>530</v>
       </c>
       <c r="D136" s="9" t="s">
-        <v>535</v>
+        <v>394</v>
       </c>
     </row>
     <row r="137" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -34354,158 +34407,154 @@
     </row>
     <row r="138" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A138" s="9" t="s">
-        <v>536</v>
+        <v>406</v>
       </c>
       <c r="B138" s="9" t="s">
-        <v>537</v>
+        <v>407</v>
       </c>
       <c r="C138" s="62" t="s">
-        <v>1113</v>
+        <v>1110</v>
       </c>
       <c r="D138" s="9" t="s">
-        <v>537</v>
+        <v>407</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A139" s="36" t="s">
-        <v>538</v>
-      </c>
-      <c r="B139" s="9" t="s">
-        <v>1098</v>
-      </c>
-      <c r="C139" s="62" t="s">
-        <v>1151</v>
-      </c>
-      <c r="D139" s="9" t="s">
-        <v>539</v>
-      </c>
+      <c r="A139" s="9"/>
+      <c r="B139" s="9"/>
+      <c r="C139" s="62"/>
+      <c r="D139" s="9"/>
     </row>
     <row r="140" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A140" s="9" t="s">
-        <v>540</v>
+        <v>531</v>
       </c>
       <c r="B140" s="9" t="s">
-        <v>1099</v>
+        <v>1096</v>
       </c>
       <c r="C140" s="62" t="s">
-        <v>1152</v>
+        <v>1149</v>
       </c>
       <c r="D140" s="9" t="s">
-        <v>541</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="141" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A141" s="9" t="s">
-        <v>542</v>
+        <v>532</v>
       </c>
       <c r="B141" s="9" t="s">
-        <v>543</v>
+        <v>12</v>
       </c>
       <c r="C141" s="62" t="s">
-        <v>1114</v>
+        <v>13</v>
       </c>
       <c r="D141" s="9" t="s">
-        <v>543</v>
+        <v>12</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A142" s="9" t="s">
-        <v>544</v>
+        <v>533</v>
       </c>
       <c r="B142" s="9" t="s">
-        <v>545</v>
+        <v>380</v>
       </c>
       <c r="C142" s="62" t="s">
-        <v>1115</v>
+        <v>380</v>
       </c>
       <c r="D142" s="9" t="s">
-        <v>545</v>
+        <v>380</v>
       </c>
     </row>
     <row r="143" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A143" s="9"/>
-      <c r="B143" s="9"/>
-      <c r="C143" s="62"/>
-      <c r="D143" s="9"/>
+      <c r="A143" s="9" t="s">
+        <v>534</v>
+      </c>
+      <c r="B143" s="9" t="s">
+        <v>535</v>
+      </c>
+      <c r="C143" s="62" t="s">
+        <v>1111</v>
+      </c>
+      <c r="D143" s="9" t="s">
+        <v>535</v>
+      </c>
     </row>
     <row r="144" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A144" s="9" t="s">
-        <v>546</v>
-      </c>
-      <c r="B144" s="9" t="s">
-        <v>1087</v>
-      </c>
-      <c r="C144" s="62" t="s">
-        <v>1145</v>
-      </c>
-      <c r="D144" s="9" t="s">
-        <v>382</v>
-      </c>
+      <c r="A144" s="9"/>
+      <c r="B144" s="9"/>
+      <c r="C144" s="62"/>
+      <c r="D144" s="9"/>
     </row>
     <row r="145" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A145" s="9" t="s">
-        <v>404</v>
+        <v>536</v>
       </c>
       <c r="B145" s="9" t="s">
-        <v>405</v>
-      </c>
-      <c r="C145" s="72" t="s">
-        <v>1116</v>
+        <v>537</v>
+      </c>
+      <c r="C145" s="62" t="s">
+        <v>1112</v>
       </c>
       <c r="D145" s="9" t="s">
-        <v>405</v>
+        <v>537</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A146" s="34"/>
-      <c r="B146" s="34" t="s">
-        <v>547</v>
-      </c>
-      <c r="C146" s="68"/>
-      <c r="D146" s="34" t="s">
-        <v>547</v>
+      <c r="A146" s="36" t="s">
+        <v>538</v>
+      </c>
+      <c r="B146" s="9" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C146" s="62" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D146" s="9" t="s">
+        <v>539</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A147" s="9" t="s">
-        <v>408</v>
+        <v>540</v>
       </c>
       <c r="B147" s="9" t="s">
-        <v>1118</v>
+        <v>1098</v>
       </c>
       <c r="C147" s="62" t="s">
-        <v>1153</v>
+        <v>1151</v>
       </c>
       <c r="D147" s="9" t="s">
-        <v>409</v>
+        <v>541</v>
       </c>
     </row>
     <row r="148" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A148" s="9" t="s">
-        <v>30</v>
+        <v>542</v>
       </c>
       <c r="B148" s="9" t="s">
-        <v>1100</v>
-      </c>
-      <c r="C148" s="60" t="s">
-        <v>1130</v>
+        <v>543</v>
+      </c>
+      <c r="C148" s="62" t="s">
+        <v>1113</v>
       </c>
       <c r="D148" s="9" t="s">
-        <v>410</v>
+        <v>543</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A149" s="9" t="s">
-        <v>31</v>
+        <v>544</v>
       </c>
       <c r="B149" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C149" s="60" t="s">
-        <v>33</v>
+        <v>545</v>
+      </c>
+      <c r="C149" s="62" t="s">
+        <v>1114</v>
       </c>
       <c r="D149" s="9" t="s">
-        <v>32</v>
+        <v>545</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -34516,404 +34565,487 @@
     </row>
     <row r="151" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A151" s="9" t="s">
+        <v>546</v>
+      </c>
+      <c r="B151" s="9" t="s">
+        <v>1087</v>
+      </c>
+      <c r="C151" s="62" t="s">
+        <v>1144</v>
+      </c>
+      <c r="D151" s="9" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="152" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A152" s="9" t="s">
+        <v>404</v>
+      </c>
+      <c r="B152" s="9" t="s">
+        <v>405</v>
+      </c>
+      <c r="C152" s="72" t="s">
+        <v>1115</v>
+      </c>
+      <c r="D152" s="9" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="153" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A153" s="34"/>
+      <c r="B153" s="34" t="s">
+        <v>547</v>
+      </c>
+      <c r="C153" s="68"/>
+      <c r="D153" s="34" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="154" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A154" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="B154" s="9" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C154" s="62" t="s">
+        <v>1152</v>
+      </c>
+      <c r="D154" s="9" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="155" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A155" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B155" s="9" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C155" s="60" t="s">
+        <v>1129</v>
+      </c>
+      <c r="D155" s="9" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="156" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A156" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B156" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C156" s="60" t="s">
+        <v>33</v>
+      </c>
+      <c r="D156" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="157" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A157" s="9"/>
+      <c r="B157" s="9"/>
+      <c r="C157" s="62"/>
+      <c r="D157" s="9"/>
+    </row>
+    <row r="158" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A158" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B151" s="9" t="s">
+      <c r="B158" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C151" s="60" t="s">
+      <c r="C158" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="D151" s="9" t="s">
+      <c r="D158" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="152" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A152" s="37"/>
-      <c r="B152" s="37"/>
-      <c r="C152" s="69"/>
-      <c r="D152" s="37"/>
-    </row>
-    <row r="153" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A153" s="6"/>
-      <c r="B153" s="38"/>
-      <c r="C153" s="70"/>
-      <c r="D153" s="38"/>
-    </row>
-    <row r="154" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A154" s="39"/>
-      <c r="B154" s="40" t="s">
+    <row r="159" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A159" s="37"/>
+      <c r="B159" s="37"/>
+      <c r="C159" s="69"/>
+      <c r="D159" s="37"/>
+    </row>
+    <row r="160" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A160" s="6"/>
+      <c r="B160" s="38"/>
+      <c r="C160" s="70"/>
+      <c r="D160" s="38"/>
+    </row>
+    <row r="161" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A161" s="39"/>
+      <c r="B161" s="40" t="s">
         <v>493</v>
       </c>
-      <c r="C154" s="71"/>
-      <c r="D154" s="40" t="s">
+      <c r="C161" s="71"/>
+      <c r="D161" s="40" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="155" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A155" s="6" t="s">
+    <row r="162" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A162" s="6" t="s">
         <v>494</v>
       </c>
-      <c r="B155" s="38" t="s">
+      <c r="B162" s="38" t="s">
         <v>1085</v>
       </c>
-      <c r="C155" s="38" t="s">
-        <v>1144</v>
-      </c>
-      <c r="D155" s="38" t="s">
+      <c r="C162" s="38" t="s">
+        <v>1143</v>
+      </c>
+      <c r="D162" s="38" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="156" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A156" s="6" t="s">
+    <row r="163" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A163" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="B156" s="38" t="s">
+      <c r="B163" s="38" t="s">
         <v>497</v>
       </c>
-      <c r="C156" s="38" t="s">
+      <c r="C163" s="38" t="s">
         <v>497</v>
       </c>
-      <c r="D156" s="38" t="s">
+      <c r="D163" s="38" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="157" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A157" s="6"/>
-      <c r="B157" s="38" t="s">
+    <row r="164" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A164" s="6"/>
+      <c r="B164" s="38" t="s">
         <v>498</v>
       </c>
-      <c r="C157" s="38" t="s">
+      <c r="C164" s="38" t="s">
         <v>498</v>
       </c>
-      <c r="D157" s="38" t="s">
+      <c r="D164" s="38" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="158" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A158" s="9"/>
-      <c r="B158" s="9"/>
-      <c r="C158" s="62"/>
-      <c r="D158" s="9"/>
-    </row>
-    <row r="159" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A159" s="29"/>
-      <c r="B159" s="35" t="s">
+    <row r="165" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A165" s="9"/>
+      <c r="B165" s="9"/>
+      <c r="C165" s="62"/>
+      <c r="D165" s="9"/>
+    </row>
+    <row r="166" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A166" s="29"/>
+      <c r="B166" s="35" t="s">
         <v>548</v>
       </c>
-      <c r="C159" s="66"/>
-      <c r="D159" s="35" t="s">
+      <c r="C166" s="66"/>
+      <c r="D166" s="35" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="160" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A160" s="9" t="s">
+    <row r="167" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A167" s="9" t="s">
         <v>549</v>
       </c>
-      <c r="B160" s="9" t="s">
-        <v>1101</v>
-      </c>
-      <c r="C160" s="62" t="s">
-        <v>1154</v>
-      </c>
-      <c r="D160" s="9" t="s">
+      <c r="B167" s="9" t="s">
+        <v>1100</v>
+      </c>
+      <c r="C167" s="62" t="s">
+        <v>1153</v>
+      </c>
+      <c r="D167" s="9" t="s">
         <v>1071</v>
       </c>
-    </row>
-    <row r="161" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A161" s="9" t="s">
-        <v>550</v>
-      </c>
-      <c r="B161" s="9" t="s">
-        <v>551</v>
-      </c>
-      <c r="C161" s="62" t="s">
-        <v>1117</v>
-      </c>
-      <c r="D161" s="9" t="s">
-        <v>551</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A162" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="B162" s="9" t="s">
-        <v>1158</v>
-      </c>
-      <c r="C162" s="62" t="s">
-        <v>1157</v>
-      </c>
-      <c r="D162" s="9" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A163" s="9"/>
-      <c r="B163" s="9"/>
-      <c r="C163" s="62"/>
-      <c r="D163" s="9"/>
-    </row>
-    <row r="164" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A164" s="1" t="s">
-        <v>552</v>
-      </c>
-      <c r="B164" s="12" t="s">
-        <v>1102</v>
-      </c>
-      <c r="C164" s="63" t="s">
-        <v>1128</v>
-      </c>
-      <c r="D164" s="12" t="s">
-        <v>553</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A165" s="1" t="s">
-        <v>554</v>
-      </c>
-      <c r="B165" s="9" t="s">
-        <v>555</v>
-      </c>
-      <c r="C165" s="62" t="s">
-        <v>23</v>
-      </c>
-      <c r="D165" s="9" t="s">
-        <v>555</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A166" s="1" t="s">
-        <v>556</v>
-      </c>
-      <c r="B166" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C166" s="62" t="s">
-        <v>16</v>
-      </c>
-      <c r="D166" s="9" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A167" s="9"/>
-      <c r="B167" s="9"/>
-      <c r="C167" s="62"/>
     </row>
     <row r="168" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A168" s="9" t="s">
-        <v>1059</v>
+        <v>550</v>
       </c>
       <c r="B168" s="9" t="s">
-        <v>1087</v>
+        <v>551</v>
       </c>
       <c r="C168" s="62" t="s">
-        <v>1145</v>
+        <v>1116</v>
       </c>
       <c r="D168" s="9" t="s">
-        <v>1087</v>
+        <v>551</v>
       </c>
     </row>
     <row r="169" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A169" s="9" t="s">
-        <v>1161</v>
+        <v>413</v>
       </c>
       <c r="B169" s="9" t="s">
-        <v>1162</v>
+        <v>1156</v>
       </c>
       <c r="C169" s="62" t="s">
-        <v>1163</v>
+        <v>1155</v>
       </c>
       <c r="D169" s="9" t="s">
-        <v>1162</v>
+        <v>414</v>
       </c>
     </row>
     <row r="170" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A170" s="9" t="s">
-        <v>1164</v>
-      </c>
-      <c r="B170" s="9" t="s">
-        <v>1165</v>
-      </c>
-      <c r="C170" s="9" t="s">
-        <v>1165</v>
-      </c>
-      <c r="D170" s="9" t="s">
-        <v>1165</v>
-      </c>
+      <c r="A170" s="9"/>
+      <c r="B170" s="9"/>
+      <c r="C170" s="62"/>
+      <c r="D170" s="9"/>
     </row>
     <row r="171" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A171" s="91" t="s">
-        <v>1166</v>
-      </c>
-      <c r="B171" s="9" t="s">
-        <v>1167</v>
-      </c>
-      <c r="C171" s="9" t="s">
-        <v>1167</v>
-      </c>
-      <c r="D171" s="9" t="s">
-        <v>1167</v>
+      <c r="A171" s="1" t="s">
+        <v>552</v>
+      </c>
+      <c r="B171" s="12" t="s">
+        <v>1101</v>
+      </c>
+      <c r="C171" s="63" t="s">
+        <v>1127</v>
+      </c>
+      <c r="D171" s="12" t="s">
+        <v>553</v>
       </c>
     </row>
     <row r="172" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A172" s="9" t="s">
-        <v>1170</v>
+      <c r="A172" s="1" t="s">
+        <v>554</v>
       </c>
       <c r="B172" s="9" t="s">
-        <v>1168</v>
-      </c>
-      <c r="C172" s="9" t="s">
-        <v>1169</v>
+        <v>555</v>
+      </c>
+      <c r="C172" s="62" t="s">
+        <v>23</v>
       </c>
       <c r="D172" s="9" t="s">
-        <v>1168</v>
+        <v>555</v>
       </c>
     </row>
     <row r="173" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B173" s="9"/>
-      <c r="C173" s="9"/>
+      <c r="A173" s="1" t="s">
+        <v>556</v>
+      </c>
+      <c r="B173" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C173" s="62" t="s">
+        <v>16</v>
+      </c>
+      <c r="D173" s="9" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="174" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A174" s="29"/>
-      <c r="B174" s="35" t="s">
-        <v>1226</v>
-      </c>
-      <c r="C174" s="66"/>
+      <c r="A174" s="9"/>
+      <c r="B174" s="9"/>
+      <c r="C174" s="62"/>
     </row>
     <row r="175" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A175" s="9" t="s">
-        <v>1225</v>
+        <v>1059</v>
       </c>
       <c r="B175" s="9" t="s">
-        <v>1284</v>
+        <v>1087</v>
       </c>
       <c r="C175" s="62" t="s">
-        <v>1228</v>
+        <v>1144</v>
       </c>
       <c r="D175" s="9" t="s">
-        <v>1227</v>
+        <v>1087</v>
       </c>
     </row>
     <row r="176" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A176" s="9" t="s">
-        <v>1229</v>
+        <v>1159</v>
       </c>
       <c r="B176" s="9" t="s">
-        <v>1284</v>
-      </c>
-      <c r="C176" s="9"/>
-    </row>
-    <row r="177" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A177" s="91" t="s">
-        <v>1230</v>
+        <v>1160</v>
+      </c>
+      <c r="C176" s="62" t="s">
+        <v>1161</v>
+      </c>
+      <c r="D176" s="9" t="s">
+        <v>1160</v>
+      </c>
+    </row>
+    <row r="177" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A177" s="9" t="s">
+        <v>1162</v>
       </c>
       <c r="B177" s="9" t="s">
-        <v>1283</v>
-      </c>
-      <c r="C177" s="9"/>
-    </row>
-    <row r="178" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A178" s="9" t="s">
-        <v>1285</v>
+        <v>1163</v>
+      </c>
+      <c r="C177" s="9" t="s">
+        <v>1163</v>
+      </c>
+      <c r="D177" s="9" t="s">
+        <v>1163</v>
+      </c>
+    </row>
+    <row r="178" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A178" s="91" t="s">
+        <v>1164</v>
       </c>
       <c r="B178" s="9" t="s">
-        <v>1286</v>
-      </c>
-      <c r="C178" s="9"/>
-    </row>
-    <row r="179" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A179" s="9"/>
-      <c r="B179" s="9"/>
-      <c r="C179" s="9"/>
-    </row>
-    <row r="180" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A180" s="9"/>
+        <v>1165</v>
+      </c>
+      <c r="C178" s="9" t="s">
+        <v>1165</v>
+      </c>
+      <c r="D178" s="9" t="s">
+        <v>1165</v>
+      </c>
+    </row>
+    <row r="179" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A179" s="9" t="s">
+        <v>1168</v>
+      </c>
+      <c r="B179" s="9" t="s">
+        <v>1166</v>
+      </c>
+      <c r="C179" s="9" t="s">
+        <v>1167</v>
+      </c>
+      <c r="D179" s="9" t="s">
+        <v>1166</v>
+      </c>
+    </row>
+    <row r="180" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="B180" s="9"/>
       <c r="C180" s="9"/>
     </row>
-    <row r="181" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A181" s="9"/>
-      <c r="B181" s="9"/>
-      <c r="C181" s="9"/>
-    </row>
-    <row r="182" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A182" s="9"/>
-      <c r="B182" s="9"/>
-      <c r="C182" s="9"/>
-    </row>
-    <row r="183" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A183" s="9"/>
-      <c r="B183" s="9"/>
-      <c r="C183" s="9"/>
-    </row>
-    <row r="184" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A184" s="9"/>
-      <c r="B184" s="9"/>
+    <row r="181" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A181" s="29"/>
+      <c r="B181" s="35" t="s">
+        <v>1223</v>
+      </c>
+      <c r="C181" s="66"/>
+    </row>
+    <row r="182" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A182" s="9" t="s">
+        <v>1222</v>
+      </c>
+      <c r="B182" s="9" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C182" s="62" t="s">
+        <v>1225</v>
+      </c>
+      <c r="D182" s="9" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="183" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A183" s="9" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B183" s="9" t="s">
+        <v>1281</v>
+      </c>
+      <c r="C183" s="62" t="s">
+        <v>1225</v>
+      </c>
+    </row>
+    <row r="184" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A184" s="91" t="s">
+        <v>1227</v>
+      </c>
+      <c r="B184" s="9" t="s">
+        <v>1280</v>
+      </c>
       <c r="C184" s="9"/>
     </row>
-    <row r="185" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A185" s="9"/>
-      <c r="B185" s="9"/>
+    <row r="185" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A185" s="9" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B185" s="9" t="s">
+        <v>1283</v>
+      </c>
       <c r="C185" s="9"/>
     </row>
-    <row r="186" spans="1:3" ht="15.75" customHeight="1">
+    <row r="186" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A186" s="9"/>
       <c r="B186" s="9"/>
       <c r="C186" s="9"/>
     </row>
-    <row r="187" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A187" s="9"/>
-      <c r="B187" s="9"/>
-      <c r="C187" s="9"/>
-    </row>
-    <row r="188" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A188" s="9"/>
-      <c r="B188" s="9"/>
-      <c r="C188" s="9"/>
-    </row>
-    <row r="189" spans="1:3" ht="15.75" customHeight="1">
+    <row r="187" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A187" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B187" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C187" s="97" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="188" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A188" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B188" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C188" s="76" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="189" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A189" s="9"/>
       <c r="B189" s="9"/>
       <c r="C189" s="9"/>
     </row>
-    <row r="190" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A190" s="9"/>
-      <c r="B190" s="9"/>
-      <c r="C190" s="9"/>
-    </row>
-    <row r="191" spans="1:3" ht="15.75" customHeight="1">
+    <row r="190" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A190" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B190" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C190" s="76" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A191" s="9"/>
       <c r="B191" s="9"/>
       <c r="C191" s="9"/>
     </row>
-    <row r="192" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A192" s="9"/>
-      <c r="B192" s="9"/>
-      <c r="C192" s="9"/>
-    </row>
-    <row r="193" spans="1:3" ht="15.75" customHeight="1">
+    <row r="192" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A192" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B192" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C192" s="76" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="193" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A193" s="9"/>
       <c r="B193" s="9"/>
       <c r="C193" s="9"/>
     </row>
-    <row r="194" spans="1:3" ht="15.75" customHeight="1">
-      <c r="A194" s="9"/>
-      <c r="B194" s="9"/>
-      <c r="C194" s="9"/>
-    </row>
-    <row r="195" spans="1:3" ht="15.75" customHeight="1">
+    <row r="194" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A194" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B194" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C194" s="76" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="195" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A195" s="9"/>
       <c r="B195" s="9"/>
       <c r="C195" s="9"/>
     </row>
-    <row r="196" spans="1:3" ht="15.75" customHeight="1">
+    <row r="196" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A196" s="9"/>
       <c r="B196" s="9"/>
       <c r="C196" s="9"/>
     </row>
-    <row r="197" spans="1:3" ht="15.75" customHeight="1">
+    <row r="197" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A197" s="9"/>
       <c r="B197" s="9"/>
       <c r="C197" s="9"/>
@@ -36400,13 +36532,14 @@
     <row r="1001" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B3" r:id="rId1" xr:uid="{00000000-0004-0000-0300-000002000000}"/>
-    <hyperlink ref="D3" r:id="rId2" xr:uid="{3EFD36B0-2228-45CC-AC19-2290C035AA1A}"/>
-    <hyperlink ref="C145" r:id="rId3" xr:uid="{D585080A-FC84-4C4E-BBDD-A485B5C6854A}"/>
-    <hyperlink ref="C2" r:id="rId4" xr:uid="{A4DEE308-051E-4F9C-9C85-8307AF9E1ACB}"/>
-    <hyperlink ref="B2" r:id="rId5" xr:uid="{6B02F5FD-321A-4EC6-B083-48F8A4F10673}"/>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{51CF91D8-7A2D-4C64-827B-6C41EEA7AE41}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{40CD9620-87B1-4D27-9D9D-9B54D2D36C19}"/>
+    <hyperlink ref="C152" r:id="rId3" xr:uid="{25FAC99D-B272-4C71-9B4D-364D57432552}"/>
+    <hyperlink ref="B2" r:id="rId4" xr:uid="{A5D45DE0-52B9-458D-A530-797F4FB8B49C}"/>
+    <hyperlink ref="C2" r:id="rId5" xr:uid="{10A69855-CD62-4F1A-BCBC-DBB64A29B7CA}"/>
+    <hyperlink ref="C187" r:id="rId6" xr:uid="{15BB9E58-3CD9-4309-9710-BEFD670B22CD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup orientation="landscape" r:id="rId6"/>
+  <pageSetup orientation="landscape" r:id="rId7"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Patient Happy Path  Updated code 09/06/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FB49A04-3DCF-441B-BC98-4A0B83DE31C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E3AEF5-69EA-4ACF-97C2-1C6DB9EA01FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2670" uniqueCount="1316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2670" uniqueCount="1322">
   <si>
     <t>KEY</t>
   </si>
@@ -3456,9 +3456,6 @@
     <t>VM07 HC Evo Prod;VM07 Loc1 Evo Prod;Patient Communication;Patient;peter;Received Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg</t>
   </si>
   <si>
-    <t>VM07 HC Evo Prod;Internal Communication;Patient;peter;Manual Test for Message;Body : Manual Test for Message;MMHtest.jpg</t>
-  </si>
-  <si>
     <t>VM07 HC Evo Prod;Any provider;No Preference;All Patients (Registered and Activated) to Patient Portal;Group MessageTesting_RANDOM;Group Message Test_RANDOM</t>
   </si>
   <si>
@@ -4003,6 +4000,27 @@
   </si>
   <si>
     <t>2 time per day</t>
+  </si>
+  <si>
+    <t>VM07 HC Evo Prod;Patient Communication;Patient;peter;Manual Test for Message;Body : Manual Test for Message;MMHtest.jpg</t>
+  </si>
+  <si>
+    <t>VM07 Loc1 Evo Prod ; Dr B Beta ; Patient to Collect Script ; Next Day;Praluent Prefilled Pen 150mg/1mL Soln for injection;Repeat Medication Testing for PATIENT TO COLLECT</t>
+  </si>
+  <si>
+    <t>VM07 Loc1 Evo Prod;praluent prefilled pen 150mg/1ml soln for injection(alirocumab);pending;Next Day - Fee: NZ$;Dr B Beta</t>
+  </si>
+  <si>
+    <t>Dr B Beta ( VM07 Loc1 Evo Prod );VM07 Loc1 Evo Prod;Patient to Collect Script;Next Day - Fee: NZ$;praluent prefilled pen 150mg/1ml soln for injection(alirocumab);Pending</t>
+  </si>
+  <si>
+    <t>VM07 Loc1 Evo Prod;GP1 Vm07 Loc1;Send Script by Post;Next Day;Panadol (Optizorb) 500mg Caplets;Repeat Medication Testing for PATIENT TO COLLECT</t>
+  </si>
+  <si>
+    <t>https://app.managemyhealth.co.nz/home</t>
+  </si>
+  <si>
+    <t>Pacifen 10mg Tab;1 tabs, Twice Daily, 1 week;14;GP2WHITE;Automation1_Loc1</t>
   </si>
 </sst>
 </file>
@@ -4945,7 +4963,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C1" s="73" t="s">
         <v>1</v>
@@ -4978,10 +4996,10 @@
         <v>2</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C2" s="74" t="s">
-        <v>1048</v>
+        <v>1320</v>
       </c>
       <c r="D2" s="57" t="s">
         <v>1123</v>
@@ -5041,10 +5059,10 @@
     </row>
     <row r="4" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A4" s="1" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="B4" s="57" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="C4" s="75"/>
       <c r="D4" s="4"/>
@@ -5070,10 +5088,10 @@
     </row>
     <row r="5" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A5" s="1" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="B5" s="57" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="C5" s="75"/>
       <c r="D5" s="4"/>
@@ -6215,7 +6233,7 @@
     </row>
     <row r="43" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="B43" s="8" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="C43"/>
       <c r="E43" s="2"/>
@@ -6240,10 +6258,10 @@
     </row>
     <row r="44" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A44" s="1" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="C44" s="76" t="s">
         <v>1126</v>
@@ -6273,10 +6291,10 @@
     </row>
     <row r="45" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A45" s="1" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="C45" s="76" t="s">
         <v>13</v>
@@ -6306,10 +6324,10 @@
     </row>
     <row r="46" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A46" s="1" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="C46" s="76" t="s">
         <v>16</v>
@@ -6372,10 +6390,10 @@
     </row>
     <row r="48" spans="1:23" ht="13.5" customHeight="1">
       <c r="A48" t="s">
+        <v>1269</v>
+      </c>
+      <c r="B48" t="s">
         <v>1270</v>
-      </c>
-      <c r="B48" t="s">
-        <v>1271</v>
       </c>
       <c r="C48"/>
       <c r="E48" s="2"/>
@@ -6444,10 +6462,10 @@
     </row>
     <row r="51" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A51" s="1" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="C51" s="76" t="s">
         <v>1126</v>
@@ -6474,10 +6492,10 @@
     </row>
     <row r="52" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A52" s="1" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="C52" s="76" t="s">
         <v>13</v>
@@ -6504,10 +6522,10 @@
     </row>
     <row r="53" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A53" s="1" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="C53" s="76" t="s">
         <v>16</v>
@@ -6564,10 +6582,10 @@
     </row>
     <row r="55" spans="1:23" ht="13.5" customHeight="1">
       <c r="A55" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="B55" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="C55"/>
       <c r="E55" s="2"/>
@@ -6674,7 +6692,7 @@
         <v>56</v>
       </c>
       <c r="C59" s="76" t="s">
-        <v>57</v>
+        <v>1316</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>56</v>
@@ -6707,7 +6725,7 @@
         <v>59</v>
       </c>
       <c r="C60" s="76" t="s">
-        <v>966</v>
+        <v>1317</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>59</v>
@@ -6740,7 +6758,7 @@
         <v>61</v>
       </c>
       <c r="C61" s="76" t="s">
-        <v>62</v>
+        <v>1318</v>
       </c>
       <c r="D61" s="1" t="s">
         <v>61</v>
@@ -6831,7 +6849,7 @@
         <v>67</v>
       </c>
       <c r="C64" s="76" t="s">
-        <v>68</v>
+        <v>1319</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>67</v>
@@ -7717,7 +7735,7 @@
         <v>104</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>1028</v>
+        <v>1321</v>
       </c>
       <c r="C93" s="76" t="s">
         <v>1049</v>
@@ -7753,7 +7771,7 @@
         <v>106</v>
       </c>
       <c r="C94" s="76" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="D94" s="1" t="s">
         <v>106</v>
@@ -8093,7 +8111,7 @@
         <v>112</v>
       </c>
       <c r="C105" s="76" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="D105" s="1" t="s">
         <v>112</v>
@@ -9363,10 +9381,10 @@
         <v>188</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="C146" s="76" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="D146" s="1" t="s">
         <v>1124</v>
@@ -9396,7 +9414,7 @@
         <v>189</v>
       </c>
       <c r="B147" s="10" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="C147" s="85" t="s">
         <v>976</v>
@@ -9429,7 +9447,7 @@
         <v>190</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="C148" s="76" t="s">
         <v>192</v>
@@ -9487,7 +9505,7 @@
         <v>193</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="C150" s="76" t="s">
         <v>1066</v>
@@ -10320,7 +10338,7 @@
         <v>1078</v>
       </c>
       <c r="C176" s="76" t="s">
-        <v>1133</v>
+        <v>1315</v>
       </c>
       <c r="D176" s="1" t="s">
         <v>1078</v>
@@ -10353,7 +10371,7 @@
         <v>1079</v>
       </c>
       <c r="C177" s="76" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="D177" s="1" t="s">
         <v>1079</v>
@@ -10419,7 +10437,7 @@
         <v>1080</v>
       </c>
       <c r="C179" s="76" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="D179" s="1" t="s">
         <v>1080</v>
@@ -10705,10 +10723,10 @@
     </row>
     <row r="189" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A189" s="1" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C189" s="55"/>
       <c r="D189" s="2"/>
@@ -10734,10 +10752,10 @@
     </row>
     <row r="190" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A190" s="1" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="C190" s="55"/>
       <c r="D190" s="2"/>
@@ -10787,10 +10805,10 @@
     </row>
     <row r="192" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A192" s="1" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C192"/>
       <c r="D192" s="2"/>
@@ -10816,10 +10834,10 @@
     </row>
     <row r="193" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A193" s="1" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="C193" s="55"/>
       <c r="D193" s="2"/>
@@ -10869,10 +10887,10 @@
     </row>
     <row r="195" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A195" s="1" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="C195" s="76" t="s">
         <v>1126</v>
@@ -10900,7 +10918,7 @@
     </row>
     <row r="196" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A196" s="1" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>12</v>
@@ -11017,10 +11035,10 @@
     </row>
     <row r="200" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A200" s="1" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="C200" s="76" t="s">
         <v>1126</v>
@@ -11048,7 +11066,7 @@
     </row>
     <row r="201" spans="1:23" ht="13.5" customHeight="1" thickBot="1">
       <c r="A201" s="1" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="B201" s="1" t="s">
         <v>12</v>
@@ -16811,7 +16829,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C1" s="7" t="s">
         <v>1</v>
@@ -16842,7 +16860,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="51" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C2" s="51" t="s">
         <v>1048</v>
@@ -16892,7 +16910,7 @@
         <v>218</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="C12" s="76" t="s">
         <v>1131</v>
@@ -16903,10 +16921,10 @@
         <v>557</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -16917,7 +16935,7 @@
         <v>559</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
     </row>
     <row r="15" spans="1:23" ht="30">
@@ -16925,10 +16943,10 @@
         <v>375</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -16961,7 +16979,7 @@
         <v>1079</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="19" spans="1:3">
@@ -17315,7 +17333,7 @@
         <v>571</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="C67" s="9" t="s">
         <v>573</v>
@@ -17327,7 +17345,7 @@
         <v>574</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="C69" s="9" t="s">
         <v>576</v>
@@ -17338,7 +17356,7 @@
         <v>577</v>
       </c>
       <c r="B70" s="9" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="C70" s="9" t="s">
         <v>578</v>
@@ -17349,7 +17367,7 @@
         <v>579</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="C71" s="9" t="s">
         <v>581</v>
@@ -17396,7 +17414,7 @@
         <v>589</v>
       </c>
       <c r="B78" s="9" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="C78" s="9" t="s">
         <v>591</v>
@@ -17429,7 +17447,7 @@
         <v>382</v>
       </c>
       <c r="C84" s="9" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="85" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17438,10 +17456,10 @@
         <v>596</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="C86" s="9" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
     </row>
     <row r="87" spans="1:3" ht="15.75" customHeight="1">
@@ -17590,10 +17608,10 @@
         <v>626</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="C110" s="9" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
     </row>
     <row r="111" spans="1:3" ht="15.75" customHeight="1">
@@ -17601,10 +17619,10 @@
         <v>627</v>
       </c>
       <c r="B111" s="9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="C111" s="9" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
     </row>
     <row r="112" spans="1:3" ht="15.75" customHeight="1">
@@ -17612,10 +17630,10 @@
         <v>628</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="C112" s="9" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
     </row>
     <row r="113" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17624,10 +17642,10 @@
         <v>629</v>
       </c>
       <c r="B114" s="9" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="C114" s="9" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
     </row>
     <row r="115" spans="1:3" ht="15.75" customHeight="1">
@@ -17635,10 +17653,10 @@
         <v>630</v>
       </c>
       <c r="B115" s="9" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="C115" s="9" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
     </row>
     <row r="116" spans="1:3" ht="15.75" customHeight="1">
@@ -17646,10 +17664,10 @@
         <v>631</v>
       </c>
       <c r="B116" s="9" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C116" s="9" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
     </row>
     <row r="117" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17695,7 +17713,7 @@
         <v>641</v>
       </c>
       <c r="C122" s="9" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
     </row>
     <row r="123" spans="1:3" ht="15.75" customHeight="1"/>
@@ -17707,7 +17725,7 @@
         <v>643</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="125" spans="1:3" ht="15.75" customHeight="1">
@@ -17718,7 +17736,7 @@
         <v>645</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="126" spans="1:3" ht="15.75" customHeight="1">
@@ -17729,7 +17747,7 @@
         <v>645</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
     </row>
     <row r="127" spans="1:3" ht="15.75" customHeight="1"/>
@@ -18637,7 +18655,7 @@
         <v>188</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="C229" s="76" t="s">
         <v>1065</v>
@@ -18648,7 +18666,7 @@
         <v>189</v>
       </c>
       <c r="B230" s="10" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="C230" s="85" t="s">
         <v>976</v>
@@ -18659,7 +18677,7 @@
         <v>190</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="C231" s="76" t="s">
         <v>192</v>
@@ -18671,7 +18689,7 @@
         <v>193</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="C233" s="76" t="s">
         <v>1066</v>
@@ -21386,7 +21404,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="9" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C1" s="18" t="s">
         <v>1</v>
@@ -22020,7 +22038,7 @@
         <v>39</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="C24" s="18"/>
       <c r="D24" s="18"/>
@@ -22836,7 +22854,7 @@
         <v>281</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="C54" s="18"/>
       <c r="D54" s="18"/>
@@ -22864,7 +22882,7 @@
         <v>282</v>
       </c>
       <c r="B55" s="9" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="C55" s="18"/>
       <c r="D55" s="18"/>
@@ -22892,7 +22910,7 @@
         <v>283</v>
       </c>
       <c r="B56" s="9" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="C56" s="18"/>
       <c r="D56" s="18"/>
@@ -22920,7 +22938,7 @@
         <v>284</v>
       </c>
       <c r="B57" s="9" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="C57" s="18"/>
       <c r="D57" s="18"/>
@@ -22948,7 +22966,7 @@
         <v>285</v>
       </c>
       <c r="B58" s="9" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="C58" s="18"/>
       <c r="D58" s="18"/>
@@ -22976,7 +22994,7 @@
         <v>286</v>
       </c>
       <c r="B59" s="9" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="C59" s="18"/>
       <c r="D59" s="18"/>
@@ -23004,7 +23022,7 @@
         <v>287</v>
       </c>
       <c r="B60" s="9" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="C60" s="18"/>
       <c r="D60" s="18"/>
@@ -23032,7 +23050,7 @@
         <v>288</v>
       </c>
       <c r="B61" s="9" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="C61" s="18"/>
       <c r="D61" s="18"/>
@@ -23060,7 +23078,7 @@
         <v>289</v>
       </c>
       <c r="B62" s="9" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="C62" s="18"/>
       <c r="D62" s="18"/>
@@ -23088,7 +23106,7 @@
         <v>290</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="C63" s="18"/>
       <c r="D63" s="18"/>
@@ -23116,7 +23134,7 @@
         <v>291</v>
       </c>
       <c r="B64" s="9" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="C64" s="18"/>
       <c r="D64" s="18"/>
@@ -23144,7 +23162,7 @@
         <v>292</v>
       </c>
       <c r="B65" s="9" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="C65" s="18"/>
       <c r="D65" s="18"/>
@@ -23172,7 +23190,7 @@
         <v>293</v>
       </c>
       <c r="B66" s="9" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="C66" s="18"/>
       <c r="D66" s="18"/>
@@ -23200,7 +23218,7 @@
         <v>294</v>
       </c>
       <c r="B67" s="9" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="C67" s="18"/>
       <c r="D67" s="18"/>
@@ -23252,7 +23270,7 @@
         <v>295</v>
       </c>
       <c r="B69" s="9" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C69" s="18"/>
       <c r="D69" s="18"/>
@@ -23308,7 +23326,7 @@
         <v>298</v>
       </c>
       <c r="B71" s="9" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="C71" s="18"/>
       <c r="D71" s="18"/>
@@ -23360,7 +23378,7 @@
         <v>299</v>
       </c>
       <c r="B73" s="9" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="C73" s="18"/>
       <c r="D73" s="18"/>
@@ -23388,7 +23406,7 @@
         <v>300</v>
       </c>
       <c r="B74" s="9" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="C74" s="18"/>
       <c r="D74" s="18"/>
@@ -23872,7 +23890,7 @@
         <v>319</v>
       </c>
       <c r="B92" s="22" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="C92" s="18"/>
       <c r="D92" s="18"/>
@@ -23900,7 +23918,7 @@
         <v>320</v>
       </c>
       <c r="B93" s="22" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C93" s="18"/>
       <c r="D93" s="18"/>
@@ -24008,7 +24026,7 @@
         <v>323</v>
       </c>
       <c r="B97" s="9" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="C97" s="18"/>
       <c r="D97" s="18"/>
@@ -24036,7 +24054,7 @@
         <v>324</v>
       </c>
       <c r="B98" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="C98" s="18"/>
       <c r="D98" s="18"/>
@@ -24064,7 +24082,7 @@
         <v>325</v>
       </c>
       <c r="B99" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="C99" s="18"/>
       <c r="D99" s="18"/>
@@ -24116,7 +24134,7 @@
         <v>326</v>
       </c>
       <c r="B101" s="9" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="C101" s="18"/>
       <c r="D101" s="18"/>
@@ -24172,7 +24190,7 @@
         <v>327</v>
       </c>
       <c r="B103" s="22" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="C103" s="18"/>
       <c r="D103" s="18"/>
@@ -24252,7 +24270,7 @@
         <v>330</v>
       </c>
       <c r="B106" s="9" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="C106" s="18"/>
       <c r="D106" s="18"/>
@@ -24280,7 +24298,7 @@
         <v>331</v>
       </c>
       <c r="B107" s="9" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="C107" s="18"/>
       <c r="D107" s="18"/>
@@ -24432,7 +24450,7 @@
         <v>333</v>
       </c>
       <c r="B113" s="9" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="C113" s="18"/>
       <c r="D113" s="18"/>
@@ -24484,7 +24502,7 @@
         <v>334</v>
       </c>
       <c r="B115" s="24" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="C115" s="18"/>
       <c r="D115" s="18"/>
@@ -24536,7 +24554,7 @@
         <v>335</v>
       </c>
       <c r="B117" s="92" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C117" s="18"/>
       <c r="D117" s="18"/>
@@ -24844,7 +24862,7 @@
         <v>340</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="C129" s="18"/>
       <c r="D129" s="18"/>
@@ -24900,7 +24918,7 @@
         <v>341</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="C131" s="18"/>
       <c r="D131" s="18"/>
@@ -25652,7 +25670,7 @@
         <v>370</v>
       </c>
       <c r="B159" s="94" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="C159" s="18"/>
       <c r="D159" s="18"/>
@@ -26028,7 +26046,7 @@
         <v>441</v>
       </c>
       <c r="B173" s="9" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="C173" s="18"/>
       <c r="D173" s="18"/>
@@ -26077,10 +26095,10 @@
     </row>
     <row r="175" spans="1:22" ht="15.75" customHeight="1">
       <c r="A175" s="91" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="B175" s="94" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C175" s="18"/>
       <c r="D175" s="18"/>
@@ -26105,10 +26123,10 @@
     </row>
     <row r="176" spans="1:22" ht="15.75" customHeight="1">
       <c r="A176" s="91" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="B176" s="94" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="C176" s="18"/>
       <c r="D176" s="18"/>
@@ -26133,10 +26151,10 @@
     </row>
     <row r="177" spans="1:22" ht="15.75" customHeight="1">
       <c r="A177" s="91" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="B177" s="94" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C177" s="18"/>
       <c r="D177" s="18"/>
@@ -26161,10 +26179,10 @@
     </row>
     <row r="178" spans="1:22" ht="15.75" customHeight="1">
       <c r="A178" s="91" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="B178" s="94" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="C178" s="18"/>
       <c r="D178" s="18"/>
@@ -26189,10 +26207,10 @@
     </row>
     <row r="179" spans="1:22" ht="15.75" customHeight="1">
       <c r="A179" s="91" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="B179" s="94" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="C179" s="18"/>
       <c r="D179" s="18"/>
@@ -26247,7 +26265,7 @@
         <v>1087</v>
       </c>
       <c r="C181" s="62" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="D181" s="18"/>
       <c r="E181" s="18"/>
@@ -26301,10 +26319,10 @@
     </row>
     <row r="183" spans="1:22" ht="15.75" customHeight="1" thickBot="1">
       <c r="A183" s="91" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="B183" s="94" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C183" s="18"/>
       <c r="D183" s="18"/>
@@ -26359,10 +26377,10 @@
     </row>
     <row r="185" spans="1:22" ht="15.75" customHeight="1">
       <c r="A185" s="91" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="B185" s="94" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="C185" s="18"/>
       <c r="D185" s="18"/>
@@ -26411,10 +26429,10 @@
     </row>
     <row r="187" spans="1:22" ht="15.75" customHeight="1">
       <c r="A187" s="91" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="B187" s="94" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="C187" s="18"/>
       <c r="D187" s="18"/>
@@ -30929,7 +30947,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C1" s="26" t="s">
         <v>1</v>
@@ -32791,7 +32809,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="26" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="C1" s="65" t="s">
         <v>1</v>
@@ -32805,7 +32823,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="96" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C2" s="72" t="s">
         <v>1048</v>
@@ -32880,7 +32898,7 @@
         <v>1082</v>
       </c>
       <c r="C8" s="62" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="D8" s="9" t="s">
         <v>417</v>
@@ -32894,7 +32912,7 @@
         <v>1083</v>
       </c>
       <c r="C9" s="62" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="D9" s="9" t="s">
         <v>420</v>
@@ -32908,7 +32926,7 @@
         <v>1118</v>
       </c>
       <c r="C10" s="62" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>423</v>
@@ -32922,7 +32940,7 @@
         <v>1119</v>
       </c>
       <c r="C11" s="62" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="D11" s="9" t="s">
         <v>426</v>
@@ -32936,7 +32954,7 @@
         <v>1120</v>
       </c>
       <c r="C12" s="62" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D12" s="9" t="s">
         <v>429</v>
@@ -32950,7 +32968,7 @@
         <v>1121</v>
       </c>
       <c r="C13" s="62" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>432</v>
@@ -32964,7 +32982,7 @@
         <v>1122</v>
       </c>
       <c r="C14" s="62" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="D14" s="9" t="s">
         <v>435</v>
@@ -33000,13 +33018,13 @@
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1">
       <c r="A17" s="91" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="B17" s="9" t="s">
         <v>442</v>
       </c>
       <c r="C17" s="62" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="D17" s="9"/>
     </row>
@@ -33015,10 +33033,10 @@
         <v>441</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="C18" s="62" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>442</v>
@@ -33029,7 +33047,7 @@
         <v>444</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="C19" s="62" t="s">
         <v>976</v>
@@ -33292,7 +33310,7 @@
         <v>67</v>
       </c>
       <c r="C43" s="60" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="D43" s="1" t="s">
         <v>67</v>
@@ -33326,7 +33344,7 @@
         <v>1070</v>
       </c>
       <c r="C46" s="60" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="D46" s="1" t="s">
         <v>1070</v>
@@ -33337,13 +33355,13 @@
         <v>89</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="C47" s="60" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
     </row>
     <row r="48" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -33374,7 +33392,7 @@
         <v>482</v>
       </c>
       <c r="C50" s="60" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="D50" s="1" t="s">
         <v>482</v>
@@ -33434,7 +33452,7 @@
         <v>485</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="C54" s="59" t="s">
         <v>1130</v>
@@ -33459,13 +33477,13 @@
     </row>
     <row r="56" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
       <c r="A56" s="91" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B56" s="15" t="s">
         <v>1303</v>
       </c>
-      <c r="B56" s="15" t="s">
+      <c r="C56" s="64" t="s">
         <v>1304</v>
-      </c>
-      <c r="C56" s="64" t="s">
-        <v>1305</v>
       </c>
       <c r="D56" s="1"/>
     </row>
@@ -33477,7 +33495,7 @@
         <v>1079</v>
       </c>
       <c r="C57" s="60" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>232</v>
@@ -33681,7 +33699,7 @@
         <v>1085</v>
       </c>
       <c r="C75" s="62" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="D75" s="9" t="s">
         <v>495</v>
@@ -33771,7 +33789,7 @@
         <v>1087</v>
       </c>
       <c r="C83" s="62" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="D83" s="9" t="s">
         <v>382</v>
@@ -33939,7 +33957,7 @@
         <v>1088</v>
       </c>
       <c r="C97" s="62" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="D97" s="9" t="s">
         <v>508</v>
@@ -34017,7 +34035,7 @@
         <v>1089</v>
       </c>
       <c r="C104" s="63" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D104" s="9" t="s">
         <v>392</v>
@@ -34028,10 +34046,10 @@
         <v>393</v>
       </c>
       <c r="B105" s="9" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="C105" s="62" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="D105" s="9" t="s">
         <v>394</v>
@@ -34073,19 +34091,19 @@
     </row>
     <row r="109" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A109" s="9" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="B109" s="9" t="s">
         <v>32</v>
       </c>
       <c r="C109" s="62" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="D109" s="9"/>
     </row>
     <row r="110" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A110" s="91" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
       <c r="B110" s="9" t="s">
         <v>15</v>
@@ -34097,7 +34115,7 @@
     </row>
     <row r="111" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A111" s="9" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
       <c r="B111" s="9" t="s">
         <v>45</v>
@@ -34109,7 +34127,7 @@
     </row>
     <row r="112" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A112" s="9" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="B112" s="9" t="s">
         <v>48</v>
@@ -34187,7 +34205,7 @@
         <v>1090</v>
       </c>
       <c r="C119" s="63" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D119" s="9" t="s">
         <v>400</v>
@@ -34201,7 +34219,7 @@
         <v>1090</v>
       </c>
       <c r="C120" s="63" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D120" s="9" t="s">
         <v>400</v>
@@ -34221,7 +34239,7 @@
         <v>1091</v>
       </c>
       <c r="C122" s="63" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D122" s="9" t="s">
         <v>516</v>
@@ -34235,7 +34253,7 @@
         <v>1092</v>
       </c>
       <c r="C123" s="63" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D123" s="9" t="s">
         <v>398</v>
@@ -34249,7 +34267,7 @@
         <v>1092</v>
       </c>
       <c r="C124" s="63" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D124" s="9" t="s">
         <v>398</v>
@@ -34269,7 +34287,7 @@
         <v>1093</v>
       </c>
       <c r="C126" s="59" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>519</v>
@@ -34283,7 +34301,7 @@
         <v>1094</v>
       </c>
       <c r="C127" s="59" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D127" s="1" t="s">
         <v>521</v>
@@ -34297,7 +34315,7 @@
         <v>1094</v>
       </c>
       <c r="C128" s="63" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D128" s="9" t="s">
         <v>521</v>
@@ -34317,7 +34335,7 @@
         <v>1090</v>
       </c>
       <c r="C130" s="63" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D130" s="9" t="s">
         <v>400</v>
@@ -34331,7 +34349,7 @@
         <v>1092</v>
       </c>
       <c r="C131" s="63" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="D131" s="9" t="s">
         <v>398</v>
@@ -34345,7 +34363,7 @@
         <v>1095</v>
       </c>
       <c r="C132" s="59" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="D132" s="1" t="s">
         <v>525</v>
@@ -34376,7 +34394,7 @@
         <v>528</v>
       </c>
       <c r="B135" s="9" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="C135" s="62" t="s">
         <v>530</v>
@@ -34390,7 +34408,7 @@
         <v>401</v>
       </c>
       <c r="B136" s="9" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="C136" s="62" t="s">
         <v>530</v>
@@ -34433,7 +34451,7 @@
         <v>1096</v>
       </c>
       <c r="C140" s="62" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="D140" s="9" t="s">
         <v>1023</v>
@@ -34509,7 +34527,7 @@
         <v>1097</v>
       </c>
       <c r="C146" s="62" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="D146" s="9" t="s">
         <v>539</v>
@@ -34523,7 +34541,7 @@
         <v>1098</v>
       </c>
       <c r="C147" s="62" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="D147" s="9" t="s">
         <v>541</v>
@@ -34571,7 +34589,7 @@
         <v>1087</v>
       </c>
       <c r="C151" s="62" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="D151" s="9" t="s">
         <v>382</v>
@@ -34609,7 +34627,7 @@
         <v>1117</v>
       </c>
       <c r="C154" s="62" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="D154" s="9" t="s">
         <v>409</v>
@@ -34693,7 +34711,7 @@
         <v>1085</v>
       </c>
       <c r="C162" s="38" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="D162" s="38" t="s">
         <v>495</v>
@@ -34749,7 +34767,7 @@
         <v>1100</v>
       </c>
       <c r="C167" s="62" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="D167" s="9" t="s">
         <v>1071</v>
@@ -34774,10 +34792,10 @@
         <v>413</v>
       </c>
       <c r="B169" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="C169" s="62" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="D169" s="9" t="s">
         <v>414</v>
@@ -34844,7 +34862,7 @@
         <v>1087</v>
       </c>
       <c r="C175" s="62" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="D175" s="9" t="s">
         <v>1087</v>
@@ -34852,58 +34870,58 @@
     </row>
     <row r="176" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A176" s="9" t="s">
+        <v>1158</v>
+      </c>
+      <c r="B176" s="9" t="s">
         <v>1159</v>
       </c>
-      <c r="B176" s="9" t="s">
+      <c r="C176" s="62" t="s">
         <v>1160</v>
       </c>
-      <c r="C176" s="62" t="s">
-        <v>1161</v>
-      </c>
       <c r="D176" s="9" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="177" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A177" s="9" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B177" s="9" t="s">
         <v>1162</v>
       </c>
-      <c r="B177" s="9" t="s">
-        <v>1163</v>
-      </c>
       <c r="C177" s="9" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="D177" s="9" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="178" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A178" s="91" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B178" s="9" t="s">
         <v>1164</v>
       </c>
-      <c r="B178" s="9" t="s">
-        <v>1165</v>
-      </c>
       <c r="C178" s="9" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="D178" s="9" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="179" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A179" s="9" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B179" s="9" t="s">
+        <v>1165</v>
+      </c>
+      <c r="C179" s="9" t="s">
         <v>1166</v>
       </c>
-      <c r="C179" s="9" t="s">
-        <v>1167</v>
-      </c>
       <c r="D179" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="180" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -34913,50 +34931,50 @@
     <row r="181" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A181" s="29"/>
       <c r="B181" s="35" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="C181" s="66"/>
     </row>
     <row r="182" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A182" s="9" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="B182" s="9" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="C182" s="62" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="D182" s="9" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
     </row>
     <row r="183" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A183" s="9" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="B183" s="9" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="C183" s="62" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
     </row>
     <row r="184" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A184" s="91" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="B184" s="9" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C184" s="9"/>
     </row>
     <row r="185" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A185" s="9" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B185" s="9" t="s">
         <v>1282</v>
-      </c>
-      <c r="B185" s="9" t="s">
-        <v>1283</v>
       </c>
       <c r="C185" s="9"/>
     </row>

</xml_diff>

<commit_message>
Provider Happy Path Updated code 09/06/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D4E3AEF5-69EA-4ACF-97C2-1C6DB9EA01FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3345DA54-5B04-442A-8A75-AD344F7C26C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Happy_Path_Patient_Web_and_MR" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2670" uniqueCount="1322">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2683" uniqueCount="1333">
   <si>
     <t>KEY</t>
   </si>
@@ -4017,10 +4017,43 @@
     <t>VM07 Loc1 Evo Prod;GP1 Vm07 Loc1;Send Script by Post;Next Day;Panadol (Optizorb) 500mg Caplets;Repeat Medication Testing for PATIENT TO COLLECT</t>
   </si>
   <si>
-    <t>https://app.managemyhealth.co.nz/home</t>
-  </si>
-  <si>
     <t>Pacifen 10mg Tab;1 tabs, Twice Daily, 1 week;14;GP2WHITE;Automation1_Loc1</t>
+  </si>
+  <si>
+    <t>https://v2portal.mmhnz.cloud/home</t>
+  </si>
+  <si>
+    <t>VM07 HC Evo Prod;VM07 Loc1 Evo Prod;Patient Communication;Patient;peter;Received Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg;Compose Message_RANDOM;Body : Reply Message Testing_RANDOM;Compose Message</t>
+  </si>
+  <si>
+    <t>NON_CLINICAL_MESSAGE_DETAILS</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Automation1_Loc1;Internal Communication;Patient;Auto;Non Clinical Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg;Compose Message_RANDOM;Body : Reply Message Testing_RANDOM;Compose Message Testing_RANDOM;TestAutomation</t>
+  </si>
+  <si>
+    <t>ALLOW_PATIENT_MESSAGE_DETAILS</t>
+  </si>
+  <si>
+    <t>Automation1_HC1;Automation1_Loc1;Internal Communication;Patient;Auto;Allow Patient Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg;Compose Message_RANDOM;Body : Reply Message Testing_RANDOM;Compose Message Testing_RANDOM;TestAutomation</t>
+  </si>
+  <si>
+    <t>VM07 HC Evo Prod;VM07 Loc1 Evo Prod;Patient Communication;Patient;peter;Allow Patient Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg;Compose Message_RANDOM;Body : Reply Message Testing_RANDOM;Compose Message</t>
+  </si>
+  <si>
+    <t>VM07 HC Evo Prod;VM07 Loc1 Evo Prod;Patient Communication;Patient;peter;Non Clinical Msg Testing_RANDOM;Body : Received Message Testing_RANDOM;MMHtest.jpg;Compose Message_RANDOM;Body : Reply Message Testing_RANDOM;Compose Message</t>
+  </si>
+  <si>
+    <t>NONCLINICAL_MESSAGE_DETAILS</t>
+  </si>
+  <si>
+    <t>ALLOWPATIENT_MESSAGE_DETAILS</t>
+  </si>
+  <si>
+    <t>Allow Patient Msg Testing_RANDOM</t>
+  </si>
+  <si>
+    <t>Non Clinical Msg Testing_RANDOM</t>
   </si>
 </sst>
 </file>
@@ -4264,7 +4297,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -4470,6 +4503,15 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -4477,7 +4519,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -4730,6 +4772,9 @@
     <xf numFmtId="0" fontId="24" fillId="11" borderId="3" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -4999,7 +5044,7 @@
         <v>1257</v>
       </c>
       <c r="C2" s="74" t="s">
-        <v>1320</v>
+        <v>1321</v>
       </c>
       <c r="D2" s="57" t="s">
         <v>1123</v>
@@ -7735,7 +7780,7 @@
         <v>104</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="C93" s="76" t="s">
         <v>1049</v>
@@ -32794,7 +32839,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W1001"/>
+  <dimension ref="A1:W1004"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="48.7109375" customWidth="1" collapsed="1"/>
@@ -33469,7 +33514,7 @@
         <v>1084</v>
       </c>
       <c r="C55" s="64" t="s">
-        <v>1132</v>
+        <v>1322</v>
       </c>
       <c r="D55" s="15" t="s">
         <v>1020</v>
@@ -33720,509 +33765,519 @@
       </c>
     </row>
     <row r="77" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A77" s="9"/>
+      <c r="A77" s="9" t="s">
+        <v>1330</v>
+      </c>
       <c r="B77" s="9" t="s">
-        <v>498</v>
-      </c>
-      <c r="C77" s="62" t="s">
-        <v>498</v>
+        <v>1331</v>
+      </c>
+      <c r="C77" s="9" t="s">
+        <v>1331</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>498</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="78" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A78" s="9" t="s">
+      <c r="A78" s="9"/>
+      <c r="B78" s="9"/>
+      <c r="C78" s="98"/>
+      <c r="D78" s="9"/>
+    </row>
+    <row r="79" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A79" s="9" t="s">
         <v>499</v>
       </c>
-      <c r="B78" s="1" t="s">
+      <c r="B79" s="1" t="s">
         <v>1086</v>
       </c>
-      <c r="C78" s="60" t="s">
+      <c r="C79" s="60" t="s">
         <v>1130</v>
       </c>
-      <c r="D78" s="1" t="s">
+      <c r="D79" s="1" t="s">
         <v>500</v>
       </c>
-    </row>
-    <row r="79" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A79" s="1"/>
-      <c r="B79" s="1"/>
-      <c r="C79" s="62"/>
-      <c r="D79" s="1"/>
     </row>
     <row r="80" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A80" s="9" t="s">
-        <v>501</v>
+        <v>1329</v>
       </c>
       <c r="B80" s="9" t="s">
-        <v>498</v>
-      </c>
-      <c r="C80" s="62" t="s">
-        <v>498</v>
+        <v>1332</v>
+      </c>
+      <c r="C80" s="9" t="s">
+        <v>1332</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>498</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="81" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A81" s="34"/>
-      <c r="B81" s="34" t="s">
-        <v>502</v>
-      </c>
-      <c r="C81" s="68"/>
-      <c r="D81" s="34" t="s">
-        <v>502</v>
+      <c r="A81" s="1" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B81" s="15" t="s">
+        <v>1326</v>
+      </c>
+      <c r="C81" s="64" t="s">
+        <v>1327</v>
+      </c>
+      <c r="D81" s="15" t="s">
+        <v>1326</v>
       </c>
     </row>
     <row r="82" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A82" s="9"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="62"/>
-      <c r="D82" s="9"/>
+      <c r="A82" s="1" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B82" s="15" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C82" s="64" t="s">
+        <v>1328</v>
+      </c>
+      <c r="D82" s="15" t="s">
+        <v>1324</v>
+      </c>
     </row>
     <row r="83" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A83" s="9" t="s">
-        <v>381</v>
+        <v>501</v>
       </c>
       <c r="B83" s="9" t="s">
-        <v>1087</v>
+        <v>498</v>
       </c>
       <c r="C83" s="62" t="s">
-        <v>1143</v>
+        <v>498</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>382</v>
+        <v>498</v>
       </c>
     </row>
     <row r="84" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A84" s="9" t="s">
-        <v>383</v>
-      </c>
-      <c r="B84" s="9" t="s">
-        <v>384</v>
-      </c>
-      <c r="C84" s="62" t="s">
-        <v>503</v>
-      </c>
-      <c r="D84" s="9" t="s">
-        <v>384</v>
+      <c r="A84" s="34"/>
+      <c r="B84" s="34" t="s">
+        <v>502</v>
+      </c>
+      <c r="C84" s="68"/>
+      <c r="D84" s="34" t="s">
+        <v>502</v>
       </c>
     </row>
     <row r="85" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A85" s="9" t="s">
-        <v>385</v>
-      </c>
-      <c r="B85" s="9" t="s">
-        <v>386</v>
-      </c>
-      <c r="C85" s="62" t="s">
-        <v>386</v>
-      </c>
-      <c r="D85" s="9" t="s">
-        <v>386</v>
-      </c>
+      <c r="A85" s="9"/>
+      <c r="B85" s="9"/>
+      <c r="C85" s="62"/>
+      <c r="D85" s="9"/>
     </row>
     <row r="86" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A86" s="9" t="s">
-        <v>411</v>
+        <v>381</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>412</v>
+        <v>1087</v>
       </c>
       <c r="C86" s="62" t="s">
-        <v>1103</v>
+        <v>1143</v>
       </c>
       <c r="D86" s="9" t="s">
-        <v>412</v>
+        <v>382</v>
       </c>
     </row>
     <row r="87" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A87" s="9" t="s">
+        <v>383</v>
+      </c>
+      <c r="B87" s="9" t="s">
+        <v>384</v>
+      </c>
+      <c r="C87" s="62" t="s">
+        <v>503</v>
+      </c>
+      <c r="D87" s="9" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A88" s="9" t="s">
+        <v>385</v>
+      </c>
+      <c r="B88" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="C88" s="62" t="s">
+        <v>386</v>
+      </c>
+      <c r="D88" s="9" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A89" s="9" t="s">
+        <v>411</v>
+      </c>
+      <c r="B89" s="9" t="s">
+        <v>412</v>
+      </c>
+      <c r="C89" s="62" t="s">
+        <v>1103</v>
+      </c>
+      <c r="D89" s="9" t="s">
+        <v>412</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A90" s="9" t="s">
         <v>504</v>
       </c>
-      <c r="B87" s="9" t="s">
+      <c r="B90" s="9" t="s">
         <v>505</v>
       </c>
-      <c r="C87" s="62" t="s">
+      <c r="C90" s="62" t="s">
         <v>1104</v>
       </c>
-      <c r="D87" s="9" t="s">
+      <c r="D90" s="9" t="s">
         <v>505</v>
       </c>
     </row>
-    <row r="88" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A88" s="34"/>
-      <c r="B88" s="34" t="s">
+    <row r="91" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A91" s="34"/>
+      <c r="B91" s="34" t="s">
         <v>506</v>
       </c>
-      <c r="C88" s="68"/>
-      <c r="D88" s="34" t="s">
+      <c r="C91" s="68"/>
+      <c r="D91" s="34" t="s">
         <v>506</v>
       </c>
     </row>
-    <row r="89" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A89" s="9"/>
-      <c r="B89" s="9"/>
-      <c r="C89" s="62"/>
-      <c r="D89" s="9"/>
-    </row>
-    <row r="90" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A90" s="9"/>
-      <c r="B90" s="9"/>
-      <c r="C90" s="62"/>
-      <c r="D90" s="9"/>
-    </row>
-    <row r="91" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A91" s="9"/>
-      <c r="B91" s="9"/>
-      <c r="C91" s="62"/>
-      <c r="D91" s="9"/>
-    </row>
     <row r="92" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A92" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B92" s="9" t="s">
-        <v>1072</v>
-      </c>
-      <c r="C92" s="60" t="s">
-        <v>1126</v>
-      </c>
-      <c r="D92" s="9" t="s">
-        <v>10</v>
-      </c>
+      <c r="A92" s="9"/>
+      <c r="B92" s="9"/>
+      <c r="C92" s="62"/>
+      <c r="D92" s="9"/>
     </row>
     <row r="93" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A93" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B93" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="C93" s="60" t="s">
-        <v>13</v>
-      </c>
-      <c r="D93" s="9" t="s">
-        <v>12</v>
-      </c>
+      <c r="A93" s="9"/>
+      <c r="B93" s="9"/>
+      <c r="C93" s="62"/>
+      <c r="D93" s="9"/>
     </row>
     <row r="94" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A94" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B94" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="C94" s="62" t="s">
-        <v>18</v>
-      </c>
-      <c r="D94" s="9" t="s">
-        <v>18</v>
-      </c>
+      <c r="A94" s="9"/>
+      <c r="B94" s="9"/>
+      <c r="C94" s="62"/>
+      <c r="D94" s="9"/>
     </row>
     <row r="95" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A95" s="9" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B95" s="9" t="s">
-        <v>15</v>
+        <v>1072</v>
       </c>
       <c r="C95" s="60" t="s">
-        <v>16</v>
+        <v>1126</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="96" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A96" s="9" t="s">
-        <v>44</v>
+        <v>11</v>
       </c>
       <c r="B96" s="9" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
       <c r="C96" s="60" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="D96" s="9" t="s">
-        <v>45</v>
+        <v>12</v>
       </c>
     </row>
     <row r="97" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A97" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B97" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C97" s="62" t="s">
+        <v>18</v>
+      </c>
+      <c r="D97" s="9" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="98" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A98" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B98" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C98" s="60" t="s">
+        <v>16</v>
+      </c>
+      <c r="D98" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A99" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B99" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C99" s="60" t="s">
+        <v>46</v>
+      </c>
+      <c r="D99" s="9" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="100" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A100" s="9" t="s">
         <v>507</v>
       </c>
-      <c r="B97" s="9" t="s">
+      <c r="B100" s="9" t="s">
         <v>1088</v>
       </c>
-      <c r="C97" s="62" t="s">
+      <c r="C100" s="62" t="s">
         <v>1144</v>
       </c>
-      <c r="D97" s="9" t="s">
+      <c r="D100" s="9" t="s">
         <v>508</v>
       </c>
     </row>
-    <row r="98" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A98" s="9"/>
-      <c r="B98" s="9"/>
-      <c r="C98" s="62"/>
-      <c r="D98" s="9"/>
-    </row>
-    <row r="99" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A99" s="1" t="s">
+    <row r="101" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A101" s="9"/>
+      <c r="B101" s="9"/>
+      <c r="C101" s="62"/>
+      <c r="D101" s="9"/>
+    </row>
+    <row r="102" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A102" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B99" s="9" t="s">
+      <c r="B102" s="9" t="s">
         <v>1101</v>
       </c>
-      <c r="C99" s="60" t="s">
+      <c r="C102" s="60" t="s">
         <v>1127</v>
       </c>
-      <c r="D99" s="9" t="s">
+      <c r="D102" s="9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="100" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A100" s="1" t="s">
+    <row r="103" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A103" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B100" s="9" t="s">
+      <c r="B103" s="9" t="s">
         <v>555</v>
       </c>
-      <c r="C100" s="60" t="s">
+      <c r="C103" s="60" t="s">
         <v>23</v>
       </c>
-      <c r="D100" s="9" t="s">
+      <c r="D103" s="9" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="101" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A101" s="1" t="s">
+    <row r="104" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A104" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B101" s="9" t="s">
+      <c r="B104" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C101" s="60" t="s">
+      <c r="C104" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="D101" s="9" t="s">
+      <c r="D104" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="102" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A102" s="9"/>
-      <c r="B102" s="9"/>
-      <c r="C102" s="62"/>
-      <c r="D102" s="9"/>
-    </row>
-    <row r="103" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A103" s="29"/>
-      <c r="B103" s="35" t="s">
+    <row r="105" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A105" s="9"/>
+      <c r="B105" s="9"/>
+      <c r="C105" s="62"/>
+      <c r="D105" s="9"/>
+    </row>
+    <row r="106" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A106" s="29"/>
+      <c r="B106" s="35" t="s">
         <v>509</v>
       </c>
-      <c r="C103" s="66"/>
-      <c r="D103" s="35" t="s">
+      <c r="C106" s="66"/>
+      <c r="D106" s="35" t="s">
         <v>509</v>
       </c>
     </row>
-    <row r="104" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A104" s="28" t="s">
+    <row r="107" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A107" s="28" t="s">
         <v>391</v>
       </c>
-      <c r="B104" s="9" t="s">
+      <c r="B107" s="9" t="s">
         <v>1089</v>
       </c>
-      <c r="C104" s="63" t="s">
+      <c r="C107" s="63" t="s">
         <v>1145</v>
       </c>
-      <c r="D104" s="9" t="s">
+      <c r="D107" s="9" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="105" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A105" s="9" t="s">
+    <row r="108" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A108" s="9" t="s">
         <v>393</v>
       </c>
-      <c r="B105" s="9" t="s">
+      <c r="B108" s="9" t="s">
         <v>1312</v>
       </c>
-      <c r="C105" s="62" t="s">
+      <c r="C108" s="62" t="s">
         <v>1305</v>
       </c>
-      <c r="D105" s="9" t="s">
+      <c r="D108" s="9" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="106" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A106" s="9" t="s">
-        <v>395</v>
-      </c>
-      <c r="B106" s="9" t="s">
-        <v>396</v>
-      </c>
-      <c r="C106" s="62" t="s">
-        <v>1105</v>
-      </c>
-      <c r="D106" s="9" t="s">
-        <v>396</v>
-      </c>
-    </row>
-    <row r="107" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A107" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="B107" s="9" t="s">
-        <v>510</v>
-      </c>
-      <c r="C107" s="62" t="s">
-        <v>49</v>
-      </c>
-      <c r="D107" s="9" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="108" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A108" s="9"/>
-      <c r="B108" s="9"/>
-      <c r="C108" s="62"/>
-      <c r="D108" s="9"/>
     </row>
     <row r="109" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A109" s="9" t="s">
-        <v>1306</v>
+        <v>395</v>
       </c>
       <c r="B109" s="9" t="s">
-        <v>32</v>
+        <v>396</v>
       </c>
       <c r="C109" s="62" t="s">
-        <v>1307</v>
-      </c>
-      <c r="D109" s="9"/>
+        <v>1105</v>
+      </c>
+      <c r="D109" s="9" t="s">
+        <v>396</v>
+      </c>
     </row>
     <row r="110" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A110" s="91" t="s">
-        <v>1308</v>
+      <c r="A110" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="B110" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C110" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D110" s="9"/>
+        <v>510</v>
+      </c>
+      <c r="C110" s="62" t="s">
+        <v>49</v>
+      </c>
+      <c r="D110" s="9" t="s">
+        <v>510</v>
+      </c>
     </row>
     <row r="111" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A111" s="9" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B111" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C111" s="9" t="s">
-        <v>46</v>
-      </c>
+      <c r="A111" s="9"/>
+      <c r="B111" s="9"/>
+      <c r="C111" s="62"/>
       <c r="D111" s="9"/>
     </row>
     <row r="112" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A112" s="9" t="s">
-        <v>1310</v>
+        <v>1306</v>
       </c>
       <c r="B112" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="C112" s="9" t="s">
-        <v>49</v>
+        <v>32</v>
+      </c>
+      <c r="C112" s="62" t="s">
+        <v>1307</v>
       </c>
       <c r="D112" s="9"/>
     </row>
     <row r="113" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A113" s="9"/>
-      <c r="B113" s="9"/>
-      <c r="C113" s="62"/>
+      <c r="A113" s="91" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B113" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C113" s="9" t="s">
+        <v>16</v>
+      </c>
       <c r="D113" s="9"/>
     </row>
     <row r="114" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A114" s="9"/>
-      <c r="B114" s="9"/>
-      <c r="C114" s="62"/>
+      <c r="A114" s="9" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B114" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="C114" s="9" t="s">
+        <v>46</v>
+      </c>
       <c r="D114" s="9"/>
     </row>
     <row r="115" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A115" s="9" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B115" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C115" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D115" s="9"/>
+    </row>
+    <row r="116" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A116" s="9"/>
+      <c r="B116" s="9"/>
+      <c r="C116" s="62"/>
+      <c r="D116" s="9"/>
+    </row>
+    <row r="117" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A117" s="9"/>
+      <c r="B117" s="9"/>
+      <c r="C117" s="62"/>
+      <c r="D117" s="9"/>
+    </row>
+    <row r="118" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A118" s="9" t="s">
         <v>402</v>
       </c>
-      <c r="B115" s="9" t="s">
+      <c r="B118" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="C115" s="62" t="s">
+      <c r="C118" s="62" t="s">
         <v>1106</v>
       </c>
-      <c r="D115" s="9" t="s">
+      <c r="D118" s="9" t="s">
         <v>511</v>
       </c>
-    </row>
-    <row r="116" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A116" s="9" t="s">
-        <v>403</v>
-      </c>
-      <c r="B116" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="C116" s="62" t="s">
-        <v>1107</v>
-      </c>
-      <c r="D116" s="9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A117" s="9" t="s">
-        <v>512</v>
-      </c>
-      <c r="B117" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="C117" s="62" t="s">
-        <v>1108</v>
-      </c>
-      <c r="D117" s="9" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="118" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A118" s="9"/>
-      <c r="B118" s="9"/>
-      <c r="C118" s="62"/>
-      <c r="D118" s="9"/>
     </row>
     <row r="119" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A119" s="9" t="s">
-        <v>513</v>
+        <v>403</v>
       </c>
       <c r="B119" s="9" t="s">
-        <v>1090</v>
-      </c>
-      <c r="C119" s="63" t="s">
-        <v>1145</v>
+        <v>25</v>
+      </c>
+      <c r="C119" s="62" t="s">
+        <v>1107</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>400</v>
+        <v>25</v>
       </c>
     </row>
     <row r="120" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A120" s="9" t="s">
-        <v>514</v>
+        <v>512</v>
       </c>
       <c r="B120" s="9" t="s">
-        <v>1090</v>
-      </c>
-      <c r="C120" s="63" t="s">
-        <v>1145</v>
+        <v>53</v>
+      </c>
+      <c r="C120" s="62" t="s">
+        <v>1108</v>
       </c>
       <c r="D120" s="9" t="s">
-        <v>400</v>
+        <v>53</v>
       </c>
     </row>
     <row r="121" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
@@ -34233,777 +34288,784 @@
     </row>
     <row r="122" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A122" s="9" t="s">
-        <v>515</v>
+        <v>513</v>
       </c>
       <c r="B122" s="9" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C122" s="63" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>516</v>
+        <v>400</v>
       </c>
     </row>
     <row r="123" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A123" s="9" t="s">
-        <v>397</v>
+        <v>514</v>
       </c>
       <c r="B123" s="9" t="s">
-        <v>1092</v>
+        <v>1090</v>
       </c>
       <c r="C123" s="63" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D123" s="9" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="124" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A124" s="9"/>
+      <c r="B124" s="9"/>
+      <c r="C124" s="62"/>
+      <c r="D124" s="9"/>
+    </row>
+    <row r="125" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A125" s="9" t="s">
+        <v>515</v>
+      </c>
+      <c r="B125" s="9" t="s">
+        <v>1091</v>
+      </c>
+      <c r="C125" s="63" t="s">
         <v>1146</v>
       </c>
-      <c r="D123" s="9" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="124" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A124" s="9" t="s">
-        <v>517</v>
-      </c>
-      <c r="B124" s="9" t="s">
-        <v>1092</v>
-      </c>
-      <c r="C124" s="63" t="s">
-        <v>1146</v>
-      </c>
-      <c r="D124" s="9" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="125" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A125" s="9"/>
-      <c r="B125" s="9"/>
-      <c r="C125" s="62"/>
-      <c r="D125" s="9"/>
+      <c r="D125" s="9" t="s">
+        <v>516</v>
+      </c>
     </row>
     <row r="126" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A126" s="9" t="s">
-        <v>518</v>
-      </c>
-      <c r="B126" s="1" t="s">
-        <v>1093</v>
-      </c>
-      <c r="C126" s="59" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D126" s="1" t="s">
-        <v>519</v>
+        <v>397</v>
+      </c>
+      <c r="B126" s="9" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C126" s="63" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D126" s="9" t="s">
+        <v>398</v>
       </c>
     </row>
     <row r="127" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A127" s="9" t="s">
-        <v>520</v>
-      </c>
-      <c r="B127" s="1" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C127" s="59" t="s">
+        <v>517</v>
+      </c>
+      <c r="B127" s="9" t="s">
+        <v>1092</v>
+      </c>
+      <c r="C127" s="63" t="s">
+        <v>1146</v>
+      </c>
+      <c r="D127" s="9" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="128" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A128" s="9"/>
+      <c r="B128" s="9"/>
+      <c r="C128" s="62"/>
+      <c r="D128" s="9"/>
+    </row>
+    <row r="129" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A129" s="9" t="s">
+        <v>518</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C129" s="59" t="s">
         <v>1147</v>
       </c>
-      <c r="D127" s="1" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="128" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A128" s="9" t="s">
-        <v>522</v>
-      </c>
-      <c r="B128" s="9" t="s">
-        <v>1094</v>
-      </c>
-      <c r="C128" s="63" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D128" s="9" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="129" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A129" s="9"/>
-      <c r="B129" s="9"/>
-      <c r="C129" s="62"/>
-      <c r="D129" s="9"/>
+      <c r="D129" s="1" t="s">
+        <v>519</v>
+      </c>
     </row>
     <row r="130" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A130" s="9" t="s">
-        <v>399</v>
-      </c>
-      <c r="B130" s="9" t="s">
-        <v>1090</v>
-      </c>
-      <c r="C130" s="63" t="s">
-        <v>1145</v>
-      </c>
-      <c r="D130" s="9" t="s">
-        <v>400</v>
+        <v>520</v>
+      </c>
+      <c r="B130" s="1" t="s">
+        <v>1094</v>
+      </c>
+      <c r="C130" s="59" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D130" s="1" t="s">
+        <v>521</v>
       </c>
     </row>
     <row r="131" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A131" s="9" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B131" s="9" t="s">
-        <v>1092</v>
+        <v>1094</v>
       </c>
       <c r="C131" s="63" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="D131" s="9" t="s">
-        <v>398</v>
+        <v>521</v>
       </c>
     </row>
     <row r="132" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A132" s="9" t="s">
-        <v>524</v>
-      </c>
-      <c r="B132" s="1" t="s">
-        <v>1095</v>
-      </c>
-      <c r="C132" s="59" t="s">
-        <v>1147</v>
-      </c>
-      <c r="D132" s="1" t="s">
-        <v>525</v>
-      </c>
+      <c r="A132" s="9"/>
+      <c r="B132" s="9"/>
+      <c r="C132" s="62"/>
+      <c r="D132" s="9"/>
     </row>
     <row r="133" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A133" s="9"/>
-      <c r="B133" s="9"/>
-      <c r="C133" s="62"/>
-      <c r="D133" s="9"/>
+      <c r="A133" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="B133" s="9" t="s">
+        <v>1090</v>
+      </c>
+      <c r="C133" s="63" t="s">
+        <v>1145</v>
+      </c>
+      <c r="D133" s="9" t="s">
+        <v>400</v>
+      </c>
     </row>
     <row r="134" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A134" s="9" t="s">
-        <v>526</v>
+        <v>523</v>
       </c>
       <c r="B134" s="9" t="s">
-        <v>527</v>
-      </c>
-      <c r="C134" s="62" t="s">
-        <v>1109</v>
+        <v>1092</v>
+      </c>
+      <c r="C134" s="63" t="s">
+        <v>1146</v>
       </c>
       <c r="D134" s="9" t="s">
-        <v>527</v>
+        <v>398</v>
       </c>
     </row>
     <row r="135" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A135" s="9" t="s">
-        <v>528</v>
-      </c>
-      <c r="B135" s="9" t="s">
-        <v>1311</v>
-      </c>
-      <c r="C135" s="62" t="s">
-        <v>530</v>
-      </c>
-      <c r="D135" s="9" t="s">
-        <v>529</v>
+        <v>524</v>
+      </c>
+      <c r="B135" s="1" t="s">
+        <v>1095</v>
+      </c>
+      <c r="C135" s="59" t="s">
+        <v>1147</v>
+      </c>
+      <c r="D135" s="1" t="s">
+        <v>525</v>
       </c>
     </row>
     <row r="136" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A136" s="9" t="s">
-        <v>401</v>
-      </c>
-      <c r="B136" s="9" t="s">
-        <v>1311</v>
-      </c>
-      <c r="C136" s="62" t="s">
-        <v>530</v>
-      </c>
-      <c r="D136" s="9" t="s">
-        <v>394</v>
-      </c>
+      <c r="A136" s="9"/>
+      <c r="B136" s="9"/>
+      <c r="C136" s="62"/>
+      <c r="D136" s="9"/>
     </row>
     <row r="137" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A137" s="9"/>
-      <c r="B137" s="9"/>
-      <c r="C137" s="62"/>
-      <c r="D137" s="9"/>
+      <c r="A137" s="9" t="s">
+        <v>526</v>
+      </c>
+      <c r="B137" s="9" t="s">
+        <v>527</v>
+      </c>
+      <c r="C137" s="62" t="s">
+        <v>1109</v>
+      </c>
+      <c r="D137" s="9" t="s">
+        <v>527</v>
+      </c>
     </row>
     <row r="138" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A138" s="9" t="s">
-        <v>406</v>
+        <v>528</v>
       </c>
       <c r="B138" s="9" t="s">
-        <v>407</v>
+        <v>1311</v>
       </c>
       <c r="C138" s="62" t="s">
-        <v>1110</v>
+        <v>530</v>
       </c>
       <c r="D138" s="9" t="s">
-        <v>407</v>
+        <v>529</v>
       </c>
     </row>
     <row r="139" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A139" s="9"/>
-      <c r="B139" s="9"/>
-      <c r="C139" s="62"/>
-      <c r="D139" s="9"/>
+      <c r="A139" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="B139" s="9" t="s">
+        <v>1311</v>
+      </c>
+      <c r="C139" s="62" t="s">
+        <v>530</v>
+      </c>
+      <c r="D139" s="9" t="s">
+        <v>394</v>
+      </c>
     </row>
     <row r="140" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A140" s="9" t="s">
-        <v>531</v>
-      </c>
-      <c r="B140" s="9" t="s">
-        <v>1096</v>
-      </c>
-      <c r="C140" s="62" t="s">
-        <v>1148</v>
-      </c>
-      <c r="D140" s="9" t="s">
-        <v>1023</v>
-      </c>
+      <c r="A140" s="9"/>
+      <c r="B140" s="9"/>
+      <c r="C140" s="62"/>
+      <c r="D140" s="9"/>
     </row>
     <row r="141" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A141" s="9" t="s">
-        <v>532</v>
+        <v>406</v>
       </c>
       <c r="B141" s="9" t="s">
-        <v>12</v>
+        <v>407</v>
       </c>
       <c r="C141" s="62" t="s">
-        <v>13</v>
+        <v>1110</v>
       </c>
       <c r="D141" s="9" t="s">
-        <v>12</v>
+        <v>407</v>
       </c>
     </row>
     <row r="142" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A142" s="9" t="s">
-        <v>533</v>
-      </c>
-      <c r="B142" s="9" t="s">
-        <v>380</v>
-      </c>
-      <c r="C142" s="62" t="s">
-        <v>380</v>
-      </c>
-      <c r="D142" s="9" t="s">
-        <v>380</v>
-      </c>
+      <c r="A142" s="9"/>
+      <c r="B142" s="9"/>
+      <c r="C142" s="62"/>
+      <c r="D142" s="9"/>
     </row>
     <row r="143" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A143" s="9" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="B143" s="9" t="s">
-        <v>535</v>
+        <v>1096</v>
       </c>
       <c r="C143" s="62" t="s">
-        <v>1111</v>
+        <v>1148</v>
       </c>
       <c r="D143" s="9" t="s">
-        <v>535</v>
+        <v>1023</v>
       </c>
     </row>
     <row r="144" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A144" s="9"/>
-      <c r="B144" s="9"/>
-      <c r="C144" s="62"/>
-      <c r="D144" s="9"/>
+      <c r="A144" s="9" t="s">
+        <v>532</v>
+      </c>
+      <c r="B144" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="C144" s="62" t="s">
+        <v>13</v>
+      </c>
+      <c r="D144" s="9" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="145" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A145" s="9" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="B145" s="9" t="s">
-        <v>537</v>
+        <v>380</v>
       </c>
       <c r="C145" s="62" t="s">
-        <v>1112</v>
+        <v>380</v>
       </c>
       <c r="D145" s="9" t="s">
-        <v>537</v>
+        <v>380</v>
       </c>
     </row>
     <row r="146" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A146" s="36" t="s">
-        <v>538</v>
+      <c r="A146" s="9" t="s">
+        <v>534</v>
       </c>
       <c r="B146" s="9" t="s">
-        <v>1097</v>
+        <v>535</v>
       </c>
       <c r="C146" s="62" t="s">
-        <v>1149</v>
+        <v>1111</v>
       </c>
       <c r="D146" s="9" t="s">
-        <v>539</v>
+        <v>535</v>
       </c>
     </row>
     <row r="147" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A147" s="9" t="s">
-        <v>540</v>
-      </c>
-      <c r="B147" s="9" t="s">
-        <v>1098</v>
-      </c>
-      <c r="C147" s="62" t="s">
-        <v>1150</v>
-      </c>
-      <c r="D147" s="9" t="s">
-        <v>541</v>
-      </c>
+      <c r="A147" s="9"/>
+      <c r="B147" s="9"/>
+      <c r="C147" s="62"/>
+      <c r="D147" s="9"/>
     </row>
     <row r="148" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A148" s="9" t="s">
-        <v>542</v>
+        <v>536</v>
       </c>
       <c r="B148" s="9" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
       <c r="C148" s="62" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="D148" s="9" t="s">
-        <v>543</v>
+        <v>537</v>
       </c>
     </row>
     <row r="149" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A149" s="9" t="s">
-        <v>544</v>
+      <c r="A149" s="36" t="s">
+        <v>538</v>
       </c>
       <c r="B149" s="9" t="s">
-        <v>545</v>
+        <v>1097</v>
       </c>
       <c r="C149" s="62" t="s">
-        <v>1114</v>
+        <v>1149</v>
       </c>
       <c r="D149" s="9" t="s">
-        <v>545</v>
+        <v>539</v>
       </c>
     </row>
     <row r="150" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A150" s="9"/>
-      <c r="B150" s="9"/>
-      <c r="C150" s="62"/>
-      <c r="D150" s="9"/>
+      <c r="A150" s="9" t="s">
+        <v>540</v>
+      </c>
+      <c r="B150" s="9" t="s">
+        <v>1098</v>
+      </c>
+      <c r="C150" s="62" t="s">
+        <v>1150</v>
+      </c>
+      <c r="D150" s="9" t="s">
+        <v>541</v>
+      </c>
     </row>
     <row r="151" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A151" s="9" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="B151" s="9" t="s">
-        <v>1087</v>
+        <v>543</v>
       </c>
       <c r="C151" s="62" t="s">
-        <v>1143</v>
+        <v>1113</v>
       </c>
       <c r="D151" s="9" t="s">
-        <v>382</v>
+        <v>543</v>
       </c>
     </row>
     <row r="152" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A152" s="9" t="s">
-        <v>404</v>
+        <v>544</v>
       </c>
       <c r="B152" s="9" t="s">
-        <v>405</v>
-      </c>
-      <c r="C152" s="72" t="s">
-        <v>1115</v>
+        <v>545</v>
+      </c>
+      <c r="C152" s="62" t="s">
+        <v>1114</v>
       </c>
       <c r="D152" s="9" t="s">
-        <v>405</v>
+        <v>545</v>
       </c>
     </row>
     <row r="153" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A153" s="34"/>
-      <c r="B153" s="34" t="s">
-        <v>547</v>
-      </c>
-      <c r="C153" s="68"/>
-      <c r="D153" s="34" t="s">
-        <v>547</v>
-      </c>
+      <c r="A153" s="9"/>
+      <c r="B153" s="9"/>
+      <c r="C153" s="62"/>
+      <c r="D153" s="9"/>
     </row>
     <row r="154" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A154" s="9" t="s">
-        <v>408</v>
+        <v>546</v>
       </c>
       <c r="B154" s="9" t="s">
-        <v>1117</v>
+        <v>1087</v>
       </c>
       <c r="C154" s="62" t="s">
-        <v>1151</v>
+        <v>1143</v>
       </c>
       <c r="D154" s="9" t="s">
-        <v>409</v>
+        <v>382</v>
       </c>
     </row>
     <row r="155" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A155" s="9" t="s">
-        <v>30</v>
+        <v>404</v>
       </c>
       <c r="B155" s="9" t="s">
-        <v>1099</v>
-      </c>
-      <c r="C155" s="60" t="s">
-        <v>1129</v>
+        <v>405</v>
+      </c>
+      <c r="C155" s="72" t="s">
+        <v>1115</v>
       </c>
       <c r="D155" s="9" t="s">
-        <v>410</v>
+        <v>405</v>
       </c>
     </row>
     <row r="156" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A156" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B156" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C156" s="60" t="s">
-        <v>33</v>
-      </c>
-      <c r="D156" s="9" t="s">
-        <v>32</v>
+      <c r="A156" s="34"/>
+      <c r="B156" s="34" t="s">
+        <v>547</v>
+      </c>
+      <c r="C156" s="68"/>
+      <c r="D156" s="34" t="s">
+        <v>547</v>
       </c>
     </row>
     <row r="157" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A157" s="9"/>
-      <c r="B157" s="9"/>
-      <c r="C157" s="62"/>
-      <c r="D157" s="9"/>
+      <c r="A157" s="9" t="s">
+        <v>408</v>
+      </c>
+      <c r="B157" s="9" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C157" s="62" t="s">
+        <v>1151</v>
+      </c>
+      <c r="D157" s="9" t="s">
+        <v>409</v>
+      </c>
     </row>
     <row r="158" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A158" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B158" s="9" t="s">
+        <v>1099</v>
+      </c>
+      <c r="C158" s="60" t="s">
+        <v>1129</v>
+      </c>
+      <c r="D158" s="9" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="159" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A159" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B159" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C159" s="60" t="s">
+        <v>33</v>
+      </c>
+      <c r="D159" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="160" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A160" s="9"/>
+      <c r="B160" s="9"/>
+      <c r="C160" s="62"/>
+      <c r="D160" s="9"/>
+    </row>
+    <row r="161" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A161" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="B158" s="9" t="s">
+      <c r="B161" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C158" s="60" t="s">
+      <c r="C161" s="60" t="s">
         <v>16</v>
       </c>
-      <c r="D158" s="9" t="s">
+      <c r="D161" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="159" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A159" s="37"/>
-      <c r="B159" s="37"/>
-      <c r="C159" s="69"/>
-      <c r="D159" s="37"/>
-    </row>
-    <row r="160" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A160" s="6"/>
-      <c r="B160" s="38"/>
-      <c r="C160" s="70"/>
-      <c r="D160" s="38"/>
-    </row>
-    <row r="161" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A161" s="39"/>
-      <c r="B161" s="40" t="s">
+    <row r="162" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A162" s="37"/>
+      <c r="B162" s="37"/>
+      <c r="C162" s="69"/>
+      <c r="D162" s="37"/>
+    </row>
+    <row r="163" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A163" s="6"/>
+      <c r="B163" s="38"/>
+      <c r="C163" s="70"/>
+      <c r="D163" s="38"/>
+    </row>
+    <row r="164" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A164" s="39"/>
+      <c r="B164" s="40" t="s">
         <v>493</v>
       </c>
-      <c r="C161" s="71"/>
-      <c r="D161" s="40" t="s">
+      <c r="C164" s="71"/>
+      <c r="D164" s="40" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="162" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A162" s="6" t="s">
+    <row r="165" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A165" s="6" t="s">
         <v>494</v>
       </c>
-      <c r="B162" s="38" t="s">
+      <c r="B165" s="38" t="s">
         <v>1085</v>
       </c>
-      <c r="C162" s="38" t="s">
+      <c r="C165" s="38" t="s">
         <v>1142</v>
       </c>
-      <c r="D162" s="38" t="s">
+      <c r="D165" s="38" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="163" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A163" s="6" t="s">
+    <row r="166" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A166" s="6" t="s">
         <v>496</v>
       </c>
-      <c r="B163" s="38" t="s">
+      <c r="B166" s="38" t="s">
         <v>497</v>
       </c>
-      <c r="C163" s="38" t="s">
+      <c r="C166" s="38" t="s">
         <v>497</v>
       </c>
-      <c r="D163" s="38" t="s">
+      <c r="D166" s="38" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="164" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A164" s="6"/>
-      <c r="B164" s="38" t="s">
+    <row r="167" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A167" s="6"/>
+      <c r="B167" s="38" t="s">
         <v>498</v>
       </c>
-      <c r="C164" s="38" t="s">
+      <c r="C167" s="38" t="s">
         <v>498</v>
       </c>
-      <c r="D164" s="38" t="s">
+      <c r="D167" s="38" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="165" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
-      <c r="A165" s="9"/>
-      <c r="B165" s="9"/>
-      <c r="C165" s="62"/>
-      <c r="D165" s="9"/>
-    </row>
-    <row r="166" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A166" s="29"/>
-      <c r="B166" s="35" t="s">
+    <row r="168" spans="1:4" ht="15.75" customHeight="1" thickTop="1" thickBot="1">
+      <c r="A168" s="9"/>
+      <c r="B168" s="9"/>
+      <c r="C168" s="62"/>
+      <c r="D168" s="9"/>
+    </row>
+    <row r="169" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A169" s="29"/>
+      <c r="B169" s="35" t="s">
         <v>548</v>
       </c>
-      <c r="C166" s="66"/>
-      <c r="D166" s="35" t="s">
+      <c r="C169" s="66"/>
+      <c r="D169" s="35" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="167" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A167" s="9" t="s">
+    <row r="170" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A170" s="9" t="s">
         <v>549</v>
       </c>
-      <c r="B167" s="9" t="s">
+      <c r="B170" s="9" t="s">
         <v>1100</v>
       </c>
-      <c r="C167" s="62" t="s">
+      <c r="C170" s="62" t="s">
         <v>1152</v>
       </c>
-      <c r="D167" s="9" t="s">
+      <c r="D170" s="9" t="s">
         <v>1071</v>
       </c>
     </row>
-    <row r="168" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A168" s="9" t="s">
+    <row r="171" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A171" s="9" t="s">
         <v>550</v>
       </c>
-      <c r="B168" s="9" t="s">
+      <c r="B171" s="9" t="s">
         <v>551</v>
       </c>
-      <c r="C168" s="62" t="s">
+      <c r="C171" s="62" t="s">
         <v>1116</v>
       </c>
-      <c r="D168" s="9" t="s">
+      <c r="D171" s="9" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="169" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A169" s="9" t="s">
+    <row r="172" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A172" s="9" t="s">
         <v>413</v>
       </c>
-      <c r="B169" s="9" t="s">
+      <c r="B172" s="9" t="s">
         <v>1155</v>
       </c>
-      <c r="C169" s="62" t="s">
+      <c r="C172" s="62" t="s">
         <v>1154</v>
       </c>
-      <c r="D169" s="9" t="s">
+      <c r="D172" s="9" t="s">
         <v>414</v>
       </c>
     </row>
-    <row r="170" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A170" s="9"/>
-      <c r="B170" s="9"/>
-      <c r="C170" s="62"/>
-      <c r="D170" s="9"/>
-    </row>
-    <row r="171" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A171" s="1" t="s">
+    <row r="173" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A173" s="9"/>
+      <c r="B173" s="9"/>
+      <c r="C173" s="62"/>
+      <c r="D173" s="9"/>
+    </row>
+    <row r="174" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A174" s="1" t="s">
         <v>552</v>
       </c>
-      <c r="B171" s="12" t="s">
+      <c r="B174" s="12" t="s">
         <v>1101</v>
       </c>
-      <c r="C171" s="63" t="s">
+      <c r="C174" s="63" t="s">
         <v>1127</v>
       </c>
-      <c r="D171" s="12" t="s">
+      <c r="D174" s="12" t="s">
         <v>553</v>
       </c>
     </row>
-    <row r="172" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A172" s="1" t="s">
+    <row r="175" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A175" s="1" t="s">
         <v>554</v>
       </c>
-      <c r="B172" s="9" t="s">
+      <c r="B175" s="9" t="s">
         <v>555</v>
       </c>
-      <c r="C172" s="62" t="s">
+      <c r="C175" s="62" t="s">
         <v>23</v>
       </c>
-      <c r="D172" s="9" t="s">
+      <c r="D175" s="9" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="173" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A173" s="1" t="s">
+    <row r="176" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A176" s="1" t="s">
         <v>556</v>
       </c>
-      <c r="B173" s="9" t="s">
+      <c r="B176" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C173" s="62" t="s">
+      <c r="C176" s="62" t="s">
         <v>16</v>
       </c>
-      <c r="D173" s="9" t="s">
+      <c r="D176" s="9" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="174" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A174" s="9"/>
-      <c r="B174" s="9"/>
-      <c r="C174" s="62"/>
-    </row>
-    <row r="175" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A175" s="9" t="s">
+    <row r="177" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A177" s="9"/>
+      <c r="B177" s="9"/>
+      <c r="C177" s="62"/>
+    </row>
+    <row r="178" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A178" s="9" t="s">
         <v>1059</v>
       </c>
-      <c r="B175" s="9" t="s">
+      <c r="B178" s="9" t="s">
         <v>1087</v>
       </c>
-      <c r="C175" s="62" t="s">
+      <c r="C178" s="62" t="s">
         <v>1143</v>
       </c>
-      <c r="D175" s="9" t="s">
+      <c r="D178" s="9" t="s">
         <v>1087</v>
-      </c>
-    </row>
-    <row r="176" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A176" s="9" t="s">
-        <v>1158</v>
-      </c>
-      <c r="B176" s="9" t="s">
-        <v>1159</v>
-      </c>
-      <c r="C176" s="62" t="s">
-        <v>1160</v>
-      </c>
-      <c r="D176" s="9" t="s">
-        <v>1159</v>
-      </c>
-    </row>
-    <row r="177" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A177" s="9" t="s">
-        <v>1161</v>
-      </c>
-      <c r="B177" s="9" t="s">
-        <v>1162</v>
-      </c>
-      <c r="C177" s="9" t="s">
-        <v>1162</v>
-      </c>
-      <c r="D177" s="9" t="s">
-        <v>1162</v>
-      </c>
-    </row>
-    <row r="178" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A178" s="91" t="s">
-        <v>1163</v>
-      </c>
-      <c r="B178" s="9" t="s">
-        <v>1164</v>
-      </c>
-      <c r="C178" s="9" t="s">
-        <v>1164</v>
-      </c>
-      <c r="D178" s="9" t="s">
-        <v>1164</v>
       </c>
     </row>
     <row r="179" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A179" s="9" t="s">
-        <v>1167</v>
+        <v>1158</v>
       </c>
       <c r="B179" s="9" t="s">
-        <v>1165</v>
-      </c>
-      <c r="C179" s="9" t="s">
-        <v>1166</v>
+        <v>1159</v>
+      </c>
+      <c r="C179" s="62" t="s">
+        <v>1160</v>
       </c>
       <c r="D179" s="9" t="s">
-        <v>1165</v>
+        <v>1159</v>
       </c>
     </row>
     <row r="180" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="B180" s="9"/>
-      <c r="C180" s="9"/>
+      <c r="A180" s="9" t="s">
+        <v>1161</v>
+      </c>
+      <c r="B180" s="9" t="s">
+        <v>1162</v>
+      </c>
+      <c r="C180" s="9" t="s">
+        <v>1162</v>
+      </c>
+      <c r="D180" s="9" t="s">
+        <v>1162</v>
+      </c>
     </row>
     <row r="181" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A181" s="29"/>
-      <c r="B181" s="35" t="s">
-        <v>1222</v>
-      </c>
-      <c r="C181" s="66"/>
+      <c r="A181" s="91" t="s">
+        <v>1163</v>
+      </c>
+      <c r="B181" s="9" t="s">
+        <v>1164</v>
+      </c>
+      <c r="C181" s="9" t="s">
+        <v>1164</v>
+      </c>
+      <c r="D181" s="9" t="s">
+        <v>1164</v>
+      </c>
     </row>
     <row r="182" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A182" s="9" t="s">
-        <v>1221</v>
+        <v>1167</v>
       </c>
       <c r="B182" s="9" t="s">
-        <v>1280</v>
-      </c>
-      <c r="C182" s="62" t="s">
-        <v>1224</v>
+        <v>1165</v>
+      </c>
+      <c r="C182" s="9" t="s">
+        <v>1166</v>
       </c>
       <c r="D182" s="9" t="s">
-        <v>1223</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="183" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A183" s="9" t="s">
-        <v>1225</v>
-      </c>
-      <c r="B183" s="9" t="s">
-        <v>1280</v>
-      </c>
-      <c r="C183" s="62" t="s">
-        <v>1224</v>
-      </c>
+      <c r="B183" s="9"/>
+      <c r="C183" s="9"/>
     </row>
     <row r="184" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A184" s="91" t="s">
-        <v>1226</v>
-      </c>
-      <c r="B184" s="9" t="s">
-        <v>1279</v>
-      </c>
-      <c r="C184" s="9"/>
+      <c r="A184" s="29"/>
+      <c r="B184" s="35" t="s">
+        <v>1222</v>
+      </c>
+      <c r="C184" s="66"/>
     </row>
     <row r="185" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A185" s="9" t="s">
+        <v>1221</v>
+      </c>
+      <c r="B185" s="9" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C185" s="62" t="s">
+        <v>1224</v>
+      </c>
+      <c r="D185" s="9" t="s">
+        <v>1223</v>
+      </c>
+    </row>
+    <row r="186" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A186" s="9" t="s">
+        <v>1225</v>
+      </c>
+      <c r="B186" s="9" t="s">
+        <v>1280</v>
+      </c>
+      <c r="C186" s="62" t="s">
+        <v>1224</v>
+      </c>
+    </row>
+    <row r="187" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A187" s="91" t="s">
+        <v>1226</v>
+      </c>
+      <c r="B187" s="9" t="s">
+        <v>1279</v>
+      </c>
+      <c r="C187" s="9"/>
+    </row>
+    <row r="188" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A188" s="9" t="s">
         <v>1281</v>
       </c>
-      <c r="B185" s="9" t="s">
+      <c r="B188" s="9" t="s">
         <v>1282</v>
       </c>
-      <c r="C185" s="9"/>
-    </row>
-    <row r="186" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A186" s="9"/>
-      <c r="B186" s="9"/>
-      <c r="C186" s="9"/>
-    </row>
-    <row r="187" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A187" s="1" t="s">
-        <v>212</v>
-      </c>
-      <c r="B187" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="C187" s="97" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="188" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A188" s="1" t="s">
-        <v>215</v>
-      </c>
-      <c r="B188" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C188" s="76" t="s">
-        <v>7</v>
-      </c>
+      <c r="C188" s="9"/>
     </row>
     <row r="189" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A189" s="9"/>
@@ -35012,51 +35074,57 @@
     </row>
     <row r="190" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
       <c r="A190" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="B190" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="C190" s="97" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="191" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A191" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B191" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C191" s="76" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="192" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A192" s="9"/>
+      <c r="B192" s="9"/>
+      <c r="C192" s="9"/>
+    </row>
+    <row r="193" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A193" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B190" s="1" t="s">
+      <c r="B193" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="C190" s="76" t="s">
+      <c r="C193" s="76" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="191" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A191" s="9"/>
-      <c r="B191" s="9"/>
-      <c r="C191" s="9"/>
-    </row>
-    <row r="192" spans="1:4" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A192" s="1" t="s">
+    <row r="194" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A194" s="9"/>
+      <c r="B194" s="9"/>
+      <c r="C194" s="9"/>
+    </row>
+    <row r="195" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
+      <c r="A195" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B192" s="1" t="s">
+      <c r="B195" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="C192" s="76" t="s">
+      <c r="C195" s="76" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="193" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A193" s="9"/>
-      <c r="B193" s="9"/>
-      <c r="C193" s="9"/>
-    </row>
-    <row r="194" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A194" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="B194" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C194" s="76" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="195" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A195" s="9"/>
-      <c r="B195" s="9"/>
-      <c r="C195" s="9"/>
     </row>
     <row r="196" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A196" s="9"/>
@@ -35064,21 +35132,27 @@
       <c r="C196" s="9"/>
     </row>
     <row r="197" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
-      <c r="A197" s="9"/>
-      <c r="B197" s="9"/>
-      <c r="C197" s="9"/>
-    </row>
-    <row r="198" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A197" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="B197" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C197" s="76" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A198" s="9"/>
       <c r="B198" s="9"/>
       <c r="C198" s="9"/>
     </row>
-    <row r="199" spans="1:3" ht="15.75" customHeight="1">
+    <row r="199" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A199" s="9"/>
       <c r="B199" s="9"/>
       <c r="C199" s="9"/>
     </row>
-    <row r="200" spans="1:3" ht="15.75" customHeight="1">
+    <row r="200" spans="1:3" ht="15.75" customHeight="1" thickBot="1">
       <c r="A200" s="9"/>
       <c r="B200" s="9"/>
       <c r="C200" s="9"/>
@@ -35913,24 +35987,36 @@
       <c r="B366" s="9"/>
       <c r="C366" s="9"/>
     </row>
-    <row r="367" spans="1:3" ht="15.75" customHeight="1"/>
-    <row r="368" spans="1:3" ht="15.75" customHeight="1"/>
-    <row r="369" ht="15.75" customHeight="1"/>
-    <row r="370" ht="15.75" customHeight="1"/>
-    <row r="371" ht="15.75" customHeight="1"/>
-    <row r="372" ht="15.75" customHeight="1"/>
-    <row r="373" ht="15.75" customHeight="1"/>
-    <row r="374" ht="15.75" customHeight="1"/>
-    <row r="375" ht="15.75" customHeight="1"/>
-    <row r="376" ht="15.75" customHeight="1"/>
-    <row r="377" ht="15.75" customHeight="1"/>
-    <row r="378" ht="15.75" customHeight="1"/>
-    <row r="379" ht="15.75" customHeight="1"/>
-    <row r="380" ht="15.75" customHeight="1"/>
-    <row r="381" ht="15.75" customHeight="1"/>
-    <row r="382" ht="15.75" customHeight="1"/>
-    <row r="383" ht="15.75" customHeight="1"/>
-    <row r="384" ht="15.75" customHeight="1"/>
+    <row r="367" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A367" s="9"/>
+      <c r="B367" s="9"/>
+      <c r="C367" s="9"/>
+    </row>
+    <row r="368" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A368" s="9"/>
+      <c r="B368" s="9"/>
+      <c r="C368" s="9"/>
+    </row>
+    <row r="369" spans="1:3" ht="15.75" customHeight="1">
+      <c r="A369" s="9"/>
+      <c r="B369" s="9"/>
+      <c r="C369" s="9"/>
+    </row>
+    <row r="370" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="371" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="372" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="373" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="374" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="375" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="376" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="377" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="378" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="379" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="380" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="381" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="382" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="383" spans="1:3" ht="15.75" customHeight="1"/>
+    <row r="384" spans="1:3" ht="15.75" customHeight="1"/>
     <row r="385" ht="15.75" customHeight="1"/>
     <row r="386" ht="15.75" customHeight="1"/>
     <row r="387" ht="15.75" customHeight="1"/>
@@ -36548,14 +36634,17 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
     <row r="1001" ht="15.75" customHeight="1"/>
+    <row r="1002" ht="15.75" customHeight="1"/>
+    <row r="1003" ht="15.75" customHeight="1"/>
+    <row r="1004" ht="15.75" customHeight="1"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B3" r:id="rId1" xr:uid="{51CF91D8-7A2D-4C64-827B-6C41EEA7AE41}"/>
     <hyperlink ref="D3" r:id="rId2" xr:uid="{40CD9620-87B1-4D27-9D9D-9B54D2D36C19}"/>
-    <hyperlink ref="C152" r:id="rId3" xr:uid="{25FAC99D-B272-4C71-9B4D-364D57432552}"/>
+    <hyperlink ref="C155" r:id="rId3" xr:uid="{25FAC99D-B272-4C71-9B4D-364D57432552}"/>
     <hyperlink ref="B2" r:id="rId4" xr:uid="{A5D45DE0-52B9-458D-A530-797F4FB8B49C}"/>
     <hyperlink ref="C2" r:id="rId5" xr:uid="{10A69855-CD62-4F1A-BCBC-DBB64A29B7CA}"/>
-    <hyperlink ref="C187" r:id="rId6" xr:uid="{15BB9E58-3CD9-4309-9710-BEFD670B22CD}"/>
+    <hyperlink ref="C190" r:id="rId6" xr:uid="{15BB9E58-3CD9-4309-9710-BEFD670B22CD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape" r:id="rId7"/>

</xml_diff>

<commit_message>
Patient Happy Path Updated code 06/08/25
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3030F9DA-20C6-462D-B0E5-1AC4BCEFEEB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2797BFE-4FB0-44A7-9F0E-A562D4E06B34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2755" uniqueCount="1369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2755" uniqueCount="1365">
   <si>
     <t>KEY</t>
   </si>
@@ -4096,24 +4096,9 @@
     <t>Automation1_HC1;Repeat Prescription;Urgent/Same day;10;Patient to Collect Script - 24 Hours -22;Next Day;33;Patient to Collect Script - 36 Hours - 33;48 Hours;44;Patient to Collect Script - 48 Hours - 44;72 Hours;55;Patient to Collect Script - 72 Hours - 55;</t>
   </si>
   <si>
-    <t>Automation1_Loc3;prostin vr 500mcg/1ml inj(alprostadil);Pending;Next Day;Gp6 White</t>
-  </si>
-  <si>
     <t>Automation1_Loc1;Trasylol 500,000KIU/50ml Inj;Pending;Next Day;GP2WHITE</t>
   </si>
   <si>
-    <t>Automation1_Loc1;Trasylol 500,000KIU/50ml Inj;Pending;Urgent/Same day;GP1 A1 L1</t>
-  </si>
-  <si>
-    <t>Automation1_Loc1;Trasylol 500,000KIU/50ml Inj;Pending;48 Hours;GP3 White</t>
-  </si>
-  <si>
-    <t>Automation1_Loc1;Trasylol 500,000KIU/50ml Inj;Pending;ZOOM Pharmacy home delivery;48 Hours;GP2WHITE</t>
-  </si>
-  <si>
-    <t>Automation1_Loc2;Trasylol 500,000KIU/50ml Inj;Pending;48 Hours;GP3 White</t>
-  </si>
-  <si>
     <t>GP1 Vm07 Loc1 ( VM07 Loc1 Evo Prod );VM07 Loc1 Evo Prod;Send Script by Post;Urgent/Same day;panadol (optizorb) 500mg caplets(paracetamol);pending</t>
   </si>
   <si>
@@ -4136,6 +4121,9 @@
   </si>
   <si>
     <t>https://app.managemyhealth.co.nz/home</t>
+  </si>
+  <si>
+    <t>Automation1_Loc3;prostin vr 500mcg/1ml inj(alprostadil);pending;Next Day;Gp6 White</t>
   </si>
 </sst>
 </file>
@@ -5130,7 +5118,7 @@
         <v>1113</v>
       </c>
       <c r="C2" s="73" t="s">
-        <v>1368</v>
+        <v>1363</v>
       </c>
       <c r="D2" s="56" t="s">
         <v>1113</v>
@@ -6857,13 +6845,13 @@
         <v>1351</v>
       </c>
       <c r="B60" s="1" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C60" s="75" t="s">
+        <v>1362</v>
+      </c>
+      <c r="D60" s="1" t="s">
         <v>1355</v>
-      </c>
-      <c r="C60" s="75" t="s">
-        <v>1367</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>1356</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" s="2"/>
@@ -6981,10 +6969,10 @@
         <v>58</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>1356</v>
+        <v>59</v>
       </c>
       <c r="C64" s="75" t="s">
-        <v>1367</v>
+        <v>1362</v>
       </c>
       <c r="D64" s="1" t="s">
         <v>59</v>
@@ -7105,7 +7093,7 @@
         <v>66</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>1357</v>
+        <v>67</v>
       </c>
       <c r="C68" s="75" t="s">
         <v>1302</v>
@@ -7229,7 +7217,7 @@
         <v>74</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>1358</v>
+        <v>1039</v>
       </c>
       <c r="C72" s="75" t="s">
         <v>75</v>
@@ -7353,7 +7341,7 @@
         <v>79</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>1359</v>
+        <v>1034</v>
       </c>
       <c r="C76" s="75" t="s">
         <v>80</v>
@@ -7477,7 +7465,7 @@
         <v>84</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>1359</v>
+        <v>1034</v>
       </c>
       <c r="C80" s="75" t="s">
         <v>80</v>
@@ -7568,7 +7556,7 @@
         <v>86</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>1359</v>
+        <v>1034</v>
       </c>
       <c r="C83" s="75" t="s">
         <v>80</v>
@@ -7659,7 +7647,7 @@
         <v>89</v>
       </c>
       <c r="B86" s="9" t="s">
-        <v>1360</v>
+        <v>1035</v>
       </c>
       <c r="C86" s="76" t="s">
         <v>90</v>
@@ -9643,7 +9631,7 @@
         <v>1240</v>
       </c>
       <c r="C150" s="75" t="s">
-        <v>1366</v>
+        <v>1361</v>
       </c>
       <c r="D150" s="1" t="s">
         <v>1114</v>
@@ -33732,10 +33720,10 @@
         <v>70</v>
       </c>
       <c r="C49" s="75" t="s">
-        <v>1361</v>
+        <v>1356</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>1362</v>
+        <v>1357</v>
       </c>
     </row>
     <row r="50" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
@@ -33830,13 +33818,13 @@
         <v>76</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>1363</v>
+        <v>1358</v>
       </c>
       <c r="C56" s="75" t="s">
-        <v>1364</v>
+        <v>1359</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>1363</v>
+        <v>1358</v>
       </c>
     </row>
     <row r="57" spans="1:23" ht="15.75" customHeight="1" thickBot="1">
@@ -33998,13 +33986,13 @@
         <v>60</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>1365</v>
+        <v>1360</v>
       </c>
       <c r="C69" s="59" t="s">
         <v>959</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>1365</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="70" spans="1:4" ht="15.75" customHeight="1" thickBot="1">

</xml_diff>